<commit_message>
Complete HealthGuard D1-D3 governance portfolio tabs
- D1: EU AI Act high-risk classification (Art. 6(1) + Annex I/MDR,
  Annex III 5(a) secondary), Arts 9-15 gap analysis, top launch blockers
- D2: per-stage GDPR/CPRA obligation map, US->EU telemetry transfer
  analysis, top 5 compliance risks for D5
- D3: attack-surface summary and three ATLAS TTPs (T0020, T0010.003,
  T0024) with scenarios, named mitigations and prioritisation

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/04-secure-ai-deployment/project/starter/governance_portfolio.xlsx
+++ b/04-secure-ai-deployment/project/starter/governance_portfolio.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Cover" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_D1_EU_AI_Act" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_D2_DFD_Compliance" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_D3_ATLAS" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_D4_Technical_Audit" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_D5_Risk_Register" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_D6_Model_Card" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_D7_KRI_Dashboard" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_D8_Launch_Decision" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="00_Cover" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="01_D1_EU_AI_Act" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="02_D2_DFD_Compliance" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="03_D3_ATLAS" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="04_D4_Technical_Audit" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="05_D5_Risk_Register" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="06_D6_Model_Card" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="07_D7_KRI_Dashboard" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="08_D8_Launch_Decision" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -223,7 +223,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="2"/>
@@ -321,6 +321,18 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -998,8 +1010,8 @@
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -1057,7 +1069,7 @@
       </c>
       <c r="F5" s="25" t="inlineStr"/>
     </row>
-    <row r="6" ht="60" customHeight="1">
+    <row r="6" ht="246" customHeight="1">
       <c r="A6" s="11" t="inlineStr">
         <is>
           <t>1</t>
@@ -1070,21 +1082,22 @@
       </c>
       <c r="C6" s="26" t="inlineStr">
         <is>
-          <t>[Yes / No / Borderline]</t>
+          <t>No</t>
         </is>
       </c>
       <c r="D6" s="26" t="inlineStr">
         <is>
-          <t>[Explain why each prohibited category does or does not apply]</t>
+          <t>None of the Article 5(1) prohibited practices apply: (a) no subliminal/manipulative techniques. Output goes to a clinician, not the patient. (b) Does not exploit age, disability or socio-economic vulnerability to distort behaviour. It uses region/insurance_type as features, which is a fairness issue for Art. 10, not a prohibited practice. (c) Not social scoring. The score is used only in the clinical context it is produced for, and insurance underwriting / coverage decisions are contractually prohibited (that restriction must stay enforced; see Art. 9 row). (d) No criminal-offence risk prediction. (e) No facial-image scraping. (f) No emotion recognition at work/school. (g) No biometric categorisation; no biometric data is processed. (h) No real-time remote biometric ID. Conclusion: not prohibited. Proceed to Art. 6.</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>Article 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="60" customHeight="1">
+          <t>Article 5(1)(a)-(h)</t>
+        </is>
+      </c>
+      <c r="F6" s="44" t="n"/>
+    </row>
+    <row r="7" ht="291" customHeight="1">
       <c r="A7" s="11" t="inlineStr">
         <is>
           <t>2</t>
@@ -1097,21 +1110,22 @@
       </c>
       <c r="C7" s="26" t="inlineStr">
         <is>
-          <t>[Yes / No / Borderline]</t>
+          <t>Yes (contested by vendor positioning; treat as Yes)</t>
         </is>
       </c>
       <c r="D7" s="26" t="inlineStr">
         <is>
-          <t>[State your answer with supporting evidence]</t>
+          <t>MDR 2017/745 is listed in Annex I Section A. MDR Art. 2(1) defines a medical device to include software intended for 'diagnosis, prevention, monitoring, prediction, prognosis' of disease. HealthGuard predicts an individual's T2D risk to drive preventive action (earlier labs, referral), so it meets the definition (MDCG 2019-11 decision steps: acts on patient-specific data, goes beyond storage/simple search, serves a medical purpose). Calling it 'decision support' does not exempt it. MDR Annex VIII Rule 11 classes software that provides information used for diagnostic/therapeutic decisions as at least Class IIa, which requires notified-body conformity assessment. Both limbs of Art. 6(1) are therefore met: (a) the AI system is itself a product covered by Annex I, and (b) it requires third-party conformity assessment. The brief's statement that HealthGuard is 'not a regulated medical device' is a regulatory-positioning gap that needs a formal MDR qualification opinion.</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>Article 6(1) + Annex I</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="60" customHeight="1">
+          <t>Article 6(1)(a)-(b) + Annex I Section A (MDR 2017/745 Art. 2(1); Annex VIII Rule 11; MDCG 2019-11)</t>
+        </is>
+      </c>
+      <c r="F7" s="44" t="n"/>
+    </row>
+    <row r="8" ht="246" customHeight="1">
       <c r="A8" s="11" t="inlineStr">
         <is>
           <t>3</t>
@@ -1124,21 +1138,22 @@
       </c>
       <c r="C8" s="26" t="inlineStr">
         <is>
-          <t>[Yes / No / Borderline]</t>
+          <t>Borderline</t>
         </is>
       </c>
       <c r="D8" s="26" t="inlineStr">
         <is>
-          <t>[State your answer with supporting evidence]</t>
+          <t>Point 5(a) covers essential public services, explicitly including healthcare services, when an AI system is used by or on behalf of public authorities to evaluate eligibility. The EU launch sites are academic medical centres, several of them publicly run. If the score gates referral into a publicly funded diabetes-prevention programme, 5(a) is engaged. Point 5(c) (life/health-insurance risk pricing) would apply only under a prohibited non-intended use. Point 5(d) (emergency triage) is excluded because ED/ICU use is out of scope. The Art. 6(3) derogation is NOT available. The system profiles natural persons (GDPR Art. 4(4): predicting health), and the last sub-paragraph of Art. 6(3) makes any Annex III system that profiles high-risk. Annex III is a secondary basis; the classification does not depend on it.</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>Annex III</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="60" customHeight="1">
+          <t>Annex III point 5(a) (5(c)/5(d) considered and excluded); Article 6(3)</t>
+        </is>
+      </c>
+      <c r="F8" s="44" t="n"/>
+    </row>
+    <row r="9" ht="291" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
         <is>
           <t>4</t>
@@ -1151,19 +1166,20 @@
       </c>
       <c r="C9" s="26" t="inlineStr">
         <is>
-          <t>[Yes / No / Borderline]</t>
+          <t>HIGH-RISK</t>
         </is>
       </c>
       <c r="D9" s="26" t="inlineStr">
         <is>
-          <t>[State your answer with supporting evidence]</t>
+          <t>HealthGuard is a high-risk AI system. Primary basis: Art. 6(1) + Annex I Section A, because it is medical-device software (MDR Class IIa under Rule 11) needing notified-body assessment. Secondary/alternative basis: Art. 6(2) + Annex III 5(a) where public hospitals use it to decide access to prevention services. It is not prohibited under Art. 5. Consequences for Klariova as provider: the Arts 9-15 requirements; a QMS (Art. 17); technical documentation (Art. 11/Annex IV); conformity assessment through the MDR notified body (Art. 43(3)); an EU declaration of conformity and CE marking (Arts 47-48); registration (Art. 49); post-market monitoring (Art. 72); and serious-incident reporting (Art. 73). Public-body deployers must also complete a FRIA (Art. 27). Timing: Art. 6(1) obligations apply from 2 Aug 2027 (Art. 113(c)), which falls inside the Q3 2027 EU launch window. Check whether the Digital Omnibus has changed this date, but plan as if the obligations apply at launch.</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>Article + Annex</t>
-        </is>
-      </c>
+          <t>Article 6(1) + Annex I Section A (MDR 2017/745); secondary: Article 6(2) + Annex III 5(a)</t>
+        </is>
+      </c>
+      <c r="F9" s="44" t="n"/>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
@@ -1204,7 +1220,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="50" customHeight="1">
+    <row r="14" ht="291" customHeight="1">
       <c r="A14" s="11" t="inlineStr">
         <is>
           <t>Art. 9</t>
@@ -1222,21 +1238,23 @@
       </c>
       <c r="D14" s="26" t="inlineStr">
         <is>
-          <t>[Met / Partially Met / Not Met]</t>
+          <t>Partially Met</t>
         </is>
       </c>
       <c r="E14" s="26" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low]</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F14" s="26" t="inlineStr">
         <is>
-          <t>[Evidence to prove compliance + remediation needed to close the gap]</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="50" customHeight="1">
+          <t>EVIDENCE OF GAP: This pre-launch GRC review is the first structured risk assessment. There is no documented, continuous lifecycle RMS. No acceptance thresholds were set in advance for testing (Art. 9(6)-(8)). Subgroup harm to vulnerable groups (Art. 9(9)) has not been evaluated. Foreseeable misuse (insurance underwriting, patient-facing use, ED/ICU use) is controlled only by contract terms.
+REMEDIATION: Adopt a written RMS procedure aligned to ISO 14971 (needed for MDR anyway) and ISO/IEC 23894, and make the D5 risk register its living output. Set pass/fail thresholds before testing, including a subgroup-FNR tolerance. Add technical misuse controls: API scoping, tenant blocks for ED/ICU, and no patient-facing endpoint. Feed post-market monitoring (Art. 72) and the D7 KRIs back into the RMS on a set review cadence.
+PROOF: an approved RMS procedure, a risk register with an owner for each risk, and residual-risk acceptance signed by the AI Review Board.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="381" customHeight="1">
       <c r="A15" s="11" t="inlineStr">
         <is>
           <t>Art. 10</t>
@@ -1254,21 +1272,22 @@
       </c>
       <c r="D15" s="26" t="inlineStr">
         <is>
-          <t>[Met / Partially Met / Not Met]</t>
+          <t>Not Met</t>
         </is>
       </c>
       <c r="E15" s="26" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low]</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="F15" s="26" t="inlineStr">
         <is>
-          <t>[Evidence to prove compliance + remediation needed to close the gap]</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="50" customHeight="1">
+          <t>EVIDENCE OF GAP: (1) The training data is not representative. It comes only from IE+DE, but the system will also be deployed in the US (CA/MA/TX). (2) Label bias: under-served patients are under-diagnosed in Source 1, and the synthetic Source 2 reproduces that pattern rather than correcting it. (3) region and insurance_type are model features. insurance_type comes from billing and can be stale (a data-quality error), and Rural patients are 45% Medicaid, so the field acts as a proxy. (4) Our own check (test n=3,000, threshold 0.26) found FNR of 37.8% for Rural vs 22.7% for Urban (1.7x), 37.5% for Uninsured and 31.3% for Medicaid vs 20.8% for Medicare, and 48.9% for ages 21-35. (5) Manifest mismatch: train.csv has 12,000 rows, against the '~8,000' in the brief. No bias examination as required by Art. 10(2)(f)-(g) is on file.
+REMEDIATION: Document data governance per Art. 10(2): origin, labelling and assumptions. Run a bias examination and mitigation: drop region/insurance_type or justify them, reweight or adjust thresholds per group, and audit labels. Source real-world rural and under-served records. Validate on a US-representative cohort before the US launch. Add freshness and validation checks on insurance_type. Reconcile the training manifest hash with the actual dataset.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="321" customHeight="1">
       <c r="A16" s="11" t="inlineStr">
         <is>
           <t>Art. 10</t>
@@ -1286,21 +1305,23 @@
       </c>
       <c r="D16" s="26" t="inlineStr">
         <is>
-          <t>[Met / Partially Met / Not Met]</t>
+          <t>Partially Met</t>
         </is>
       </c>
       <c r="E16" s="26" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low]</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F16" s="26" t="inlineStr">
         <is>
-          <t>[Evidence to prove compliance + remediation needed to close the gap]</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="50" customHeight="1">
+          <t>EVIDENCE OF COMPLIANCE: Source 1 has explicit opt-in for secondary use under the DPA, and hospitals manage consent.
+GAPS: No DPIA (GDPR Art. 35) is referenced. The Art. 10(5) safeguards for using special-category data in bias work are not documented: strict necessity, pseudonymisation, access restriction, deletion once correction is done, and records of processing. The synthetic Source 2 was generated from real patients, and nobody has tested it for memorisation or re-identification. The Model Registry keeps every training dataset indefinitely (a minimisation and storage-limitation issue). US inference telemetry goes to Frankfurt without a documented transfer assessment.
+REMEDIATION: Complete a DPIA and record the GDPR Art. 9(2)(h)/(j) legal basis. Document the Art. 10(5)(a)-(f) safeguards. Run membership-inference and nearest-neighbour privacy tests on the synthetic data. Set a retention and deletion schedule and RBAC for training data in the registry. Data-map the telemetry flow and minimise or pseudonymise it (see D2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="336" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
           <t>Art. 11</t>
@@ -1318,21 +1339,31 @@
       </c>
       <c r="D17" s="26" t="inlineStr">
         <is>
-          <t>[Met / Partially Met / Not Met]</t>
+          <t>Not Met</t>
         </is>
       </c>
       <c r="E17" s="26" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low]</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F17" s="26" t="inlineStr">
         <is>
-          <t>[Evidence to prove compliance + remediation needed to close the gap]</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="50" customHeight="1">
+          <t>EVIDENCE OF GAP: All that exists is a model-card precursor: version healthguard-v1.0-rc7, training date 2027-03-12 and a manifest hash. The Annex IV elements are missing:
+- general description and intended purpose
+- design specs and architecture (6 components)
+- data requirements and provenance
+- validation and testing procedures and results, including subgroup metrics
+- human-oversight measures
+- RMS description
+- change-management / predetermined-change plan (relevant because overrides feed retraining)
+- post-market monitoring plan
+Under Art. 11(2) this must be one technical-documentation set, combined with MDR Annexes II/III.
+REMEDIATION: Compile the Annex IV technical file under version control, linked to the Model Registry artifact hash and data manifest. Use the D4 audit, D6 model card and D5 register as inputs, and keep the file current for every model version. The notified body needs it before conformity assessment, so this blocks CE marking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="261" customHeight="1">
       <c r="A18" s="11" t="inlineStr">
         <is>
           <t>Art. 12</t>
@@ -1350,21 +1381,23 @@
       </c>
       <c r="D18" s="26" t="inlineStr">
         <is>
-          <t>[Met / Partially Met / Not Met]</t>
+          <t>Partially Met</t>
         </is>
       </c>
       <c r="E18" s="26" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low]</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F18" s="26" t="inlineStr">
         <is>
-          <t>[Evidence to prove compliance + remediation needed to close the gap]</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="50" customHeight="1">
+          <t>EVIDENCE OF COMPLIANCE: Component 6 logs every request, response, clinician override and drift metric, with 7-year retention. That exceeds the Art. 19 minimum of 6 months and supports Art. 72.
+GAPS: The log schema is not mapped to Art. 12(2) (identifying risk situations or substantial modifications, post-market monitoring, deployer monitoring). Per-inference tagging of model version and clinician ID is unconfirmed. Logs have no integrity or tamper-evidence controls. Keeping identifiable feature vectors for 7 years conflicts with GDPR minimisation unless it is justified and the data is pseudonymised.
+REMEDIATION: Map log fields to Art. 12(2)(a)-(c). Stamp each record with model version, threshold and clinician. Use WORM or hash-chained storage with restricted access. Pseudonymise patient IDs in monitoring logs. Document the retention justification in the DPIA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="306" customHeight="1">
       <c r="A19" s="11" t="inlineStr">
         <is>
           <t>Art. 13</t>
@@ -1382,21 +1415,29 @@
       </c>
       <c r="D19" s="26" t="inlineStr">
         <is>
-          <t>[Met / Partially Met / Not Met]</t>
+          <t>Not Met</t>
         </is>
       </c>
       <c r="E19" s="26" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low]</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F19" s="26" t="inlineStr">
         <is>
-          <t>[Evidence to prove compliance + remediation needed to close the gap]</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="50" customHeight="1">
+          <t>EVIDENCE OF GAP: The dashboard shows only a 'rough explanation, not full SHAP', and there are no Instructions for Use. Art. 13(3) requires:
+- intended purpose
+- accuracy metrics and their levels, including for specific groups (Art. 13(3)(b)(v))
+- known limitations (worse FNR for Rural, Uninsured, Medicaid and young patients; a population not representative of the US)
+- foreseeable misuse
+- input-data specifications
+- oversight measures
+- how to interpret the output
+REMEDIATION: Publish IFU and a clinician-facing model card (D6) that disclose overall and subgroup performance and limitations. Replace the rough explanation with validated per-patient SHAP top factors, checked for fidelity. Show an inline caution when a patient belongs to a subgroup with higher FNR. State plainly that a 'not high-risk' result does not rule out diabetes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="261" customHeight="1">
       <c r="A20" s="11" t="inlineStr">
         <is>
           <t>Art. 14</t>
@@ -1414,21 +1455,23 @@
       </c>
       <c r="D20" s="26" t="inlineStr">
         <is>
-          <t>[Met / Partially Met / Not Met]</t>
+          <t>Partially Met</t>
         </is>
       </c>
       <c r="E20" s="26" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low]</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F20" s="26" t="inlineStr">
         <is>
-          <t>[Evidence to prove compliance + remediation needed to close the gap]</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="50" customHeight="1">
+          <t>EVIDENCE OF COMPLIANCE: A clinician reviews every prediction, and the dashboard has a sign-off step.
+GAPS: The Art. 14(4)(a)-(c) measures are missing: no clinician training on capabilities and limits, no automation-bias controls, and no display of uncertainty. The main failure mode is a false 'not high-risk' result. Clinicians rarely question a reassuring score, so the human check is weakest exactly where subgroup FNR is highest. Deployer guidance under Art. 26 (competent oversight staff) has not been issued.
+REMEDIATION: Make clinician training mandatory, with sign-off. Show a calibrated probability band and a borderline-zone flag instead of just a binary label. Add subgroup caution prompts, and prompt clinicians to apply standard screening criteria (e.g., ADA/FINDRISC) to negative results. Track override and concordance rates by subgroup as a KRI. Give deployers an oversight SOP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="216" customHeight="1">
       <c r="A21" s="11" t="inlineStr">
         <is>
           <t>Art. 14</t>
@@ -1446,21 +1489,23 @@
       </c>
       <c r="D21" s="26" t="inlineStr">
         <is>
-          <t>[Met / Partially Met / Not Met]</t>
+          <t>Partially Met</t>
         </is>
       </c>
       <c r="E21" s="26" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low]</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F21" s="26" t="inlineStr">
         <is>
-          <t>[Evidence to prove compliance + remediation needed to close the gap]</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="50" customHeight="1">
+          <t>EVIDENCE OF COMPLIANCE: Clinicians can disagree with the score, and overrides are logged (Art. 14(4)(d)).
+GAPS: There is no documented 'stop' / suspend capability for the deployer or provider (Art. 14(4)(e)), such as a kill-switch per hospital or per model version. Override reasons are not captured in a structured form. Overrides flow straight into retraining data without review, which creates a feedback loop and a poisoning path (see Art. 15).
+REMEDIATION: Build and test a per-tenant kill-switch with rollback to the previous model version. Add structured override-reason codes. Put a human-reviewed quarantine step in front of any override data used for retraining. Show the evidence in a runbook and a tested drill.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="276" customHeight="1">
       <c r="A22" s="11" t="inlineStr">
         <is>
           <t>Art. 15</t>
@@ -1478,21 +1523,23 @@
       </c>
       <c r="D22" s="26" t="inlineStr">
         <is>
-          <t>[Met / Partially Met / Not Met]</t>
+          <t>Partially Met</t>
         </is>
       </c>
       <c r="E22" s="26" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low]</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="F22" s="26" t="inlineStr">
         <is>
-          <t>[Evidence to prove compliance + remediation needed to close the gap]</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="50" customHeight="1">
+          <t>EVIDENCE: Overall performance at threshold 0.26 is ROC AUC 0.812, recall 0.744 and precision 0.476. That is reasonable for a sensitivity-tuned screening aid.
+GAPS: Accuracy is not appropriate for every group. Rural FNR is 37.8% and Uninsured FNR is 37.5%, against 22.7% for Urban and 20.8% for Medicare. Nothing compares performance with standard of care (e.g., FINDRISC or the ADA risk test), so the risk-appetite test ('not materially worse than standard of care') cannot be shown. No external validation has been done (brief Section 8). Accuracy levels are not declared in the IFU (Art. 15(3)).
+REMEDIATION: Agree a subgroup-FNR acceptance criterion with the AI Review Board, e.g., no group's FNR worse than standard of care and a max/min FNR ratio of 1.25x or less. Re-validate after mitigation. Commission independent external validation on held-out EU sites, and on US sites before the US launch. Declare the metrics in the IFU.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="276" customHeight="1">
       <c r="A23" s="11" t="inlineStr">
         <is>
           <t>Art. 15</t>
@@ -1510,21 +1557,23 @@
       </c>
       <c r="D23" s="26" t="inlineStr">
         <is>
-          <t>[Met / Partially Met / Not Met]</t>
+          <t>Partially Met</t>
         </is>
       </c>
       <c r="E23" s="26" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low]</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F23" s="26" t="inlineStr">
         <is>
-          <t>[Evidence to prove compliance + remediation needed to close the gap]</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="50" customHeight="1">
+          <t>EVIDENCE OF COMPLIANCE: Drift metrics are captured, and the threshold is fixed and recorded with the model.
+GAPS: No robustness testing has been done on missing or out-of-range inputs, stale insurance_type values, or a shift in population (EU to US). The pipeline's OneHotEncoder(handle_unknown='ignore') silently zeroes unseen categories, such as a new US insurance code, instead of failing safe. Drift has no alert thresholds. Feeding overrides into retraining with no controls creates biased feedback loops, which Art. 15(4) says must be addressed.
+REMEDIATION: Validate the input schema and value ranges at the Inference API, and reject or flag unknown categories. Run a perturbation, missingness and category-shift test suite in CI. Turn drift metrics into KRIs with thresholds (D7). Add a governance gate for retraining (Art. 15(4)), and fall back safely to standard screening when inputs fail validation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="291" customHeight="1">
       <c r="A24" s="11" t="inlineStr">
         <is>
           <t>Art. 15</t>
@@ -1542,17 +1591,19 @@
       </c>
       <c r="D24" s="26" t="inlineStr">
         <is>
-          <t>[Met / Partially Met / Not Met]</t>
+          <t>Partially Met</t>
         </is>
       </c>
       <c r="E24" s="26" t="inlineStr">
         <is>
-          <t>[Critical / High / Medium / Low]</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F24" s="26" t="inlineStr">
         <is>
-          <t>[Evidence to prove compliance + remediation needed to close the gap]</t>
+          <t>EVIDENCE OF COMPLIANCE: mTLS at the hospital edge, and rate limiting at 200 requests/min per hospital.
+GAPS: The model ships as a joblib pickle. Loading it can execute arbitrary code, and nothing checks its integrity (a model-tampering / supply-chain risk). The Model Registry holds every training dataset, which makes it a high-value target. Unvetted override feedback is a data-poisoning path (ATLAS AML.T0020). The inference API allows high-volume querying, which enables model extraction or inversion. No AI-specific pen test or red-team exercise has been done.
+REMEDIATION: Sign artifacts and verify their hash at load time, or move to a safe format (skops/ONNX). Apply least-privilege RBAC and audit logging to the registry, and encrypt training data. Add poisoning controls on feedback data. Detect anomalous query patterns and tighten per-client quotas. Before launch, run an AI red-team exercise against the D3 ATLAS TTPs, and produce an SBOM for dependencies.</t>
         </is>
       </c>
     </row>
@@ -1563,10 +1614,19 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="120" customHeight="1">
+    <row r="27" ht="355" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>[Identify the top 2–3 launch-blocking gaps in priority order. For each, explain why it is launch-blocking under the company's risk appetite (see A1) and what would need to be true to clear it.]</t>
+          <t>1) SUBGROUP UNDER-DETECTION (Art. 10 data governance + Art. 15 accuracy). CRITICAL, LAUNCH-BLOCKING.
+Why it blocks: Patient-safety appetite is LOW. The Board will not deploy a system whose 'foreseeable failure modes can produce a missed diagnosis or delayed referral for any identifiable patient subgroup at a rate materially worse than standard of care.' HealthGuard misses 37.8% of true diabetes cases in Rural patients and 37.5% in Uninsured patients, against about 21-23% for Urban and Medicare patients. The cause is identifiable: region and insurance_type act as socio-economic proxies, and the training labels carry historical under-diagnosis that the synthetic data copies. Human oversight cannot make up for this, because clinicians are least likely to question a reassuring 'not high-risk' result.
+To clear: Mitigate the bias (remove or justify the proxy features, reweight or set per-group thresholds, audit the labels). Then show through independent external validation that every subgroup's FNR is within the Board-approved tolerance (e.g., a max/min ratio of 1.25x or less) and no worse than a standard-of-care baseline such as FINDRISC. A US-representative validation is a separate gate before the US launch.
+2) NO LAWFUL ROUTE TO MARKET: MDR qualification, conformity assessment and technical documentation (Art. 6(1), 9, 11, 17, 43). CRITICAL, LAUNCH-BLOCKING.
+Why it blocks: Appetite for regulatory non-compliance is LOW. The Board 'will not deploy a system that we know to be non-compliant.' HealthGuard is high-risk via Annex I/MDR. It cannot be placed on the EU market without a QMS, an Annex IV technical file, a documented RMS, notified-body conformity assessment, a declaration of conformity, CE marking and EU database registration. The partial-compliance exception does not apply here. No compensating control can stand in for a missing conformity assessment, and launching without one is a regulator-reportable event (reputational appetite: LOW).
+To clear: Obtain a formal MDR qualification and classification opinion (expect Class IIa) and engage a notified body. Complete the Annex IV/MDR technical file, the RMS and the QMS. Pass conformity assessment, then sign the DoC and register the system before the first EU patient is scored.
+3) TRANSPARENCY AND HUMAN OVERSIGHT DO NOT WORK (Art. 13 + Art. 14). HIGH; BLOCKS LAUNCH BECAUSE IT IS THE COMPENSATING CONTROL.
+Why it blocks: The Board's 'partial compliance with an approved compensating control' route would rely on clinician review to accept any residual subgroup risk. Today that control is not effective. Clinicians get no IFU and no subgroup performance figures or limitations, only a rough explanation. They have no training and no safeguards against automation bias, and overrides go straight into retraining.
+To clear: Issue an IFU and model card that disclose subgroup FNR and limitations. Ship validated per-patient explanations and subgroup caution flags, and deliver mandatory clinician training. Track override and concordance KRIs by subgroup. Have a tested kill-switch and rollback, and a review gate before override data is used for retraining.
+Next tier (must-fix, but can be fixed after launch under a dated plan): Art. 15 cybersecurity (unsigned pickle artifact, registry access, poisoning via feedback), Art. 10(5)/GDPR safeguards (DPIA, privacy testing of the synthetic data, cross-border telemetry), and Art. 12 log integrity.</t>
         </is>
       </c>
       <c r="B27" s="5" t="n"/>
@@ -1600,10 +1660,10 @@
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="62" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1670,7 +1730,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="70" customHeight="1">
+    <row r="6" ht="186" customHeight="1">
       <c r="A6" s="11" t="inlineStr">
         <is>
           <t>1</t>
@@ -1688,26 +1748,32 @@
       </c>
       <c r="D6" s="26" t="inlineStr">
         <is>
-          <t>[GDPR obligation(s) at this stage — cite specific Articles]</t>
+          <t>The hospital is the controller. Lawful basis: Art. 6(1)(e)/(c) plus Art. 9(2)(h) (provision of health care), with any national health-data conditions under Art. 9(4) for records arriving via cross-border registries.
+Arts 13/14: patient notices must cover AI risk scoring and name Klariova as a recipient.
+Art. 28(3): the DPA with Klariova.
+Art. 35: DPIA (large-scale health data, new technology, profiling), with Klariova assisting under Art. 28(3)(f).</t>
         </is>
       </c>
       <c r="E6" s="26" t="inlineStr">
         <is>
-          <t>[CPRA obligation(s) at this stage — cite specific Sections]</t>
+          <t>Patient PHI held by the CA hospital is exempt from CCPA/CPRA (Civ. Code §1798.146(a)(1)(A)). It falls under HIPAA and CMIA (Civ. Code §56.10) instead, so a HIPAA BAA is required (45 CFR §164.502(e), §164.504(e)).
+CPRA still covers non-PHI personal information, such as clinician users: the hospital gives notice at collection under §1798.100(a).</t>
         </is>
       </c>
       <c r="F6" s="26" t="inlineStr">
         <is>
-          <t>[Met / Gap]</t>
+          <t>Gap</t>
         </is>
       </c>
       <c r="G6" s="26" t="inlineStr">
         <is>
-          <t>[Specific gap, evidence needed, or remediation]</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="70" customHeight="1">
+          <t>MET: the DPA exists, and consent management is assigned to the hospital.
+GAP: Klariova has no evidence that (a) each EU hospital's privacy notice covers AI risk scoring, (b) hospital DPIAs exist, or (c) US BAAs are signed and allow EU sub-processing. Having no consent capture is acceptable for treatment under Art. 9(2)(h) and HIPAA treatment/payment/operations, but it does NOT cover secondary use for retraining (see stage 7).
+CLOSE: add a DPA annex requiring notice wording and a DPIA attestation from each hospital. Execute a BAA with each US IDN before go-live. Check data from cross-border registries against national health-data law (Art. 9(4)).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="141" customHeight="1">
       <c r="A7" s="11" t="inlineStr">
         <is>
           <t>2</t>
@@ -1725,26 +1791,33 @@
       </c>
       <c r="D7" s="26" t="inlineStr">
         <is>
-          <t>[GDPR obligation(s) at this stage — cite specific Articles]</t>
+          <t>Art. 32 / Art. 28(3)(c): security of processing (mTLS gives authenticated encryption in transit).
+Art. 5(1)(c): minimisation. Whole FHIR records arrive, but the model uses 13 fields.
+Art. 5(1)(e): retention in the Kafka buffer.
+Art. 33(2): the processor notifies the controller of a breach without undue delay.
+Art. 30(2): the processor's record of processing.</t>
         </is>
       </c>
       <c r="E7" s="26" t="inlineStr">
         <is>
-          <t>[CPRA obligation(s) at this stage — cite specific Sections]</t>
+          <t>PHI is exempt (§1798.146), so the HIPAA Security Rule applies: transmission security §164.312(e)(1) and audit controls §164.312(b).
+For any non-exempt PI: reasonable security (§1798.100(e)), the private right of action for breach (§1798.150), and minimisation (§1798.100(c)).</t>
         </is>
       </c>
       <c r="F7" s="26" t="inlineStr">
         <is>
-          <t>[Met / Gap]</t>
+          <t>Gap</t>
         </is>
       </c>
       <c r="G7" s="26" t="inlineStr">
         <is>
-          <t>[Specific gap, evidence needed, or remediation]</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="70" customHeight="1">
+          <t>MET: mTLS mutual authentication at the hospital edge.
+GAP: hospitals push full patient records every 15 min, which is more than the model needs. Kafka topic encryption at rest, ACLs and retention are not documented.
+CLOSE: set a field allow-list for FHIR resources so only the required Patient/Observation elements are pushed. Encrypt Kafka at rest, add per-topic ACLs and limit retention to 7 days or less. Write a breach-notification SLA (24h or less to the controller) into the DPA and BAA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="171" customHeight="1">
       <c r="A8" s="11" t="inlineStr">
         <is>
           <t>3</t>
@@ -1762,26 +1835,33 @@
       </c>
       <c r="D8" s="26" t="inlineStr">
         <is>
-          <t>[GDPR obligation(s) at this stage — cite specific Articles]</t>
+          <t>Art. 5(1)(a) fairness.
+Art. 5(1)(b) purpose limitation: data from the billing system is reused for clinical prediction.
+Art. 5(1)(c) minimisation: insurance_type and region have no clinical rationale.
+Art. 5(1)(d) accuracy: insurance_type may be stale.
+Art. 25 data protection by design.
+Art. 16: rectifications made at the source must flow through.</t>
         </is>
       </c>
       <c r="E8" s="26" t="inlineStr">
         <is>
-          <t>[CPRA obligation(s) at this stage — cite specific Sections]</t>
+          <t>PHI is exempt (§1798.146), so the HIPAA minimum-necessary standard applies (§164.502(b)).
+For non-exempt PI: processing must be reasonably necessary and proportionate (§1798.100(c)), consumers have a right to correct (§1798.106), and health data is sensitive PI (§1798.140(ae)).</t>
         </is>
       </c>
       <c r="F8" s="26" t="inlineStr">
         <is>
-          <t>[Met / Gap]</t>
+          <t>Gap</t>
         </is>
       </c>
       <c r="G8" s="26" t="inlineStr">
         <is>
-          <t>[Specific gap, evidence needed, or remediation]</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="70" customHeight="1">
+          <t>GAP: joining insurance_type (from billing, possibly out of date) and region adds socio-economic proxies with no clinical need. D1/D4 show these features track the FNR disparity: Rural 37.8% and Uninsured 37.5%, vs 22.7% Urban and 20.8% Medicare. Feeding inaccurate data into a health decision breaches Art. 5(1)(d) and the fairness principle in Art. 5(1)(a).
+CLOSE: drop insurance_type and region from the feature set, or document a necessity test in the DPIA. If either is kept, add a freshness check against the billing-change date with an 'unknown' fallback. Flag imputed values. Pass corrections from the hospital's systems through to the pipeline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="171" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
         <is>
           <t>4</t>
@@ -1799,26 +1879,32 @@
       </c>
       <c r="D9" s="26" t="inlineStr">
         <is>
-          <t>[GDPR obligation(s) at this stage — cite specific Articles]</t>
+          <t>Art. 22 / Art. 4(4) profiling: the decision is not solely automated because a clinician reviews it. But in CJEU C-634/21 (SCHUFA), a score that a third party 'draws strongly on' was itself treated as the decision, so the human review must be meaningful.
+Arts 13(2)(f)/14(2)(g)/15(1)(h): meaningful information about the logic (delivered via the hospital).
+Art. 35(3)(a): a DPIA is mandatory.
+Art. 32: API security.</t>
         </is>
       </c>
       <c r="E9" s="26" t="inlineStr">
         <is>
-          <t>[CPRA obligation(s) at this stage — cite specific Sections]</t>
+          <t>PHI is exempt, so HIPAA applies.
+For any non-exempt PI, the CCPA regulations apply from 2027. ADMT rules (11 CCR §7200 et seq.; 'significant decisions' include healthcare services) require a pre-use notice, opt-out or human appeal, and access. A risk assessment is also required (11 CCR §7150).</t>
         </is>
       </c>
       <c r="F9" s="26" t="inlineStr">
         <is>
-          <t>[Met / Gap]</t>
+          <t>Gap</t>
         </is>
       </c>
       <c r="G9" s="26" t="inlineStr">
         <is>
-          <t>[Specific gap, evidence needed, or remediation]</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="70" customHeight="1">
+          <t>MET: rate limit of 200 req/min per hospital; the output goes only to the clinician.
+GAP: there is no DPIA. Controllers get no plain-language explanation of the logic to put in their notices. Nothing shows the human review is meaningful (no override-rate monitoring). Authorisation stops at hospital level, with no per-user check.
+CLOSE: write a DPIA led by Klariova for hospitals to adopt. Publish a plain-language logic notice. Track override and concordance rates as a KRI to show the review is real. Add per-user OAuth scopes and log the purpose of each call.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="186" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
           <t>5</t>
@@ -1836,26 +1922,35 @@
       </c>
       <c r="D10" s="26" t="inlineStr">
         <is>
-          <t>[GDPR obligation(s) at this stage — cite specific Articles]</t>
+          <t>Art. 5(1)(e) storage limitation: patient identifiers and feature vectors are kept 7 years.
+Art. 5(1)(c) minimisation.
+Art. 32: encryption at rest, RBAC, pseudonymisation.
+Art. 28(3)(e): Klariova helps the controller answer requests under Arts 15-17 and 21.
+Art. 28(3)(g): data is deleted or returned when the contract ends.
+Art. 30: record of processing.
+Regional residency avoids a Chapter V transfer for EU data.</t>
         </is>
       </c>
       <c r="E10" s="26" t="inlineStr">
         <is>
-          <t>[CPRA obligation(s) at this stage — cite specific Sections]</t>
+          <t>Retention period must be disclosed (§1798.100(a)(3)); minimisation (§1798.100(c)); deletion right (§1798.105, for non-exempt PI); breach liability (§1798.150).
+HIPAA: encryption (§164.312(a)(2)(iv)) and access logging (§164.312(b)).</t>
         </is>
       </c>
       <c r="F10" s="26" t="inlineStr">
         <is>
-          <t>[Met / Gap]</t>
+          <t>Gap</t>
         </is>
       </c>
       <c r="G10" s="26" t="inlineStr">
         <is>
-          <t>[Specific gap, evidence needed, or remediation]</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="70" customHeight="1">
+          <t>MET: data stays in its region (EU in Frankfurt, US in AWS US-East).
+GAP: patient identifiers and full feature vectors are kept for 7 years. EU AI Act Art. 72 requires a post-market monitoring system, not 7 years of identifiable data, and Art. 19 sets a minimum of 6 months for logs. There is no erasure workflow and no retention schedule.
+CLOSE: split the store. Keep identifiable predictions under each hospital's medical-record retention policy (the controller decides). Keep the monitoring copy pseudonymised, with tokenised patient IDs and the keys held by the hospital. Document a retention schedule, an erasure/DSAR workflow, KMS encryption, RBAC and access logging.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="171" customHeight="1">
       <c r="A11" s="11" t="inlineStr">
         <is>
           <t>6</t>
@@ -1873,26 +1968,33 @@
       </c>
       <c r="D11" s="26" t="inlineStr">
         <is>
-          <t>[GDPR obligation(s) at this stage — cite specific Articles]</t>
+          <t>Arts 5(1)(f) and 32: access control (treating clinician only) and an audit trail.
+Art. 25(2): data protection by default (show only the data the decision needs).
+Art. 22(3) and Recital 71: meaningful human intervention.
+Arts 6 and 88, plus Art. 13 notice to clinicians: per-clinician override data is processing of staff data.
+Art. 5(1)(b): override data is reused for retraining.</t>
         </is>
       </c>
       <c r="E11" s="26" t="inlineStr">
         <is>
-          <t>[CPRA obligation(s) at this stage — cite specific Sections]</t>
+          <t>Clinicians' PI has been fully in CPRA scope since 1 Jan 2023. The hospital gives notice at collection (§1798.100(a)). Klariova acts as a service provider (§1798.140(ag)) under a contract meeting §1798.100(d). Clinicians have rights under §1798.105, §1798.106 and §1798.110.
+Patient PHI on screen falls under HIPAA minimum necessary and access logging (§164.312(b)).</t>
         </is>
       </c>
       <c r="F11" s="26" t="inlineStr">
         <is>
-          <t>[Met / Gap]</t>
+          <t>Gap</t>
         </is>
       </c>
       <c r="G11" s="26" t="inlineStr">
         <is>
-          <t>[Specific gap, evidence needed, or remediation]</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="70" customHeight="1">
+          <t>MET: there is a human sign-off step, and overrides are logged.
+GAP: RBAC, a care-relationship check and break-glass access are not described. Per-clinician override data is a new processing of staff data with no stated purpose or limit, so it could end up used for performance management. The dashboard shows 'patient history' beyond what the decision needs.
+CLOSE: check role and care relationship before showing a patient, with break-glass access that is reviewed afterwards. Restrict override data to model-quality use and aggregate reporting. Give clinicians a privacy notice. Reduce the patient history shown.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="201" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
           <t>7</t>
@@ -1910,26 +2012,33 @@
       </c>
       <c r="D12" s="26" t="inlineStr">
         <is>
-          <t>[GDPR obligation(s) at this stage — cite specific Articles]</t>
+          <t>Klariova decides the purposes of model development, so for that purpose it is the controller (Art. 4(7); Art. 28(10)). It therefore needs its own basis under Art. 6 and Art. 9(2)(j) with Art. 89(1) safeguards, or explicit consent under Art. 9(2)(a).
+Art. 6(4): compatibility test for reusing inference and override data.
+Recital 26 and EDPB Opinion 28/2024: models and synthetic data are not automatically anonymous.
+Art. 5(1)(e): every dataset is kept indefinitely.
+Art. 32.</t>
         </is>
       </c>
       <c r="E12" s="26" t="inlineStr">
         <is>
-          <t>[CPRA obligation(s) at this stage — cite specific Sections]</t>
+          <t>De-identified patient information is exempt only if it meets HIPAA de-identification (§164.514(b)) and the contract terms in §1798.146(a)(4). Re-identification is prohibited (§1798.148). The privacy policy must disclose it (§1798.130(a)(5)).
+HIPAA: a BA may use PHI for model development only if its BAA permits that use.</t>
         </is>
       </c>
       <c r="F12" s="26" t="inlineStr">
         <is>
-          <t>[Met / Gap]</t>
+          <t>Gap</t>
         </is>
       </c>
       <c r="G12" s="26" t="inlineStr">
         <is>
-          <t>[Specific gap, evidence needed, or remediation]</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="70" customHeight="1">
+          <t>MET: Source 1 has explicit opt-in for secondary use, and the manifest hash is recorded.
+GAP: (a) override and inference data fed back for retraining has no secondary-use basis and is outside the processor mandate. (b) Synthetic Source 2 has not been tested for re-identification or memorisation. (c) Every dataset ever used is kept indefinitely in one store. (d) Access control is not documented.
+CLOSE: decide Klariova's role, then amend the DPA/BAA or set up an Art. 26 joint-controller arrangement. Run an Art. 6(4) / 9(2)(j) assessment, or collect opt-in. Run membership-inference and distance-to-closest-record tests before calling the synthetic data anonymous. Keep manifests and hashes but delete raw datasets after a set period. Add RBAC, encryption and an audit log to the registry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="171" customHeight="1">
       <c r="A13" s="11" t="inlineStr">
         <is>
           <t>8</t>
@@ -1947,22 +2056,28 @@
       </c>
       <c r="D13" s="26" t="inlineStr">
         <is>
-          <t>[GDPR obligation(s) at this stage — cite specific Articles]</t>
+          <t>Art. 3(1): Frankfurt processing happens in the context of Klariova's EU establishment, so GDPR applies even to US patients' data.
+Arts 4(1)/4(5) and Recital 26: request metadata that can be linked to the US prediction DB is pseudonymised personal (health-derived) data.
+Chapter V (Arts 44-46) does NOT apply to the US→EU leg, but DOES apply to any EU→US return flow. Those need DPF adequacy (Art. 45) or SCCs (Art. 46(2)(c)).
+Arts 28, 30(2) and 32 apply.</t>
         </is>
       </c>
       <c r="E13" s="26" t="inlineStr">
         <is>
-          <t>[CPRA obligation(s) at this stage — cite specific Sections]</t>
+          <t>CPRA has no transfer restriction, but the service-provider contract must cover offshore processing (§1798.100(d), §1798.140(ag)).
+If the data is PHI: a HIPAA subcontractor BAA between Klariova Inc. (US) and Klariova Ltd (EU) (§164.502(e)(1)(ii), §164.504(e)(2)(ii)(D)), plus CMIA §56.10.
+Texas SB 1188 (2025) requires Texas patients' EHR to be stored in the US. Confirm the telemetry is out of scope.</t>
         </is>
       </c>
       <c r="F13" s="26" t="inlineStr">
         <is>
-          <t>[Met / Gap]</t>
+          <t>Gap</t>
         </is>
       </c>
       <c r="G13" s="26" t="inlineStr">
         <is>
-          <t>[Specific gap, evidence needed, or remediation]</t>
+          <t>GAP: nobody has tested the 'metadata, not full records' claim. Hospital ID, timestamp, request or patient ID and feature-drift statistics can be linked back to a patient and are derived from health data. There is no identifiability assessment, no RoPA entry, no intra-group BAA or DPA, and no transfer mechanism for return flows (alerts or dashboards viewed from Boston).
+CLOSE: see Section B. In short: send aggregate statistics only, register DPF plus SCCs Module 4, sign an intra-group subcontractor BAA, and update the RoPA.</t>
         </is>
       </c>
     </row>
@@ -1973,10 +2088,13 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="80" customHeight="1">
+    <row r="16" ht="190" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>[Address the US→EU telemetry flow described in A1 §6. Name the specific transfer mechanism that applies (SCCs / adequacy / BCRs). State whether a Transfer Impact Assessment is required and why. Note any update needed to the Article 30 RoPA.]</t>
+          <t>1) WHAT FLOWS. For drift monitoring, inference request metadata from AWS US-East goes to the Frankfurt data centre: hospital ID, timestamps, model version, request/patient IDs, feature-value distributions and latency. Klariova also holds the US prediction database that maps request IDs to patients. That makes this metadata pseudonymised personal data, and because it describes clinical feature values it is health data (GDPR Arts 4(1), 4(5), 4(15); Recital 26). Not being 'full patient records' does not make it anonymous. Klariova can re-identify it, so the SRB v EDPS (C-413/23 P) recipient-perspective argument does not help.
+2) IS IT A GDPR TRANSFER? The US→EU leg is NOT a Chapter V transfer, because Chapter V regulates exports OUT of the EEA. But once the data is in Frankfurt it is processed in the context of Klariova's EU establishment, so GDPR applies in full (Art. 3(1)): processor terms, Art. 32 security, Art. 30 records, Art. 33 breach handling, and requests from US data subjects. Chapter V IS triggered by the return legs: drift alerts or reports sent to the US, monitoring dashboards opened from Boston, remote access to Frankfurt by US-subsidiary engineers, and any onward sharing with US hospitals.
+3) MECHANISM. Primary: the EU-US Data Privacy Framework adequacy decision (Art. 45; in force since 10 Jul 2023; upheld by the General Court in Latombe, T-553/23, Sep 2025). This requires Klariova Health Inc. to self-certify with the US Dept. of Commerce. Fallback, given the political risk to the DPF: 2021 SCCs (Decision 2021/914) in an intra-group data-transfer agreement. Use Module 4 (EU processor → non-EU controller) where Frankfurt sends US hospitals' own data back to them. Use Module 1/2 where Klariova Ltd, as controller for AI Act Art. 72 post-market monitoring, shares data with Klariova Inc. BCRs are disproportionate for a group of two entities.
+4) TRANSFER IMPACT ASSESSMENT. NOT legally required for the US→EU leg, because there is no Chapter V transfer. REQUIRED (Schrems II C-311/18; SCC Clause 14; EDPB Recommendations 01/2020) for any EU→US return that relies on SCCs. Under Module 4, Clause 14 applies only if the EU processor combines the US data with data it collected in the EU, and pooled EU+US drift monitoring will do that. No TIA is needed while relying on DPF adequacy. Recommendation: document a short TIA now anyway, relying on EO 14086 and the Data Protection Review Court, so the SCC fallback is ready the day the DPF falls.</t>
         </is>
       </c>
       <c r="B16" s="5" t="n"/>
@@ -1986,6 +2104,29 @@
       <c r="F16" s="5" t="n"/>
       <c r="G16" s="6" t="n"/>
     </row>
+    <row r="17" ht="220" customHeight="1">
+      <c r="A17" s="26" t="inlineStr">
+        <is>
+          <t>5) US-SIDE LAWFULNESS. The flow must also be lawful under US law. That needs a HIPAA subcontractor BAA between Klariova Inc. and Klariova Ltd (45 CFR §164.502(e)(1)(ii), §164.504(e)(2)(ii)(D)), and hospital BAAs that allow offshore processing (many IDN BAAs forbid it). It also needs the CMIA §56.10 disclosure rules for the CA hospital, confirmation that the Texas SB 1188 requirement to store EHR in the US does not reach the telemetry, and CPRA service-provider terms (§1798.100(d)) for any PI that is not PHI.
+6) MINIMISE FIRST. This is the best control. Send aggregate drift statistics instead of per-request rows: per-feature histograms and PSI per hospital per day, with a minimum cell size of 20 or more. Drop patient and request IDs. If per-request data really is needed, tokenise it with keys held only in US-East. Truly aggregate statistics are no longer personal data, which removes most of points 2-5.
+7) ARTICLE 30 RoPA UPDATE. Add a processing activity called 'Model-drift monitoring of US inference telemetry', recording:
+- Klariova's role: processor for the US hospitals, or controller for AI Act Art. 72 post-market monitoring (this needs deciding).
+- The names of the controllers.
+- Data subjects: US patients, and US clinicians if user IDs are included.
+- Data categories: pseudonymised request metadata and health-derived feature statistics.
+- Recipients: Klariova Inc. staff.
+- Third-country transfers and their mechanism: DPF / SCCs Module 4.
+- Retention period, and the Art. 32 measures.
+Mirror the entry in the processor record (Art. 30(2)) and the HIPAA asset inventory, and reference it in the DPIA.</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n"/>
+      <c r="C17" s="5" t="n"/>
+      <c r="D17" s="5" t="n"/>
+      <c r="E17" s="5" t="n"/>
+      <c r="F17" s="5" t="n"/>
+      <c r="G17" s="6" t="n"/>
+    </row>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
@@ -1993,10 +2134,25 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="110" customHeight="1">
+    <row r="19" ht="400" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>[List the 5 most consequential compliance gaps you identified. Each will be carried forward to D5 (Risk Register) with a Likelihood × Impact score and a proposed control.]</t>
+          <t>Ranked by suggested D5 score (Likelihood × Impact, 1-5 scale). Each is carried into D5 as a row.
+C1. SECONDARY USE OF CLINICAL DATA FOR RETRAINING WITHOUT A LAWFUL BASIS (stages 6-7). L4 × I4 = 16. Privacy/Regulatory · Govern.
+Inference outputs and clinician overrides go into the Model Registry for retraining. That is a new purpose, outside Klariova's processor mandate (GDPR Arts 5(1)(b), 6(4), 9(2)(j), 28(10)) and probably outside HIPAA BA permitted uses. It would make Klariova a controller with no lawful basis for EU and US data alike.
+Control: a formal role decision and DPA/BAA amendment (or an Art. 26 joint-controller arrangement); an Art. 6(4) / 9(2)(j) + 89(1) assessment; quarantine all override data until a basis exists.
+C2. INACCURATE AND UNNECESSARY SOCIO-ECONOMIC DATA IN HEALTH PROFILING (stage 3). L4 × I4 = 16. Fairness/Privacy · Map/Measure.
+insurance_type (stale billing data) and region are processed with no clinical necessity, and they drive the subgroup FNR gap (Rural 37.8%, Uninsured 37.5%). This breaches the GDPR principles of fairness, minimisation and accuracy (Art. 5(1)(a), (c), (d)) and data protection by design (Art. 25). It is the same root cause as D1 gap #1.
+Control: remove both features or justify them in the DPIA with a necessity test; add a freshness check and an 'unknown' fallback; re-run the D4 audit.
+C3. NO DPIA AND NO PROFILING SAFEGUARDS (stages 1, 4). L5 × I3 = 15. Regulatory · Govern.
+Large-scale profiling on health data makes a DPIA mandatory (Art. 35(3)(a)), and none exists. Patient notices do not explain the logic (Arts 13(2)(f), 14(2)(g)), and nothing shows the human review would satisfy SCHUFA (C-634/21). In California, any non-PHI data is caught by the CCPA risk-assessment and ADMT regulations (11 CCR §7150, §7200).
+Control: a DPIA written by Klariova and adopted by each hospital before go-live; plain-language logic notice; override and concordance KRI as evidence of meaningful review.
+C4. US→EU TELEMETRY TREATED AS NON-PERSONAL AND UNGOVERNED (stage 8). L3 × I4 = 12. Privacy · Govern.
+The metadata can be linked back to patients and is derived from health data. GDPR applies in Frankfurt (Art. 3(1)). Return flows to the US have no DPF certification or SCCs, there is no HIPAA subcontractor BAA between the group companies, and the flow is not in the RoPA. Exposure: a GDPR Art. 83(5) fine of up to 4% of turnover, plus a HIPAA violation under the US hospitals' BAAs.
+Control: aggregate-only telemetry; DPF self-certification plus SCCs Module 4 as fallback; a short TIA; a subcontractor BAA; a RoPA entry.
+C5. OVER-COLLECTION AND OVER-RETENTION CONCENTRATE BREACH IMPACT (stages 2, 5, 7). L4 × I3 = 12. Privacy/Security · Manage.
+Hospitals push full FHIR records. Identifiable feature vectors are kept for 7 years, and every training dataset ever used sits indefinitely in the registry (GDPR Art. 5(1)(c), (e) and Art. 32; CPRA §1798.100(a)(3), (c); breach liability under §1798.150).
+Control: an allow-list of FHIR fields; a pseudonymised monitoring store; a documented retention schedule; KMS encryption, RBAC and access logging on the prediction DB and registry.</t>
         </is>
       </c>
       <c r="B19" s="5" t="n"/>
@@ -2007,8 +2163,9 @@
       <c r="G19" s="6" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A17:G17"/>
     <mergeCell ref="A18:G18"/>
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="A16:G16"/>
@@ -2030,13 +2187,13 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="38" customWidth="1" min="5" max="5"/>
-    <col width="38" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
+    <col width="62" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -2067,19 +2224,26 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="70" customHeight="1">
+    <row r="5" ht="235" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
         <is>
-          <t>[List the named architecture components from A1 §5 and the attack surface each presents. Use this as input to selecting the 3 TTPs.]</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="6" t="n"/>
+          <t>Upstream (external): Hospital EHR and billing systems. These are the trust boundary we do not control. The billing system supplies insurance_type, which is weakly governed and can be stale (D2 stage 3). Any compromise or data-quality failure here enters the model as 'truth'.
+C1 Data Ingestion Pipeline (HL7 FHIR R4 → Kafka). Surface: the mTLS client certificate held at each of the 7 hospital edges; Kafka topics (encryption at rest and ACLs are undocumented); full FHIR records pushed every 15 min. Threats: stolen hospital certificate used to inject records, eavesdropping on the buffer, replaying records.
+C2 Preprocessing Layer. Surface: the feature-engineering code; the join with billing demographics; imputation logic. Threats: tampered preprocessing code, manipulated insurance_type/region values. Silent imputation can hide input attacks.
+C3 Model Inference API (FastAPI + scikit-learn, loads a joblib pickle). Surface: accepts a raw feature vector, returns a full-precision probability, and allows 200 req/min per hospital (about 288k/day). Threats: query-based extraction, membership inference or inversion, adversarial inputs. Deserialising a pickle on load means arbitrary code execution.
+C4 Clinician-Facing Dashboard. Surface: web app, clinician credentials (phishing is the leading healthcare breach vector), override capture. Threats: account takeover, malicious or systematically biased overrides that become training labels.
+C5 Model Registry. Surface: every model artifact, training-data manifest and training dataset ever used, plus override feedback. It is the highest-value target. Threats: artifact substitution (supply chain), training-data poisoning, bulk exfiltration of patient training data.
+C6 Logging &amp; Monitoring. Surface: 7 years of inference logs with patient IDs; cross-border US→EU telemetry (D2 stage 8). Threats: log tampering to hide an attack, exfiltration, poisoning of drift baselines so real drift does not alert.
+→ Where the surface is largest: the C4→C5 feedback loop (untrusted labels flow straight into training), the C5→C3 artifact path (unsigned pickle is loaded in production), and C3 API exposure (raw vectors in, raw probabilities out). The three TTPs below are chosen from these.</t>
+        </is>
+      </c>
+      <c r="B5" s="45" t="n"/>
+      <c r="C5" s="45" t="n"/>
+      <c r="D5" s="45" t="n"/>
+      <c r="E5" s="45" t="n"/>
+      <c r="F5" s="45" t="n"/>
+      <c r="G5" s="45" t="n"/>
+      <c r="H5" s="46" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
@@ -2130,7 +2294,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="110" customHeight="1">
+    <row r="9" ht="321" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
         <is>
           <t>1</t>
@@ -2138,41 +2302,52 @@
       </c>
       <c r="B9" s="26" t="inlineStr">
         <is>
-          <t>[AML.T####]</t>
+          <t>AML.T0020</t>
         </is>
       </c>
       <c r="C9" s="26" t="inlineStr">
         <is>
-          <t>[Technique name]</t>
+          <t>Poison Training Data
+(tactic: Resource Development; related: AML.T0018.000 Poison AI Model, AML.T0019 Publish Poisoned Datasets)</t>
         </is>
       </c>
       <c r="D9" s="26" t="inlineStr">
         <is>
-          <t>[Specific Component (1-6)]</t>
+          <t>C4 Clinician Dashboard → C5 Model Registry (override feedback loop). Secondary: Source 2 synthetic-data generator.</t>
         </is>
       </c>
       <c r="E9" s="26" t="inlineStr">
         <is>
-          <t>[Concrete attack scenario in the healthcare context]</t>
+          <t>ACTOR: a malicious insider, or an attacker who has phished a clinician's credentials at one of the 7 launch hospitals. The same effect also happens with no attacker at all, if clinicians systematically dismiss flags for under-served patients.
+1. The attacker logs in to the C4 dashboard as a legitimate clinician.
+2. Over 8-12 weeks they record 'disagree - not high-risk' overrides on true-positive patients in a narrow subgroup, e.g. Medicaid patients aged 21-35, around 5 a day so each one looks like ordinary clinical judgement.
+3. Every override is written to the C5 Model Registry and becomes a training label. Nothing reviews or caps it.
+4. At the next retraining (healthguard-v1.1), the model learns that this subgroup is low-risk. If the poisoned rows also seed the Source 2 generator, the synthetic data multiplies them.
+5. The subgroup is small, so overall AUC moves less than 0.01 and the release passes. Subgroup FNR, already 31-49% (D4), rises further.
+IMPACT: missed or late T2D diagnoses for an identifiable, already disadvantaged group. This breaches the Board's low patient-safety appetite and is a reportable serious incident (AI Act Art. 73). It is invisible to aggregate monitoring.</t>
         </is>
       </c>
       <c r="F9" s="26" t="inlineStr">
         <is>
-          <t>[Specific control — name a mechanism, not 'monitor the system']</t>
-        </is>
-      </c>
-      <c r="G9" s="26" t="inlineStr">
-        <is>
-          <t>[H / M-H / M / L-M / L]</t>
-        </is>
-      </c>
-      <c r="H9" s="26" t="inlineStr">
-        <is>
-          <t>[H / M / L]</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="110" customHeight="1">
+          <t>Targets the integrity of the training pipeline (ATLAS AML.M0007 Sanitize Training Data, AML.M0025 Maintain AI Dataset Provenance, AML.M0008 Validate AI Model):
+1. OVERRIDE QUARANTINE: overrides go to a separate staging table and are never used for training until a second clinician adjudicates a stratified sample. Structured reason codes are mandatory.
+2. CONTRIBUTION CAPS AND ANOMALY CHECKS: cap the number of override labels any one clinician or site can contribute per release. Run per-clinician override-rate z-scores by subgroup, and screen for label errors with cleanlab (confident learning) before training.
+3. SUBGROUP REGRESSION GATE in CI: score each candidate model on a frozen, clinician-adjudicated golden test set that only the release pipeline can read. Block promotion if any region, insurance or age subgroup's FNR rises by more than 2 percentage points, or breaches the D7 KRI threshold (lab/kri.py).
+4. LINEAGE: version the training data in DVC or lakeFS, with the sha256 manifest signed and recorded in the registry, so a poisoned batch can be traced and rolled back.</t>
+        </is>
+      </c>
+      <c r="G9" s="47" t="inlineStr">
+        <is>
+          <t>M-H</t>
+        </is>
+      </c>
+      <c r="H9" s="47" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="306" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
           <t>2</t>
@@ -2180,41 +2355,53 @@
       </c>
       <c r="B10" s="26" t="inlineStr">
         <is>
-          <t>[AML.T####]</t>
+          <t>AML.T0010.003</t>
         </is>
       </c>
       <c r="C10" s="26" t="inlineStr">
         <is>
-          <t>[Technique name]</t>
+          <t>AI Supply Chain Compromise: Model
+(related: AML.T0011.000 User Execution: Unsafe AI Artifacts; AML.T0018 Manipulate AI Model)</t>
         </is>
       </c>
       <c r="D10" s="26" t="inlineStr">
         <is>
-          <t>[Specific Component (1-6)]</t>
+          <t>C5 Model Registry → C3 Model Inference API (loading the joblib artifact).</t>
         </is>
       </c>
       <c r="E10" s="26" t="inlineStr">
         <is>
-          <t>[Concrete attack scenario in the healthcare context]</t>
+          <t>ACTOR: an attacker holding stolen ML-engineer or CI/CD credentials, or a compromised dependency in the training environment.
+1. They build a joblib/pickle file that wraps the real healthguard GradientBoostingClassifier and adds a __reduce__ payload. Predictions still look normal.
+2. They upload it to the C5 registry as healthguard-v1.0-rc8, or overwrite rc7. No signature check exists, and the brief records only a manifest hash for the data, not for the model.
+3. On the next deployment, the C3 FastAPI service calls joblib.load() and the payload runs with the service's privileges inside the Frankfurt production environment.
+4a. LOUD VARIANT: a reverse shell reaches the Kafka feeds and the prediction DB, which holds patient IDs and feature vectors for every scored patient. The result is a PHI exfiltration or ransomware event at a medical-device vendor.
+4b. STEALTH VARIANT: the payload monkey-patches predict_proba to subtract 0.08 when region == 'Rural'. Rural FNR (already 37.8%) rises, nothing crashes, and the harm looks like 'model behaviour'.
+IMPACT: a GDPR Art. 33/34 breach plus HIPAA breach notification, MDR vigilance, and the loss of conformity status for the device.</t>
         </is>
       </c>
       <c r="F10" s="26" t="inlineStr">
         <is>
-          <t>[Specific control — name a mechanism, not 'monitor the system']</t>
-        </is>
-      </c>
-      <c r="G10" s="26" t="inlineStr">
-        <is>
-          <t>[H / M-H / M / L-M / L]</t>
-        </is>
-      </c>
-      <c r="H10" s="26" t="inlineStr">
-        <is>
-          <t>[H / M / L]</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="110" customHeight="1">
+          <t>Targets the integrity of the artifacts (ATLAS AML.M0014 Verify AI Artifacts, AML.M0013 Code Signing, AML.M0016 Vulnerability Scanning, AML.M0023 AI Bill of Materials, AML.M0005 Control Access to AI Models and Data at Rest):
+1. SAFE SERIALISATION: replace joblib/pickle with skops.io, loading with an explicit trusted-types allow-list, or export to ONNX and serve with onnxruntime. The deployment then never runs pickle.
+2. SIGN AND VERIFY: the CI pipeline signs each artifact with Sigstore cosign (keyless, OIDC identity of the CI job). Before loading, the Inference API checks the signature and that the sha256 matches the registry entry, and refuses to start otherwise.
+3. SCAN: modelscan / picklescan runs as a CI gate on every artifact.
+4. REGISTRY HARDENING: artifact storage is immutable (S3 Object Lock / WORM). Only the CI service identity can write; humans need MFA plus a two-person approval to promote a model.
+5. ML-BOM: a CycloneDX ML-BOM for each release, pinning scikit-learn 1.7 and the numpy versions.</t>
+        </is>
+      </c>
+      <c r="G10" s="47" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H10" s="47" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="321" customHeight="1">
       <c r="A11" s="11" t="inlineStr">
         <is>
           <t>3</t>
@@ -2222,37 +2409,46 @@
       </c>
       <c r="B11" s="26" t="inlineStr">
         <is>
-          <t>[AML.T####]</t>
+          <t>AML.T0024</t>
         </is>
       </c>
       <c r="C11" s="26" t="inlineStr">
         <is>
-          <t>[Technique name]</t>
+          <t>Exfiltration via AI Inference API
+(.000 Infer Training Data Membership; .002 Extract AI Model. Enabled by AML.T0040 AI Model Inference API Access)</t>
         </is>
       </c>
       <c r="D11" s="26" t="inlineStr">
         <is>
-          <t>[Specific Component (1-6)]</t>
+          <t>C3 Model Inference API (and the hospital-edge mTLS client certificates in C1/C3).</t>
         </is>
       </c>
       <c r="E11" s="26" t="inlineStr">
         <is>
-          <t>[Concrete attack scenario in the healthcare context]</t>
+          <t>ACTOR: someone with access to a hospital integration server (a contractor, or a compromised host holding the mTLS client certificate). Or a commercial party who wants a HealthGuard equivalent for INSURANCE UNDERWRITING, which is an explicitly prohibited use.
+1. The attacker uses the hospital's certificate to call C3 directly. C3 accepts arbitrary feature vectors and returns a full-precision probability.
+2. EXTRACTION (.002): they submit about 250k synthetic vectors spread across the 13-feature space, staying under 200 req/min (about 1 day of traffic), and train a surrogate GBM that agrees with HealthGuard more than 95% of the time. The surrogate is then used for premium pricing outside any clinician oversight. That is exactly the prohibited use, and it sits beyond Klariova's contractual controls.
+3. MEMBERSHIP (.000): for a known Irish or German patient (an employee or a public figure), they query their real attributes and compare the confidence with near-neighbour perturbations. Unusually high confidence suggests the record was in Source 1 training, revealing that the person was a patient at a specific hospital and probably their diabetes outcome.
+IMPACT: disclosure of special-category data (GDPR Art. 9, breach under Art. 33), loss of IP, and enabling of a prohibited use.</t>
         </is>
       </c>
       <c r="F11" s="26" t="inlineStr">
         <is>
-          <t>[Specific control — name a mechanism, not 'monitor the system']</t>
-        </is>
-      </c>
-      <c r="G11" s="26" t="inlineStr">
-        <is>
-          <t>[H / M-H / M / L-M / L]</t>
-        </is>
-      </c>
-      <c r="H11" s="26" t="inlineStr">
-        <is>
-          <t>[H / M / L]</t>
+          <t>Targets exposure of the API (ATLAS AML.M0004 Restrict Number of AI Model Queries, AML.M0002 Passive AI Output Obfuscation, AML.M0019 Control Access to AI Models and Data in Production):
+1. REFERENCE-ONLY INPUT: change C3 so it accepts a patient reference plus a clinician OAuth2 token, not a raw feature vector. The server builds features from the ingested FHIR data. Attackers can no longer choose query points, which defeats both extraction and membership probing.
+2. OUTPUT COARSENING: return a risk band (low / moderate / high) and the top-3 SHAP factors, not a 4-decimal probability.
+3. PER-IDENTITY QUOTAS: per-clinician limits sized to clinical reality (e.g., 60 scores per hour) instead of 200 rpm per hospital. Use Upstash rate limiting keyed on clinician ID, and alert on unusual coverage of the feature space.
+4. PRIVACY RELEASE GATE: run an ML Privacy Meter membership-inference audit on each release, with a maximum attack AUC of 0.55, before promotion.</t>
+        </is>
+      </c>
+      <c r="G11" s="47" t="inlineStr">
+        <is>
+          <t>L-M</t>
+        </is>
+      </c>
+      <c r="H11" s="47" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -2263,19 +2459,24 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="130" customHeight="1">
+    <row r="14" ht="205" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>[Why these 3 TTPs in this order? Explain the reasoning given the healthcare deployment context, the existing architecture, and the data quality concerns surfaced in D2.]</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="n"/>
-      <c r="C14" s="5" t="n"/>
-      <c r="D14" s="5" t="n"/>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="5" t="n"/>
-      <c r="G14" s="5" t="n"/>
-      <c r="H14" s="6" t="n"/>
+          <t>I ranked the three by likelihood × patient-safety impact in THIS deployment. Each one exploits a weakness already found in D1/D2, not a generic ML threat.
+1) AML.T0020 Poison Training Data is first because the attack path is built into the design. Clinician overrides go straight from C4 into the C5 registry for retraining, with no review (D1 Art. 14/15 rows; D2 stage 7 and risk C1). The precondition, a clinician login, is the most commonly compromised credential in healthcare. And the outcome needs no attacker at all: biased overrides on under-served patients cause the same harm. It also targets the system's weakest point. D4 already shows FNR of 37.8% for Rural and 37.5% for Uninsured patients, and the labels already carry historical under-diagnosis that the synthetic Source 2 copies (D2 data-quality concerns). Poisoning makes an existing fairness failure worse, invisibly to aggregate AUC, so it hits the Board's low patient-safety appetite directly.
+2) AML.T0010.003 AI Supply Chain Compromise: Model is second. Its impact is the highest of the three (code execution inside the PHI environment, or stealthy per-subgroup sabotage), and the weakness is concrete: an unsigned joblib pickle loaded by C3. Likelihood is lower (M) because it needs privileged registry or CI access, not a clinician login. It is also the most clear-cut to fix: safe serialisation plus signature verification removes the whole class before launch.
+3) AML.T0024 Exfiltration via Inference API is third. C3's design (raw vectors in, raw probabilities out, 200 req/min per hospital) makes it feasible, and it is the AI-specific route to the privacy and prohibited-use risks in D2 (health-data disclosure; insurance underwriting). Likelihood is L-M: the API is not internet-facing, it sits behind hospital mTLS, and membership inference against a regularised GBM on about 12k records gives only modest advantage. Impact is M rather than H because it causes privacy and IP harm, not direct clinical harm.
+Considered and deprioritised: AML.T0015 Evade AI Model / AML.T0043 Craft Adversarial Data. Patients and clinicians have no plausible motive to make a preventive screening score lower, and the realistic 'adversarial input', stale insurance_type from billing, is a data-quality problem already handled under D2 stage 3 and Art. 15 robustness. Prompt-injection and LLM techniques do not apply: there is no generative component.
+Carry to D5: one risk row per TTP (Security; NIST AI RMF Manage). #1 also links to the subgroup-FNR KRI in D7.</t>
+        </is>
+      </c>
+      <c r="B14" s="45" t="n"/>
+      <c r="C14" s="45" t="n"/>
+      <c r="D14" s="45" t="n"/>
+      <c r="E14" s="45" t="n"/>
+      <c r="F14" s="45" t="n"/>
+      <c r="G14" s="45" t="n"/>
+      <c r="H14" s="46" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>

<commit_message>
Implement HealthGuard lab modules and run D4 technical audit
- lab/: fairness metrics, subgroup/intersectional audit, proxy-pathway
  test, SHAP explainer + proxy detection, and the three KRIs (34/34 tests)
- Pin numpy 2.0.2 and scikit-learn 1.7.2 so the shipped model artifact
  loads without unpickling errors or version warnings
- Notebook: write D4 B40/B41 and keep zero-valued KRI metrics in D7
- Executed notebook populates D4 and D7; add proxy-bias narrative to D4

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/04-secure-ai-deployment/project/starter/governance_portfolio.xlsx
+++ b/04-secure-ai-deployment/project/starter/governance_portfolio.xlsx
@@ -2237,13 +2237,13 @@
 → Where the surface is largest: the C4→C5 feedback loop (untrusted labels flow straight into training), the C5→C3 artifact path (unsigned pickle is loaded in production), and C3 API exposure (raw vectors in, raw probabilities out). The three TTPs below are chosen from these.</t>
         </is>
       </c>
-      <c r="B5" s="45" t="n"/>
-      <c r="C5" s="45" t="n"/>
-      <c r="D5" s="45" t="n"/>
-      <c r="E5" s="45" t="n"/>
-      <c r="F5" s="45" t="n"/>
-      <c r="G5" s="45" t="n"/>
-      <c r="H5" s="46" t="n"/>
+      <c r="B5" s="5" t="n"/>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="5" t="n"/>
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="5" t="n"/>
+      <c r="G5" s="5" t="n"/>
+      <c r="H5" s="6" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
@@ -2470,13 +2470,13 @@
 Carry to D5: one risk row per TTP (Security; NIST AI RMF Manage). #1 also links to the subgroup-FNR KRI in D7.</t>
         </is>
       </c>
-      <c r="B14" s="45" t="n"/>
-      <c r="C14" s="45" t="n"/>
-      <c r="D14" s="45" t="n"/>
-      <c r="E14" s="45" t="n"/>
-      <c r="F14" s="45" t="n"/>
-      <c r="G14" s="45" t="n"/>
-      <c r="H14" s="46" t="n"/>
+      <c r="B14" s="5" t="n"/>
+      <c r="C14" s="5" t="n"/>
+      <c r="D14" s="5" t="n"/>
+      <c r="E14" s="5" t="n"/>
+      <c r="F14" s="5" t="n"/>
+      <c r="G14" s="5" t="n"/>
+      <c r="H14" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -2498,7 +2498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F58"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -2557,7 +2557,9 @@
           <t>ROC AUC</t>
         </is>
       </c>
-      <c r="B6" s="11" t="n"/>
+      <c r="B6" s="11" t="n">
+        <v>0.8120000000000001</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
@@ -2565,7 +2567,9 @@
           <t>Recall (sensitivity)</t>
         </is>
       </c>
-      <c r="B7" s="11" t="n"/>
+      <c r="B7" s="11" t="n">
+        <v>0.744</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
@@ -2573,7 +2577,9 @@
           <t>Precision</t>
         </is>
       </c>
-      <c r="B8" s="11" t="n"/>
+      <c r="B8" s="11" t="n">
+        <v>0.476</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
@@ -2581,7 +2587,9 @@
           <t>F1</t>
         </is>
       </c>
-      <c r="B9" s="11" t="n"/>
+      <c r="B9" s="11" t="n">
+        <v>0.581</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
@@ -2589,7 +2597,9 @@
           <t>Accuracy</t>
         </is>
       </c>
-      <c r="B10" s="11" t="n"/>
+      <c r="B10" s="11" t="n">
+        <v>0.731</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
@@ -2597,7 +2607,9 @@
           <t>Decision threshold</t>
         </is>
       </c>
-      <c r="B11" s="11" t="n"/>
+      <c r="B11" s="11" t="n">
+        <v>0.26</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
@@ -2605,7 +2617,9 @@
           <t>Test n</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n"/>
+      <c r="B12" s="11" t="n">
+        <v>3000</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
@@ -2613,7 +2627,9 @@
           <t>Prevalence</t>
         </is>
       </c>
-      <c r="B13" s="11" t="n"/>
+      <c r="B13" s="11" t="n">
+        <v>0.25</v>
+      </c>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
@@ -2655,28 +2671,70 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="n"/>
-      <c r="B18" s="11" t="n"/>
-      <c r="C18" s="11" t="n"/>
-      <c r="D18" s="11" t="n"/>
-      <c r="E18" s="11" t="n"/>
-      <c r="F18" s="11" t="n"/>
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="n">
+        <v>633</v>
+      </c>
+      <c r="C18" s="11" t="n">
+        <v>111</v>
+      </c>
+      <c r="D18" s="11" t="n">
+        <v>0.378</v>
+      </c>
+      <c r="E18" s="11" t="n">
+        <v>0.195</v>
+      </c>
+      <c r="F18" s="11" t="n">
+        <v>0.27</v>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="n"/>
-      <c r="B19" s="11" t="n"/>
-      <c r="C19" s="11" t="n"/>
-      <c r="D19" s="11" t="n"/>
-      <c r="E19" s="11" t="n"/>
-      <c r="F19" s="11" t="n"/>
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>Suburban</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="n">
+        <v>1031</v>
+      </c>
+      <c r="C19" s="11" t="n">
+        <v>273</v>
+      </c>
+      <c r="D19" s="11" t="n">
+        <v>0.245</v>
+      </c>
+      <c r="E19" s="11" t="n">
+        <v>0.309</v>
+      </c>
+      <c r="F19" s="11" t="n">
+        <v>0.427</v>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="n"/>
-      <c r="B20" s="11" t="n"/>
-      <c r="C20" s="11" t="n"/>
-      <c r="D20" s="11" t="n"/>
-      <c r="E20" s="11" t="n"/>
-      <c r="F20" s="11" t="n"/>
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>Urban</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="n">
+        <v>1336</v>
+      </c>
+      <c r="C20" s="11" t="n">
+        <v>366</v>
+      </c>
+      <c r="D20" s="11" t="n">
+        <v>0.227</v>
+      </c>
+      <c r="E20" s="11" t="n">
+        <v>0.287</v>
+      </c>
+      <c r="F20" s="11" t="n">
+        <v>0.42</v>
+      </c>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="8" t="inlineStr">
@@ -2718,68 +2776,196 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="11" t="n"/>
-      <c r="B27" s="11" t="n"/>
-      <c r="C27" s="11" t="n"/>
-      <c r="D27" s="11" t="n"/>
-      <c r="E27" s="11" t="n"/>
-      <c r="F27" s="11" t="n"/>
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>Urban</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="n">
+        <v>819</v>
+      </c>
+      <c r="D27" s="11" t="n">
+        <v>233</v>
+      </c>
+      <c r="E27" s="11" t="n">
+        <v>0.245</v>
+      </c>
+      <c r="F27" s="11" t="n">
+        <v>0.426</v>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="11" t="n"/>
-      <c r="B28" s="11" t="n"/>
-      <c r="C28" s="11" t="n"/>
-      <c r="D28" s="11" t="n"/>
-      <c r="E28" s="11" t="n"/>
-      <c r="F28" s="11" t="n"/>
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>Suburban</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="n">
+        <v>572</v>
+      </c>
+      <c r="D28" s="11" t="n">
+        <v>153</v>
+      </c>
+      <c r="E28" s="11" t="n">
+        <v>0.235</v>
+      </c>
+      <c r="F28" s="11" t="n">
+        <v>0.435</v>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="11" t="n"/>
-      <c r="B29" s="11" t="n"/>
-      <c r="C29" s="11" t="n"/>
-      <c r="D29" s="11" t="n"/>
-      <c r="E29" s="11" t="n"/>
-      <c r="F29" s="11" t="n"/>
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>Urban</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>Medicare</t>
+        </is>
+      </c>
+      <c r="C29" s="11" t="n">
+        <v>252</v>
+      </c>
+      <c r="D29" s="11" t="n">
+        <v>64</v>
+      </c>
+      <c r="E29" s="11" t="n">
+        <v>0.172</v>
+      </c>
+      <c r="F29" s="11" t="n">
+        <v>0.437</v>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="11" t="n"/>
-      <c r="B30" s="11" t="n"/>
-      <c r="C30" s="11" t="n"/>
-      <c r="D30" s="11" t="n"/>
-      <c r="E30" s="11" t="n"/>
-      <c r="F30" s="11" t="n"/>
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="n">
+        <v>195</v>
+      </c>
+      <c r="D30" s="11" t="n">
+        <v>52</v>
+      </c>
+      <c r="E30" s="11" t="n">
+        <v>0.231</v>
+      </c>
+      <c r="F30" s="11" t="n">
+        <v>0.369</v>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="11" t="n"/>
-      <c r="B31" s="11" t="n"/>
-      <c r="C31" s="11" t="n"/>
-      <c r="D31" s="11" t="n"/>
-      <c r="E31" s="11" t="n"/>
-      <c r="F31" s="11" t="n"/>
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>Urban</t>
+        </is>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>Medicaid</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="n">
+        <v>204</v>
+      </c>
+      <c r="D31" s="11" t="n">
+        <v>52</v>
+      </c>
+      <c r="E31" s="11" t="n">
+        <v>0.192</v>
+      </c>
+      <c r="F31" s="11" t="n">
+        <v>0.397</v>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="11" t="n"/>
-      <c r="B32" s="11" t="n"/>
-      <c r="C32" s="11" t="n"/>
-      <c r="D32" s="11" t="n"/>
-      <c r="E32" s="11" t="n"/>
-      <c r="F32" s="11" t="n"/>
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>Suburban</t>
+        </is>
+      </c>
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>Medicare</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="n">
+        <v>196</v>
+      </c>
+      <c r="D32" s="11" t="n">
+        <v>50</v>
+      </c>
+      <c r="E32" s="11" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="F32" s="11" t="n">
+        <v>0.464</v>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="11" t="n"/>
-      <c r="B33" s="11" t="n"/>
-      <c r="C33" s="11" t="n"/>
-      <c r="D33" s="11" t="n"/>
-      <c r="E33" s="11" t="n"/>
-      <c r="F33" s="11" t="n"/>
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>Suburban</t>
+        </is>
+      </c>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>Medicaid</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="n">
+        <v>185</v>
+      </c>
+      <c r="D33" s="11" t="n">
+        <v>49</v>
+      </c>
+      <c r="E33" s="11" t="n">
+        <v>0.245</v>
+      </c>
+      <c r="F33" s="11" t="n">
+        <v>0.416</v>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="11" t="n"/>
-      <c r="B34" s="11" t="n"/>
-      <c r="C34" s="11" t="n"/>
-      <c r="D34" s="11" t="n"/>
-      <c r="E34" s="11" t="n"/>
-      <c r="F34" s="11" t="n"/>
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>Medicaid</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="n">
+        <v>284</v>
+      </c>
+      <c r="D34" s="11" t="n">
+        <v>33</v>
+      </c>
+      <c r="E34" s="11" t="n">
+        <v>0.606</v>
+      </c>
+      <c r="F34" s="11" t="n">
+        <v>0.204</v>
+      </c>
     </row>
     <row r="36" ht="22" customHeight="1">
       <c r="A36" s="8" t="inlineStr">
@@ -2794,7 +2980,11 @@
           <t>Subgroup</t>
         </is>
       </c>
-      <c r="B37" s="11" t="n"/>
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>('Rural', 'Medicaid')</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="33" t="inlineStr">
@@ -2802,7 +2992,9 @@
           <t>Most-harmed metric (FNR)</t>
         </is>
       </c>
-      <c r="B38" s="11" t="n"/>
+      <c r="B38" s="11" t="n">
+        <v>0.606</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="33" t="inlineStr">
@@ -2810,7 +3002,9 @@
           <t>n_positives</t>
         </is>
       </c>
-      <c r="B39" s="11" t="n"/>
+      <c r="B39" s="11" t="n">
+        <v>33</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="33" t="inlineStr">
@@ -2820,7 +3014,7 @@
       </c>
       <c r="B40" s="11" t="inlineStr">
         <is>
-          <t>(Notebook computes)</t>
+          <t>Urban: Medicaid − Private = -5.2 pp</t>
         </is>
       </c>
     </row>
@@ -2832,7 +3026,7 @@
       </c>
       <c r="B41" s="11" t="inlineStr">
         <is>
-          <t>(Notebook computes)</t>
+          <t>+15.2 pp</t>
         </is>
       </c>
     </row>
@@ -2842,7 +3036,11 @@
           <t>Within-region gap (Rural + Medicaid − Rural + Private)</t>
         </is>
       </c>
-      <c r="B42" s="11" t="n"/>
+      <c r="B42" s="11" t="inlineStr">
+        <is>
+          <t>+37.5 pp</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="33" t="inlineStr">
@@ -2850,7 +3048,11 @@
           <t>Verdict</t>
         </is>
       </c>
-      <c r="B43" s="11" t="n"/>
+      <c r="B43" s="11" t="inlineStr">
+        <is>
+          <t>proxy_supported</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="22" customHeight="1">
       <c r="A46" s="8" t="inlineStr">
@@ -2892,68 +3094,196 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="11" t="n"/>
-      <c r="B48" s="11" t="n"/>
-      <c r="C48" s="11" t="n"/>
-      <c r="D48" s="11" t="n"/>
-      <c r="E48" s="11" t="n"/>
-      <c r="F48" s="11" t="n"/>
+      <c r="A48" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B48" s="11" t="inlineStr">
+        <is>
+          <t>num__glucose</t>
+        </is>
+      </c>
+      <c r="C48" s="11" t="n">
+        <v>0.806</v>
+      </c>
+      <c r="D48" s="11" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="E48" s="11" t="n">
+        <v>0.047</v>
+      </c>
+      <c r="F48" s="11" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="11" t="n"/>
-      <c r="B49" s="11" t="n"/>
-      <c r="C49" s="11" t="n"/>
-      <c r="D49" s="11" t="n"/>
-      <c r="E49" s="11" t="n"/>
-      <c r="F49" s="11" t="n"/>
+      <c r="A49" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B49" s="11" t="inlineStr">
+        <is>
+          <t>num__bmi</t>
+        </is>
+      </c>
+      <c r="C49" s="11" t="n">
+        <v>0.294</v>
+      </c>
+      <c r="D49" s="11" t="n">
+        <v>-0.006</v>
+      </c>
+      <c r="E49" s="11" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="F49" s="11" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" s="11" t="n"/>
-      <c r="B50" s="11" t="n"/>
-      <c r="C50" s="11" t="n"/>
-      <c r="D50" s="11" t="n"/>
-      <c r="E50" s="11" t="n"/>
-      <c r="F50" s="11" t="n"/>
+      <c r="A50" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="B50" s="11" t="inlineStr">
+        <is>
+          <t>num__age</t>
+        </is>
+      </c>
+      <c r="C50" s="11" t="n">
+        <v>0.278</v>
+      </c>
+      <c r="D50" s="11" t="n">
+        <v>-0.006</v>
+      </c>
+      <c r="E50" s="11" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="F50" s="11" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="51">
-      <c r="A51" s="11" t="n"/>
-      <c r="B51" s="11" t="n"/>
-      <c r="C51" s="11" t="n"/>
-      <c r="D51" s="11" t="n"/>
-      <c r="E51" s="11" t="n"/>
-      <c r="F51" s="11" t="n"/>
+      <c r="A51" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="B51" s="11" t="inlineStr">
+        <is>
+          <t>num__family_history</t>
+        </is>
+      </c>
+      <c r="C51" s="11" t="n">
+        <v>0.142</v>
+      </c>
+      <c r="D51" s="11" t="n">
+        <v>-0.005</v>
+      </c>
+      <c r="E51" s="11" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="F51" s="11" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" s="11" t="n"/>
-      <c r="B52" s="11" t="n"/>
-      <c r="C52" s="11" t="n"/>
-      <c r="D52" s="11" t="n"/>
-      <c r="E52" s="11" t="n"/>
-      <c r="F52" s="11" t="n"/>
+      <c r="A52" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="B52" s="11" t="inlineStr">
+        <is>
+          <t>num__pedigree</t>
+        </is>
+      </c>
+      <c r="C52" s="11" t="n">
+        <v>0.114</v>
+      </c>
+      <c r="D52" s="11" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="E52" s="11" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="F52" s="11" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" s="11" t="n"/>
-      <c r="B53" s="11" t="n"/>
-      <c r="C53" s="11" t="n"/>
-      <c r="D53" s="11" t="n"/>
-      <c r="E53" s="11" t="n"/>
-      <c r="F53" s="11" t="n"/>
+      <c r="A53" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="B53" s="11" t="inlineStr">
+        <is>
+          <t>num__blood_pressure</t>
+        </is>
+      </c>
+      <c r="C53" s="11" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="D53" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" s="11" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="F53" s="11" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="54">
-      <c r="A54" s="11" t="n"/>
-      <c r="B54" s="11" t="n"/>
-      <c r="C54" s="11" t="n"/>
-      <c r="D54" s="11" t="n"/>
-      <c r="E54" s="11" t="n"/>
-      <c r="F54" s="11" t="n"/>
+      <c r="A54" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="B54" s="11" t="inlineStr">
+        <is>
+          <t>num__pregnancies</t>
+        </is>
+      </c>
+      <c r="C54" s="11" t="n">
+        <v>0.096</v>
+      </c>
+      <c r="D54" s="11" t="n">
+        <v>-0.001</v>
+      </c>
+      <c r="E54" s="11" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="F54" s="11" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="55">
-      <c r="A55" s="11" t="n"/>
-      <c r="B55" s="11" t="n"/>
-      <c r="C55" s="11" t="n"/>
-      <c r="D55" s="11" t="n"/>
-      <c r="E55" s="11" t="n"/>
-      <c r="F55" s="11" t="n"/>
+      <c r="A55" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="B55" s="11" t="inlineStr">
+        <is>
+          <t>cat__insurance_type_Medicaid</t>
+        </is>
+      </c>
+      <c r="C55" s="11" t="n">
+        <v>0.076</v>
+      </c>
+      <c r="D55" s="11" t="n">
+        <v>-0.002</v>
+      </c>
+      <c r="E55" s="11" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="F55" s="11" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="22" customHeight="1">
       <c r="A57" s="8" t="inlineStr">
@@ -2962,10 +3292,15 @@
         </is>
       </c>
     </row>
-    <row r="58" ht="180" customHeight="1">
+    <row r="58" ht="310" customHeight="1">
       <c r="A58" s="11" t="inlineStr">
         <is>
-          <t>[Populated by audit_notebook.ipynb after the technical audit runs.]</t>
+          <t>HYPOTHESIS. HealthGuard's Rural FNR disparity is not a 'Rural' effect. It runs through insurance_type and region acting as proxies for historical under-diagnosis. In the training labels, poorer rural patients (Medicaid / Uninsured) were diagnosed at about half the true rate. The model learned that being 'Rural + Medicaid/Uninsured' means low risk, and now repeats the access gap at the point of care.
+EVIDENCE (test n=3,000, threshold 0.26):
+1) Disparity is concentrated in one cell. Rural FNR is 37.8% vs 22.7% for Urban (+15.2 pp region gap). Within Rural, Medicaid FNR is 60.6% (n_pos=33, Wilson 95% CI about 44-75%) vs 23.1% for Rural × Private (n_pos=52, CI about 14-36%), a +37.5 pp gap. In the Urban reference the same comparison is -5.2 pp (Medicaid 19.2% vs Private 24.5%). Insurance matters only inside Rural, and Rural × Private performs like Urban. Verdict from assess_proxy_pathway: proxy_supported (+42.8 pp excess over the reference, margin 5 pp). This is the most-harmed cell at n_pos &gt;= 20. KRI-1 = Red (43.4 pp gap, Rural × Medicaid vs Urban × Medicare).
+2) The training labels carry the bias. Recorded diabetes prevalence in train is 13.5% for Rural × Medicaid and 12.7% for Rural × Uninsured, against 26-29% in every other cell, including Urban × Medicaid at 26.1%. In train, Rural is 45% Medicaid. This matches brief §8: under-served patients get fewer encounters, so fewer diagnoses, and the Source 2 synthetic generator copied the pattern.
+3) The missed patients are clinically comparable. True positives in Rural × Medicaid have mean glucose 129, BMI 31.2 and age 54, compared with 133 / 30.2 / 54 for Rural × Private, and a higher family-history rate (0.39 vs 0.29). Milder disease does not explain the misses.
+4) SHAP shows the mechanism locally. On false negatives in Rural × (Medicaid|Uninsured), region + insurance_type contribute -0.63 log-odds on average, against +0.07 on FNs in all other cells. Across all patients the same features give -0.59 to Rural × Medicaid/Uninsured and +0.15 to Urban × Private, a 0.74 log-odds swing from non-clinical features alone. The notebook's local examples show cat__region_Rural (about -0.27) and cat__insurance_type_Medicaid/Uninsured (-0.23 / -0.34) among the top-3 negative drivers. Removing only the region + insurance attributions would lift 8 of 25 (32%) of these FNs above the threshold, against 3 of 167 (2%) elsewhere.</t>
         </is>
       </c>
       <c r="B58" s="5" t="n"/>
@@ -2974,8 +3309,23 @@
       <c r="E58" s="5" t="n"/>
       <c r="F58" s="6" t="n"/>
     </row>
+    <row r="59" ht="310" customHeight="1">
+      <c r="A59" s="11" t="inlineStr">
+        <is>
+          <t>WHY THE GLOBAL SHAP TABLE SAYS 'no'. detect_proxy_features ranks insurance_type_Medicaid 8th (mean |SHAP| 0.076) but finds signed_strength of only about 0.03. So the notebook's is_likely_proxy rule (mean_shap &lt; -0.01 AND strength &gt;= 0.5) flags nothing. The proxy effect points in opposite directions in different cells (negative for Rural/Medicaid, positive for Urban/Private) and lands on about 12% of patients, so it averages out in a population-level summary. Lesson for D6/D8: a global-SHAP proxy screen is necessary but NOT sufficient. Proxy detection must be subgroup-conditional, meaning SHAP averaged within each intersectional cell.
+VERDICT: proxy-bias pathway SUPPORTED. insurance_type (with region) acts as a proxy for under-diagnosis in the labels, not for diabetes risk. The harm is about 2.6x the missed-diagnosis rate (60.6% vs 23.1%) for an identifiable, disadvantaged group. That breaches the Board's low patient-safety appetite (D1 gap #1; D5 Fairness risk; D7 KRI-1 Red).
+LIMITATIONS. (a) The test labels carry the same under-diagnosis: Rural × Medicaid prevalence is 11.6% vs about 26% elsewhere. Undiagnosed diabetics in this cell are labelled 0 and cannot count as misses, so the measured 60.6% FNR is probably an UNDER-estimate. (b) Rural × Uninsured (FNR 50%, n_pos=10) and Rural × Medicare (n_pos=16) fall below the n_pos &gt;= 20 power filter and cannot be quantified (residual risk for D5). (c) SHAP attributions are not counterfactuals. The 32% 'would-flip' figure is an attribution heuristic, not a causal estimate. (d) Synthetic, single-split data from IE/DE only. Not validated for the US population.
+WHAT WOULD CONFIRM OR REFUTE IT (pre-launch actions): (1) Ablation: retrain without region and insurance_type, then re-run this audit. Expect the Rural × Medicaid FNR gap to shrink but not close, because the label bias remains. (2) Label audit: re-adjudicate a sample of Rural × Medicaid negatives against HbA1c/fasting-glucose criteria to estimate the hidden positives. (3) Mitigate through relabelling / reweighting plus group-aware threshold review, then re-test against KRI-1 (Green &lt;= 8 pp). (4) Add subgroup-conditional SHAP to the CI release gate.</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="n"/>
+      <c r="C59" s="5" t="n"/>
+      <c r="D59" s="5" t="n"/>
+      <c r="E59" s="5" t="n"/>
+      <c r="F59" s="6" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="A46:F46"/>
@@ -2983,6 +3333,7 @@
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A58:F58"/>
     <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A59:F59"/>
     <mergeCell ref="A25:F25"/>
     <mergeCell ref="A57:F57"/>
   </mergeCells>
@@ -4497,25 +4848,79 @@
       <c r="I10" s="41" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="n"/>
-      <c r="B11" s="11" t="n"/>
-      <c r="C11" s="11" t="n"/>
-      <c r="D11" s="11" t="n"/>
-      <c r="E11" s="11" t="n"/>
+      <c r="A11" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>KRI-1</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>43.4</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>FNR gap 43.4 pp: worst Rural × Medicaid 60.6% vs best Urban × Medicare 17.2% across 9 cells with &gt;= 20 positives (Green &lt;= 8, Amber &lt;= 15, Red &gt; 15).</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="n"/>
-      <c r="B12" s="11" t="n"/>
-      <c r="C12" s="11" t="n"/>
-      <c r="D12" s="11" t="n"/>
-      <c r="E12" s="11" t="n"/>
+      <c r="A12" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>KRI-2</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>0.06</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>override rate 6.0% &lt;= 10% and structured share 85.0% &gt;= 80%</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="n"/>
-      <c r="B13" s="11" t="n"/>
-      <c r="C13" s="11" t="n"/>
-      <c r="D13" s="11" t="n"/>
-      <c r="E13" s="11" t="n"/>
+      <c r="A13" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>KRI-3</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>0 anomalous of 2,000 inferences = 0.00 per 1,000 (Green &lt; 1, Amber 1-5, Red &gt; 5).</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Complete HealthGuard D5 risk register and D6 model card
- D5: 12-risk NIST AI RMF register drawn from D1-D4 with L x I scores,
  named controls, residual risk and five Top-N enterprise risks
- D6: model details, use limits, training-data provenance and quality
  findings, explainability limitations, ATLAS threats, regulatory and
  KRI monitoring context
- Notebook now writes D6 sec. 4 performance and sec. 5 SHAP findings from
  the audit; re-executed

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/04-secure-ai-deployment/project/starter/governance_portfolio.xlsx
+++ b/04-secure-ai-deployment/project/starter/governance_portfolio.xlsx
@@ -223,7 +223,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="2"/>
@@ -332,6 +332,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3351,17 +3354,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="38" customWidth="1" min="9" max="9"/>
+    <col width="62" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="48" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -3514,7 +3517,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="36" customHeight="1">
+    <row r="7" ht="126" customHeight="1">
       <c r="A7" s="11" t="inlineStr">
         <is>
           <t>RR-01</t>
@@ -3522,60 +3525,54 @@
       </c>
       <c r="B7" s="26" t="inlineStr">
         <is>
-          <t>[Risk description — be specific]</t>
+          <t>SUBGROUP UNDER-DETECTION (proxy bias). Rural × Medicaid patients have FNR 60.6% (n_pos=33, 95% CI about 44-75%) vs 23.1% for Rural × Private. KRI-1 is Red at a 43.4 pp gap. region and insurance_type act as proxies for historical under-diagnosis in the training labels, so true diabetics in a disadvantaged group are missed and their referral is delayed.</t>
         </is>
       </c>
       <c r="C7" s="26" t="inlineStr">
         <is>
-          <t>[Regulatory / Security / Fairness / Privacy / Operational]</t>
+          <t>Fairness</t>
         </is>
       </c>
       <c r="D7" s="26" t="inlineStr">
         <is>
-          <t>[Govern / Map / Measure / Manage]</t>
-        </is>
-      </c>
-      <c r="E7" s="26" t="inlineStr">
-        <is>
-          <t>[D1 / D2 / D3 / D4]</t>
-        </is>
-      </c>
-      <c r="F7" s="26" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
-      </c>
-      <c r="G7" s="26" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
-      </c>
-      <c r="H7" s="11">
+          <t>Measure</t>
+        </is>
+      </c>
+      <c r="E7" s="47" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
+      <c r="F7" s="47" t="n">
+        <v>5</v>
+      </c>
+      <c r="G7" s="47" t="n">
+        <v>5</v>
+      </c>
+      <c r="H7" s="48">
         <f>IFERROR(F7*G7,"")</f>
         <v/>
       </c>
       <c r="I7" s="26" t="inlineStr">
         <is>
-          <t>[Specific control — name a framework, library entry, or mechanism]</t>
-        </is>
-      </c>
-      <c r="J7" s="26" t="inlineStr">
-        <is>
-          <t>[Low / Low-Medium / Medium / Medium-High / High]</t>
-        </is>
-      </c>
-      <c r="K7" s="26" t="inlineStr">
-        <is>
-          <t>[TRUE / FALSE]</t>
-        </is>
+          <t>1) Ablation retrain without region and insurance_type, then re-run the D4 audit. 2) Label audit: re-adjudicate a sample of Rural × Medicaid negatives against HbA1c / fasting-glucose criteria, then relabel or reweight. 3) Mitigate with fairlearn (ExponentiatedGradient with an EqualizedOdds constraint), plus a clinical review of any group-specific thresholds. 4) Release gate: KRI-1 Green (&lt;= 8 pp), and no subgroup FNR worse than a FINDRISC standard-of-care baseline, confirmed by independent external validation.</t>
+        </is>
+      </c>
+      <c r="J7" s="47" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K7" s="47" t="b">
+        <v>1</v>
       </c>
       <c r="L7" s="26" t="inlineStr">
         <is>
-          <t>[Optional notes / justification for high scores]</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="36" customHeight="1">
+          <t>NIST MEASURE 2.11 (fairness and bias evaluated). Breaches the Board's LOW patient-safety appetite. D1 launch-blocking gap #1 (Art. 10 + 15). L5: the risk is already present in the shipped model. I5: missed diagnoses for an identifiable group. Residual stays Medium because label bias can only be reduced, not removed, until real-world rural data is collected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="111" customHeight="1">
       <c r="A8" s="11" t="inlineStr">
         <is>
           <t>RR-02</t>
@@ -3583,60 +3580,54 @@
       </c>
       <c r="B8" s="26" t="inlineStr">
         <is>
-          <t>[Risk description — be specific]</t>
+          <t>NO LAWFUL ROUTE TO EU MARKET. HealthGuard is high-risk under Art. 6(1) + Annex I (MDR Class IIa, Rule 11), but it is positioned as 'not a medical device'. There is no QMS (Art. 17), no Annex IV technical file (Art. 11), no documented RMS (Art. 9), and no notified-body conformity assessment, DoC, CE marking or EU database registration (Arts 43, 47-49). Q3 2027 launch falls after the 2 Aug 2027 application date.</t>
         </is>
       </c>
       <c r="C8" s="26" t="inlineStr">
         <is>
-          <t>[Regulatory / Security / Fairness / Privacy / Operational]</t>
+          <t>Regulatory</t>
         </is>
       </c>
       <c r="D8" s="26" t="inlineStr">
         <is>
-          <t>[Govern / Map / Measure / Manage]</t>
-        </is>
-      </c>
-      <c r="E8" s="26" t="inlineStr">
-        <is>
-          <t>[D1 / D2 / D3 / D4]</t>
-        </is>
-      </c>
-      <c r="F8" s="26" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
-      </c>
-      <c r="G8" s="26" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
-      </c>
-      <c r="H8" s="11">
+          <t>Govern</t>
+        </is>
+      </c>
+      <c r="E8" s="47" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="F8" s="47" t="n">
+        <v>5</v>
+      </c>
+      <c r="G8" s="47" t="n">
+        <v>4</v>
+      </c>
+      <c r="H8" s="48">
         <f>IFERROR(F8*G8,"")</f>
         <v/>
       </c>
       <c r="I8" s="26" t="inlineStr">
         <is>
-          <t>[Specific control — name a framework, library entry, or mechanism]</t>
-        </is>
-      </c>
-      <c r="J8" s="26" t="inlineStr">
-        <is>
-          <t>[Low / Low-Medium / Medium / Medium-High / High]</t>
-        </is>
-      </c>
-      <c r="K8" s="26" t="inlineStr">
-        <is>
-          <t>[TRUE / FALSE]</t>
-        </is>
+          <t>1) A formal MDR qualification and classification opinion (MDCG 2019-11), with a notified body engaged now. 2) Build the QMS to ISO 13485, with AI-specific controls under ISO/IEC 42001. 3) Compile the Annex IV / MDR technical file, versioned against the Model Registry hash. 4) RMS to ISO 14971 + ISO/IEC 23894, with this register as its living output. 5) Conformity assessment → DoC → CE marking → registration before the first EU patient is scored.</t>
+        </is>
+      </c>
+      <c r="J8" s="47" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="K8" s="47" t="b">
+        <v>1</v>
       </c>
       <c r="L8" s="26" t="inlineStr">
         <is>
-          <t>[Optional notes / justification for high scores]</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="36" customHeight="1">
+          <t>NIST GOVERN 1.1 (legal and regulatory requirements understood, managed and documented). Breaches the Board's LOW appetite for regulatory non-compliance. No compensating control can stand in for a missing conformity assessment, so this is a hard launch gate. Fines up to €15M / 3% of turnover (AI Act Art. 99(4)) plus MDR market withdrawal. D1 gap #2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="126" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
         <is>
           <t>RR-03</t>
@@ -3644,60 +3635,54 @@
       </c>
       <c r="B9" s="26" t="inlineStr">
         <is>
-          <t>[Risk description — be specific]</t>
+          <t>NON-REPRESENTATIVE AND LOW-QUALITY TRAINING DATA (Art. 10). Training data comes only from IE+DE, but the system also deploys to US sites (CA/MA/TX). The synthetic Source 2 copies Source 1's under-diagnosis. insurance_type comes from billing and can be stale. OneHotEncoder(handle_unknown='ignore') silently zeroes unseen categories, such as US insurance codes. The training manifest says about 8k records but train.csv has 12k. There is no external validation.</t>
         </is>
       </c>
       <c r="C9" s="26" t="inlineStr">
         <is>
-          <t>[Regulatory / Security / Fairness / Privacy / Operational]</t>
+          <t>Regulatory</t>
         </is>
       </c>
       <c r="D9" s="26" t="inlineStr">
         <is>
-          <t>[Govern / Map / Measure / Manage]</t>
-        </is>
-      </c>
-      <c r="E9" s="26" t="inlineStr">
-        <is>
-          <t>[D1 / D2 / D3 / D4]</t>
-        </is>
-      </c>
-      <c r="F9" s="26" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
-      </c>
-      <c r="G9" s="26" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
-      </c>
-      <c r="H9" s="11">
+          <t>Map</t>
+        </is>
+      </c>
+      <c r="E9" s="47" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="F9" s="47" t="n">
+        <v>4</v>
+      </c>
+      <c r="G9" s="47" t="n">
+        <v>4</v>
+      </c>
+      <c r="H9" s="48">
         <f>IFERROR(F9*G9,"")</f>
         <v/>
       </c>
       <c r="I9" s="26" t="inlineStr">
         <is>
-          <t>[Specific control — name a framework, library entry, or mechanism]</t>
-        </is>
-      </c>
-      <c r="J9" s="26" t="inlineStr">
-        <is>
-          <t>[Low / Low-Medium / Medium / Medium-High / High]</t>
-        </is>
-      </c>
-      <c r="K9" s="26" t="inlineStr">
-        <is>
-          <t>[TRUE / FALSE]</t>
-        </is>
+          <t>1) Write an Art. 10(2) data-governance record and a Datasheet for each source. 2) Reconcile the manifest sha256 with the actual dataset, and track lineage in DVC or lakeFS. 3) Validate the input schema at the Inference API, rejecting or flagging unknown categories and stale insurance_type (compare against the billing-change date). 4) Gate the US launch on validation with a US-representative cohort. 5) Source real-world rural and under-served records to replace synthetic Source 2.</t>
+        </is>
+      </c>
+      <c r="J9" s="47" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K9" s="47" t="b">
+        <v>0</v>
       </c>
       <c r="L9" s="26" t="inlineStr">
         <is>
-          <t>[Optional notes / justification for high scores]</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="36" customHeight="1">
+          <t>NIST MAP 2.3 (data selection, provenance and TEVV considerations identified). The root cause behind RR-01 and RR-12. Not separately flagged as Top-N because it is escalated through RR-01.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="111" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
           <t>RR-04</t>
@@ -3705,60 +3690,54 @@
       </c>
       <c r="B10" s="26" t="inlineStr">
         <is>
-          <t>[Risk description — be specific]</t>
+          <t>TRANSPARENCY AND HUMAN OVERSIGHT DO NOT WORK (Arts 13-14). Clinicians get no IFU, no subgroup performance figures and only a 'rough explanation'. They have no training and no automation-bias safeguards, so a reassuring 'not high-risk' result is unlikely to be questioned, exactly where FNR is highest. There is no tested kill-switch or rollback.</t>
         </is>
       </c>
       <c r="C10" s="26" t="inlineStr">
         <is>
-          <t>[Regulatory / Security / Fairness / Privacy / Operational]</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="D10" s="26" t="inlineStr">
         <is>
-          <t>[Govern / Map / Measure / Manage]</t>
-        </is>
-      </c>
-      <c r="E10" s="26" t="inlineStr">
-        <is>
-          <t>[D1 / D2 / D3 / D4]</t>
-        </is>
-      </c>
-      <c r="F10" s="26" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
-      </c>
-      <c r="G10" s="26" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
-      </c>
-      <c r="H10" s="11">
+          <t>Manage</t>
+        </is>
+      </c>
+      <c r="E10" s="47" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="F10" s="47" t="n">
+        <v>4</v>
+      </c>
+      <c r="G10" s="47" t="n">
+        <v>4</v>
+      </c>
+      <c r="H10" s="48">
         <f>IFERROR(F10*G10,"")</f>
         <v/>
       </c>
       <c r="I10" s="26" t="inlineStr">
         <is>
-          <t>[Specific control — name a framework, library entry, or mechanism]</t>
-        </is>
-      </c>
-      <c r="J10" s="26" t="inlineStr">
-        <is>
-          <t>[Low / Low-Medium / Medium / Medium-High / High]</t>
-        </is>
-      </c>
-      <c r="K10" s="26" t="inlineStr">
-        <is>
-          <t>[TRUE / FALSE]</t>
-        </is>
+          <t>1) Publish an IFU and a clinician-facing model card (D6) disclosing subgroup FNR and limitations. 2) Validated per-patient SHAP top-3 factors in the dashboard, plus a caution banner for subgroups with high FNR. 3) Mandatory clinician training with competency sign-off. 4) KRI-2 Override Channel Health, broken down by subgroup. 5) A per-tenant kill-switch with rollback to the previous model, tested in a drill and documented in the SRE runbook.</t>
+        </is>
+      </c>
+      <c r="J10" s="47" t="inlineStr">
+        <is>
+          <t>Low-Medium</t>
+        </is>
+      </c>
+      <c r="K10" s="47" t="b">
+        <v>1</v>
       </c>
       <c r="L10" s="26" t="inlineStr">
         <is>
-          <t>[Optional notes / justification for high scores]</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="36" customHeight="1">
+          <t>NIST MANAGE 2.4 (mechanisms to supersede, disengage or deactivate) and GOVERN 3.2 (human-AI oversight roles). Top-N because clinician review is the compensating control the Board would rely on to accept the residual risk in RR-01. Without it, the 'documented partial compliance' route is closed. D1 gap #3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="111" customHeight="1">
       <c r="A11" s="11" t="inlineStr">
         <is>
           <t>RR-05</t>
@@ -3766,60 +3745,54 @@
       </c>
       <c r="B11" s="26" t="inlineStr">
         <is>
-          <t>[Risk description — be specific]</t>
+          <t>TRAINING-DATA POISONING THROUGH THE OVERRIDE FEEDBACK LOOP (ATLAS AML.T0020). Clinician overrides are written to the Model Registry and used for retraining with no review. A phished clinician account, or just systematically biased overrides, can teach the next model that an under-served subgroup is low-risk. That would push its FNR above the current 60.6%, while overall AUC moves by less than 0.01.</t>
         </is>
       </c>
       <c r="C11" s="26" t="inlineStr">
         <is>
-          <t>[Regulatory / Security / Fairness / Privacy / Operational]</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="D11" s="26" t="inlineStr">
         <is>
-          <t>[Govern / Map / Measure / Manage]</t>
-        </is>
-      </c>
-      <c r="E11" s="26" t="inlineStr">
-        <is>
-          <t>[D1 / D2 / D3 / D4]</t>
-        </is>
-      </c>
-      <c r="F11" s="26" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
-      </c>
-      <c r="G11" s="26" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
-      </c>
-      <c r="H11" s="11">
+          <t>Manage</t>
+        </is>
+      </c>
+      <c r="E11" s="47" t="inlineStr">
+        <is>
+          <t>D3</t>
+        </is>
+      </c>
+      <c r="F11" s="47" t="n">
+        <v>4</v>
+      </c>
+      <c r="G11" s="47" t="n">
+        <v>4</v>
+      </c>
+      <c r="H11" s="48">
         <f>IFERROR(F11*G11,"")</f>
         <v/>
       </c>
       <c r="I11" s="26" t="inlineStr">
         <is>
-          <t>[Specific control — name a framework, library entry, or mechanism]</t>
-        </is>
-      </c>
-      <c r="J11" s="26" t="inlineStr">
-        <is>
-          <t>[Low / Low-Medium / Medium / Medium-High / High]</t>
-        </is>
-      </c>
-      <c r="K11" s="26" t="inlineStr">
-        <is>
-          <t>[TRUE / FALSE]</t>
-        </is>
+          <t>1) Quarantine override data, with second-clinician adjudication of a stratified sample before any use in training (ATLAS AML.M0007). 2) Cap label contributions per clinician and per site, plus cleanlab label-issue screening. 3) CI release gate on a frozen, clinician-adjudicated golden set: block if any subgroup's FNR rises by more than 2 pp (AML.M0008). 4) Signed dataset manifests and lineage in DVC/lakeFS (AML.M0025).</t>
+        </is>
+      </c>
+      <c r="J11" s="47" t="inlineStr">
+        <is>
+          <t>Low-Medium</t>
+        </is>
+      </c>
+      <c r="K11" s="47" t="b">
+        <v>1</v>
       </c>
       <c r="L11" s="26" t="inlineStr">
         <is>
-          <t>[Optional notes / justification for high scores]</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="36" customHeight="1">
+          <t>NIST MEASURE 2.7 / MANAGE 2.2. Top-N because it directly amplifies RR-01 and nothing alerts on it. The precondition (clinician credentials) is the most commonly compromised credential in healthcare. D3 rank 1 (likelihood M-H, impact H).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="111" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
           <t>RR-06</t>
@@ -3827,60 +3800,54 @@
       </c>
       <c r="B12" s="26" t="inlineStr">
         <is>
-          <t>[Risk description — be specific]</t>
+          <t>MODEL ARTIFACT SUPPLY-CHAIN COMPROMISE (ATLAS AML.T0010.003 / AML.T0011.000). The model ships as an unsigned joblib pickle. Anyone who can write to the registry can plant a payload that runs on load inside the Frankfurt PHI environment, or quietly patch predict_proba to lower scores for Rural patients.</t>
         </is>
       </c>
       <c r="C12" s="26" t="inlineStr">
         <is>
-          <t>[Regulatory / Security / Fairness / Privacy / Operational]</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="D12" s="26" t="inlineStr">
         <is>
-          <t>[Govern / Map / Measure / Manage]</t>
-        </is>
-      </c>
-      <c r="E12" s="26" t="inlineStr">
-        <is>
-          <t>[D1 / D2 / D3 / D4]</t>
-        </is>
-      </c>
-      <c r="F12" s="26" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
-      </c>
-      <c r="G12" s="26" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
-      </c>
-      <c r="H12" s="11">
+          <t>Manage</t>
+        </is>
+      </c>
+      <c r="E12" s="47" t="inlineStr">
+        <is>
+          <t>D3</t>
+        </is>
+      </c>
+      <c r="F12" s="47" t="n">
+        <v>3</v>
+      </c>
+      <c r="G12" s="47" t="n">
+        <v>5</v>
+      </c>
+      <c r="H12" s="48">
         <f>IFERROR(F12*G12,"")</f>
         <v/>
       </c>
       <c r="I12" s="26" t="inlineStr">
         <is>
-          <t>[Specific control — name a framework, library entry, or mechanism]</t>
-        </is>
-      </c>
-      <c r="J12" s="26" t="inlineStr">
-        <is>
-          <t>[Low / Low-Medium / Medium / Medium-High / High]</t>
-        </is>
-      </c>
-      <c r="K12" s="26" t="inlineStr">
-        <is>
-          <t>[TRUE / FALSE]</t>
-        </is>
+          <t>1) Replace pickle with skops.io (trusted-types allow-list) or ONNX + onnxruntime. 2) Sign artifacts with Sigstore cosign in CI, and verify signature and sha256 before loading (AML.M0013, AML.M0014). 3) modelscan / picklescan as a CI gate (AML.M0016). 4) Immutable registry storage (S3 Object Lock) with CI-only writes and two-person promotion. 5) A CycloneDX ML-BOM for each release (AML.M0023).</t>
+        </is>
+      </c>
+      <c r="J12" s="47" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="K12" s="47" t="b">
+        <v>0</v>
       </c>
       <c r="L12" s="26" t="inlineStr">
         <is>
-          <t>[Optional notes / justification for high scores]</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="36" customHeight="1">
+          <t>NIST MEASURE 2.7 (security and resilience evaluated) and GOVERN 6.1 (third-party / supply-chain risk). I5 because the result would be a PHI breach and stealthy patient harm. Not Top-N because the fix is cheap, well understood, and can be closed before launch. Treat it as a must-fix launch condition, not an executive escalation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="111" customHeight="1">
       <c r="A13" s="11" t="inlineStr">
         <is>
           <t>RR-07</t>
@@ -3888,60 +3855,54 @@
       </c>
       <c r="B13" s="26" t="inlineStr">
         <is>
-          <t>[Risk description — be specific]</t>
+          <t>EXFILTRATION THROUGH THE INFERENCE API (ATLAS AML.T0024: membership inference and model extraction). C3 accepts raw feature vectors and returns full-precision probabilities at 200 req/min per hospital. A party holding a hospital mTLS certificate could copy the model for prohibited insurance underwriting, or test whether a known patient was in the training data, which would reveal their health status.</t>
         </is>
       </c>
       <c r="C13" s="26" t="inlineStr">
         <is>
-          <t>[Regulatory / Security / Fairness / Privacy / Operational]</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="D13" s="26" t="inlineStr">
         <is>
-          <t>[Govern / Map / Measure / Manage]</t>
-        </is>
-      </c>
-      <c r="E13" s="26" t="inlineStr">
-        <is>
-          <t>[D1 / D2 / D3 / D4]</t>
-        </is>
-      </c>
-      <c r="F13" s="26" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
-      </c>
-      <c r="G13" s="26" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
-      </c>
-      <c r="H13" s="11">
+          <t>Manage</t>
+        </is>
+      </c>
+      <c r="E13" s="47" t="inlineStr">
+        <is>
+          <t>D3</t>
+        </is>
+      </c>
+      <c r="F13" s="47" t="n">
+        <v>2</v>
+      </c>
+      <c r="G13" s="47" t="n">
+        <v>3</v>
+      </c>
+      <c r="H13" s="48">
         <f>IFERROR(F13*G13,"")</f>
         <v/>
       </c>
       <c r="I13" s="26" t="inlineStr">
         <is>
-          <t>[Specific control — name a framework, library entry, or mechanism]</t>
-        </is>
-      </c>
-      <c r="J13" s="26" t="inlineStr">
-        <is>
-          <t>[Low / Low-Medium / Medium / Medium-High / High]</t>
-        </is>
-      </c>
-      <c r="K13" s="26" t="inlineStr">
-        <is>
-          <t>[TRUE / FALSE]</t>
-        </is>
+          <t>1) Reference-only input: the API takes a patient ID plus a clinician OAuth2 token, and builds features server-side (AML.M0019). 2) Return a risk band, not a raw probability (AML.M0002). 3) Per-clinician quotas using Upstash rate limiting, with alerts on unusual coverage of the feature space (AML.M0004). 4) An ML Privacy Meter membership-inference audit as a release gate (attack AUC &lt;= 0.55).</t>
+        </is>
+      </c>
+      <c r="J13" s="47" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="K13" s="47" t="b">
+        <v>0</v>
       </c>
       <c r="L13" s="26" t="inlineStr">
         <is>
-          <t>[Optional notes / justification for high scores]</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="36" customHeight="1">
+          <t>NIST MEASURE 2.7 / MEASURE 2.10 (privacy risk examined). Likelihood is low because the API sits behind hospital mTLS and is not internet-facing. Links to D2 (prohibited insurance use; health-data disclosure).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="96" customHeight="1">
       <c r="A14" s="11" t="inlineStr">
         <is>
           <t>RR-08</t>
@@ -3949,60 +3910,54 @@
       </c>
       <c r="B14" s="26" t="inlineStr">
         <is>
-          <t>[Risk description — be specific]</t>
+          <t>UNLAWFUL SECONDARY USE OF CLINICAL DATA FOR RETRAINING. Inference outputs and clinician overrides are reused to retrain the model. That is a new purpose outside Klariova's processor mandate, which makes Klariova a controller with no lawful basis (GDPR Arts 5(1)(b), 6(4), 9(2)(j), 28(10)). It is also probably outside HIPAA business-associate permitted uses.</t>
         </is>
       </c>
       <c r="C14" s="26" t="inlineStr">
         <is>
-          <t>[Regulatory / Security / Fairness / Privacy / Operational]</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="D14" s="26" t="inlineStr">
         <is>
-          <t>[Govern / Map / Measure / Manage]</t>
-        </is>
-      </c>
-      <c r="E14" s="26" t="inlineStr">
-        <is>
-          <t>[D1 / D2 / D3 / D4]</t>
-        </is>
-      </c>
-      <c r="F14" s="26" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
-      </c>
-      <c r="G14" s="26" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
-      </c>
-      <c r="H14" s="11">
+          <t>Govern</t>
+        </is>
+      </c>
+      <c r="E14" s="47" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="F14" s="47" t="n">
+        <v>4</v>
+      </c>
+      <c r="G14" s="47" t="n">
+        <v>4</v>
+      </c>
+      <c r="H14" s="48">
         <f>IFERROR(F14*G14,"")</f>
         <v/>
       </c>
       <c r="I14" s="26" t="inlineStr">
         <is>
-          <t>[Specific control — name a framework, library entry, or mechanism]</t>
-        </is>
-      </c>
-      <c r="J14" s="26" t="inlineStr">
-        <is>
-          <t>[Low / Low-Medium / Medium / Medium-High / High]</t>
-        </is>
-      </c>
-      <c r="K14" s="26" t="inlineStr">
-        <is>
-          <t>[TRUE / FALSE]</t>
-        </is>
+          <t>1) A formal role decision, then a DPA/BAA amendment or an Art. 26 joint-controller arrangement with each hospital. 2) An Art. 6(4) compatibility test plus an Art. 9(2)(j) / 89(1) research-safeguard assessment, or patient opt-in. 3) Block override and inference data from training pipelines until a lawful basis is documented (same quarantine as RR-05). 4) Add it to the RoPA and DPIA.</t>
+        </is>
+      </c>
+      <c r="J14" s="47" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="K14" s="47" t="b">
+        <v>1</v>
       </c>
       <c r="L14" s="26" t="inlineStr">
         <is>
-          <t>[Optional notes / justification for high scores]</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="36" customHeight="1">
+          <t>NIST GOVERN 1.1. Top-N: breaches the Board's LOW appetite for regulatory non-compliance in both the EU and the US. It is also the legal side of RR-05, since the same feedback loop is both unlawful and a poisoning path. D2 risk C1 (score 16).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="96" customHeight="1">
       <c r="A15" s="11" t="inlineStr">
         <is>
           <t>RR-09</t>
@@ -4010,60 +3965,54 @@
       </c>
       <c r="B15" s="26" t="inlineStr">
         <is>
-          <t>[Risk description — be specific]</t>
+          <t>NO DPIA AND NO PROFILING SAFEGUARDS. Large-scale health profiling makes a DPIA mandatory (GDPR Art. 35(3)(a)), and none exists. Patient notices do not explain the logic (Arts 13(2)(f), 14(2)(g)), and nothing shows the human review would satisfy SCHUFA (C-634/21). For CA non-PHI data, the CCPA risk-assessment and ADMT regulations (11 CCR §7150, §7200) apply.</t>
         </is>
       </c>
       <c r="C15" s="26" t="inlineStr">
         <is>
-          <t>[Regulatory / Security / Fairness / Privacy / Operational]</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="D15" s="26" t="inlineStr">
         <is>
-          <t>[Govern / Map / Measure / Manage]</t>
-        </is>
-      </c>
-      <c r="E15" s="26" t="inlineStr">
-        <is>
-          <t>[D1 / D2 / D3 / D4]</t>
-        </is>
-      </c>
-      <c r="F15" s="26" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
-      </c>
-      <c r="G15" s="26" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
-      </c>
-      <c r="H15" s="11">
+          <t>Govern</t>
+        </is>
+      </c>
+      <c r="E15" s="47" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="F15" s="47" t="n">
+        <v>5</v>
+      </c>
+      <c r="G15" s="47" t="n">
+        <v>3</v>
+      </c>
+      <c r="H15" s="48">
         <f>IFERROR(F15*G15,"")</f>
         <v/>
       </c>
       <c r="I15" s="26" t="inlineStr">
         <is>
-          <t>[Specific control — name a framework, library entry, or mechanism]</t>
-        </is>
-      </c>
-      <c r="J15" s="26" t="inlineStr">
-        <is>
-          <t>[Low / Low-Medium / Medium / Medium-High / High]</t>
-        </is>
-      </c>
-      <c r="K15" s="26" t="inlineStr">
-        <is>
-          <t>[TRUE / FALSE]</t>
-        </is>
+          <t>1) A DPIA template led by Klariova, adopted and signed by each hospital (the controller) before go-live. 2) A plain-language notice text explaining the logic, supplied to hospitals for their privacy notices. 3) Override and concordance KRI (KRI-2) kept as evidence of meaningful human review. 4) CCPA risk-assessment record for any CA processing that is not PHI.</t>
+        </is>
+      </c>
+      <c r="J15" s="47" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="K15" s="47" t="b">
+        <v>0</v>
       </c>
       <c r="L15" s="26" t="inlineStr">
         <is>
-          <t>[Optional notes / justification for high scores]</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="36" customHeight="1">
+          <t>NIST GOVERN 1.1 / MAP 1.1 (context and impacts documented). L5 because the gap is certain today. I3 because it is fixable on paper within weeks and the main exposure is a supervisory finding. D2 risk C3 (score 15).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="111" customHeight="1">
       <c r="A16" s="11" t="inlineStr">
         <is>
           <t>RR-10</t>
@@ -4071,60 +4020,54 @@
       </c>
       <c r="B16" s="26" t="inlineStr">
         <is>
-          <t>[Risk description — be specific]</t>
+          <t>US→EU TELEMETRY TREATED AS NON-PERSONAL. The request metadata can be linked back to patients and is derived from health data. GDPR applies to it in Frankfurt (Art. 3(1)). Return flows (alerts, dashboards viewed from Boston) have no DPF certification or SCCs. There is no HIPAA subcontractor BAA between the group companies, Texas SB 1188's US-storage requirement has not been assessed, and the flow is not in the Art. 30 RoPA.</t>
         </is>
       </c>
       <c r="C16" s="26" t="inlineStr">
         <is>
-          <t>[Regulatory / Security / Fairness / Privacy / Operational]</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="D16" s="26" t="inlineStr">
         <is>
-          <t>[Govern / Map / Measure / Manage]</t>
-        </is>
-      </c>
-      <c r="E16" s="26" t="inlineStr">
-        <is>
-          <t>[D1 / D2 / D3 / D4]</t>
-        </is>
-      </c>
-      <c r="F16" s="26" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
-      </c>
-      <c r="G16" s="26" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
-      </c>
-      <c r="H16" s="11">
+          <t>Govern</t>
+        </is>
+      </c>
+      <c r="E16" s="47" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="F16" s="47" t="n">
+        <v>3</v>
+      </c>
+      <c r="G16" s="47" t="n">
+        <v>4</v>
+      </c>
+      <c r="H16" s="48">
         <f>IFERROR(F16*G16,"")</f>
         <v/>
       </c>
       <c r="I16" s="26" t="inlineStr">
         <is>
-          <t>[Specific control — name a framework, library entry, or mechanism]</t>
-        </is>
-      </c>
-      <c r="J16" s="26" t="inlineStr">
-        <is>
-          <t>[Low / Low-Medium / Medium / Medium-High / High]</t>
-        </is>
-      </c>
-      <c r="K16" s="26" t="inlineStr">
-        <is>
-          <t>[TRUE / FALSE]</t>
-        </is>
+          <t>1) Send aggregate-only telemetry: per-feature histograms and PSI per hospital per day, with cell size k &gt;= 20 and no patient or request IDs. 2) Self-certify Klariova Inc. under the EU-US DPF, with 2021 SCCs Module 4 as the fallback. 3) A short TIA kept on file for the SCC fallback. 4) A HIPAA subcontractor BAA (45 CFR §164.504(e)(2)(ii)(D)). 5) An Art. 30 RoPA entry.</t>
+        </is>
+      </c>
+      <c r="J16" s="47" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="K16" s="47" t="b">
+        <v>0</v>
       </c>
       <c r="L16" s="26" t="inlineStr">
         <is>
-          <t>[Optional notes / justification for high scores]</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="36" customHeight="1">
+          <t>NIST GOVERN 1.1 / MEASURE 2.10. This supersedes the RR-EX example. The US→EU leg is not itself a Chapter V transfer; the return legs are (see D2 Section B). I4 because both GDPR (Art. 83(5)) and HIPAA (hospital BAAs) are exposed. D2 risk C4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="111" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
           <t>RR-11</t>
@@ -4132,60 +4075,54 @@
       </c>
       <c r="B17" s="26" t="inlineStr">
         <is>
-          <t>[Risk description — be specific]</t>
+          <t>OVER-COLLECTION AND OVER-RETENTION CONCENTRATE BREACH IMPACT. Hospitals push full FHIR records although the model uses 13 fields. Identifiable feature vectors are kept for 7 years, every training dataset ever used sits in the registry indefinitely, and Kafka encryption and retention are undocumented (GDPR Arts 5(1)(c), 5(1)(e), 32; CPRA §1798.100(a)(3), (c); breach liability under §1798.150).</t>
         </is>
       </c>
       <c r="C17" s="26" t="inlineStr">
         <is>
-          <t>[Regulatory / Security / Fairness / Privacy / Operational]</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="D17" s="26" t="inlineStr">
         <is>
-          <t>[Govern / Map / Measure / Manage]</t>
-        </is>
-      </c>
-      <c r="E17" s="26" t="inlineStr">
-        <is>
-          <t>[D1 / D2 / D3 / D4]</t>
-        </is>
-      </c>
-      <c r="F17" s="26" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
-      </c>
-      <c r="G17" s="26" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
-      </c>
-      <c r="H17" s="11">
+          <t>Manage</t>
+        </is>
+      </c>
+      <c r="E17" s="47" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="F17" s="47" t="n">
+        <v>4</v>
+      </c>
+      <c r="G17" s="47" t="n">
+        <v>3</v>
+      </c>
+      <c r="H17" s="48">
         <f>IFERROR(F17*G17,"")</f>
         <v/>
       </c>
       <c r="I17" s="26" t="inlineStr">
         <is>
-          <t>[Specific control — name a framework, library entry, or mechanism]</t>
-        </is>
-      </c>
-      <c r="J17" s="26" t="inlineStr">
-        <is>
-          <t>[Low / Low-Medium / Medium / Medium-High / High]</t>
-        </is>
-      </c>
-      <c r="K17" s="26" t="inlineStr">
-        <is>
-          <t>[TRUE / FALSE]</t>
-        </is>
+          <t>1) A FHIR field allow-list at ingestion. 2) Split storage: identifiable predictions kept under the hospital's retention policy, and a pseudonymised monitoring store with tokenised IDs. 3) A documented retention and deletion schedule for the registry and Kafka (Kafka retention 7 days or less). 4) KMS encryption, RBAC and access logging on the prediction DB and registry.</t>
+        </is>
+      </c>
+      <c r="J17" s="47" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="K17" s="47" t="b">
+        <v>0</v>
       </c>
       <c r="L17" s="26" t="inlineStr">
         <is>
-          <t>[Optional notes / justification for high scores]</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="36" customHeight="1">
+          <t>NIST MANAGE 1.3 (responses to high-priority risks planned) / MEASURE 2.10. D2 risk C5. Also makes the impact of RR-05, RR-06 and RR-07 smaller if any of them happens.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="111" customHeight="1">
       <c r="A18" s="11" t="inlineStr">
         <is>
           <t>RR-12</t>
@@ -4193,56 +4130,50 @@
       </c>
       <c r="B18" s="26" t="inlineStr">
         <is>
-          <t>[Risk description — be specific]</t>
+          <t>SUBGROUP HARM WE CANNOT FULLY MEASURE. Rural × Uninsured (FNR 50%, n_pos=10) and Rural × Medicare (n_pos=16) are below the n_pos &gt;= 20 power filter. Test labels carry the same under-diagnosis (Rural × Medicaid prevalence 11.6% vs about 26%), so the measured FNR is probably an under-estimate. The global SHAP proxy screen flagged nothing (is_likely_proxy = 'no' for every feature). There is no standard-of-care baseline.</t>
         </is>
       </c>
       <c r="C18" s="26" t="inlineStr">
         <is>
-          <t>[Regulatory / Security / Fairness / Privacy / Operational]</t>
+          <t>Fairness</t>
         </is>
       </c>
       <c r="D18" s="26" t="inlineStr">
         <is>
-          <t>[Govern / Map / Measure / Manage]</t>
-        </is>
-      </c>
-      <c r="E18" s="26" t="inlineStr">
-        <is>
-          <t>[D1 / D2 / D3 / D4]</t>
-        </is>
-      </c>
-      <c r="F18" s="26" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
-      </c>
-      <c r="G18" s="26" t="inlineStr">
-        <is>
-          <t>[1-5]</t>
-        </is>
-      </c>
-      <c r="H18" s="11">
+          <t>Measure</t>
+        </is>
+      </c>
+      <c r="E18" s="47" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
+      <c r="F18" s="47" t="n">
+        <v>4</v>
+      </c>
+      <c r="G18" s="47" t="n">
+        <v>4</v>
+      </c>
+      <c r="H18" s="48">
         <f>IFERROR(F18*G18,"")</f>
         <v/>
       </c>
       <c r="I18" s="26" t="inlineStr">
         <is>
-          <t>[Specific control — name a framework, library entry, or mechanism]</t>
-        </is>
-      </c>
-      <c r="J18" s="26" t="inlineStr">
-        <is>
-          <t>[Low / Low-Medium / Medium / Medium-High / High]</t>
-        </is>
-      </c>
-      <c r="K18" s="26" t="inlineStr">
-        <is>
-          <t>[TRUE / FALSE]</t>
-        </is>
+          <t>1) Pooled validation across several sites, sized by a power calculation so every region × insurance cell reaches n_pos &gt;= 20. 2) Report Wilson 95% CIs alongside every subgroup FNR. 3) Re-adjudicate a label sample to estimate hidden positives. 4) Add subgroup-conditional SHAP (mean SHAP per intersectional cell) to the CI release gate. 5) Benchmark against FINDRISC / ADA risk score on the same cohort.</t>
+        </is>
+      </c>
+      <c r="J18" s="47" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K18" s="47" t="b">
+        <v>0</v>
       </c>
       <c r="L18" s="26" t="inlineStr">
         <is>
-          <t>[Optional notes / justification for high scores]</t>
+          <t>NIST MEASURE 2.5 (validity and reliability demonstrated) / MEASURE 2.13 (effectiveness of TEVV metrics). This is the known limitation of the small-n filter in find_most_harmed_subgroup. Reported in D8 limitations. Not Top-N on its own because it is escalated with RR-01.</t>
         </is>
       </c>
     </row>
@@ -4369,8 +4300,8 @@
   <dimension ref="A1:B30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="70" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -4402,10 +4333,24 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="140" customHeight="1">
+    <row r="6" ht="265" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
         <is>
-          <t>[Model: HealthGuard. Version: v1.0-rc7. Framework: scikit-learn 1.7 (gradient-boosted tree classifier). Decision threshold: 0.26. Owner: Office of the Chief AI Risk Officer at Klariova Health.]</t>
+          <t>Name: HealthGuard, a type-2 diabetes (T2D) risk prediction system (clinical decision support).
+Version: healthguard-v1.0-rc7 (release candidate). STATUS: NOT APPROVED FOR DEPLOYMENT, pending the launch decision (D8).
+Model type: scikit-learn Pipeline.
+- ColumnTransformer: StandardScaler on 9 numeric features (age, bmi, glucose, blood_pressure, insulin, skin_thickness, pregnancies, family_history, pedigree), and OneHotEncoder(handle_unknown='ignore') on 4 categorical features (sex, age_group, region, insurance_type). That gives 22 model inputs after encoding.
+- GradientBoostingClassifier(n_estimators=180, learning_rate=0.08, random_state=20260425).
+Framework: scikit-learn 1.7 (artifact serialised with 1.7.2 / numpy 2.x as an unsigned joblib pickle; see §6). Trained in-house; no pretrained or third-party model components.
+Output: probability of developing T2D, plus a binary high-risk / not-high-risk flag.
+Decision threshold: 0.26, chosen for sensitivity (it favours recall over precision). There is no documented clinical cost-benefit rationale yet, and deployers must not change it.
+Training run: 2027-03-12. Training-data manifest: sha256:7f3c…a82e (Model Registry).
+Ownership:
+- Provider under EU AI Act Art. 3(3): Klariova Health (Dublin).
+- Accountable model owner: Head of Machine Learning.
+- Risk oversight and launch approver: Chief AI Risk Officer, with AI Review Board sign-off.
+External validation: none to date.
+Card version: v0.1, pre-launch review draft. Update on every model version, threshold change or new deployment region.</t>
         </is>
       </c>
       <c r="B6" s="6" t="n"/>
@@ -4424,10 +4369,26 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="140" customHeight="1">
+    <row r="10" ht="385" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>[Intended use: clinician decision-support during routine primary-care visits — prioritize HbA1c testing, trigger referrals to diabetes-prevention program. Decision-support only; clinician HITL on every prediction. Non-intended: insurance underwriting; automated denial of care; direct patient-facing communication; employment screening; use outside primary-care; any use that would constitute a regulated medical-device decision under MDR 2017/745.]</t>
+          <t>INTENDED USE: Decision support for licensed primary-care and endocrinology clinicians during routine visits with adult patients (training ages 18-85) who have no existing diabetes diagnosis. The score helps prioritise earlier HbA1c / fasting-glucose testing, lifestyle counselling, and referral to a diabetes-prevention programme. A clinician reviews every prediction before any action is taken. The tool informs clinical judgement and does not replace it.
+Deployment: EU first (4 academic medical centres in IE, DE, NL and SE; Q3 2027), then the US (3 IDNs in CA, MA and TX; Q4 2027, gated on US validation; see §3).
+IMPORTANT: a 'not high-risk' result does NOT rule out diabetes, and must not suppress guideline-based screening (e.g., ADA: screen all adults from age 35, and earlier for adults with overweight plus risk factors).
+PROHIBITED USES (contractual, from brief §3; enforced technically where possible):
+- Insurance underwriting, pricing or coverage decisions.
+- Automated denial of care, referral or coverage.
+- Showing risk scores directly to patients without clinician interpretation (no patient-facing endpoint).
+- Employment, occupational-health or any other non-clinical screening.
+- Use outside primary care / endocrinology, e.g. the ED or ICU (blocked per tenant).
+- Autonomous or diagnostic use.
+OUT OF SCOPE (not validated):
+- Patients under 18.
+- Type 1 diabetes, gestational-diabetes screening, or patients already diagnosed.
+- US populations, until US-representative validation is complete.
+- Any decision threshold other than 0.26.
+USE WITH CAUTION: subgroups with a known high miss rate, i.e. Rural × Medicaid / Uninsured and ages 21-35 (§4).
+REGULATORY NOTE: the brief positions HealthGuard as 'not an MDR device'. D1 finds it probably IS medical-device software (MDR Rule 11, Class IIa). Treat it as such until a formal qualification opinion is obtained.</t>
         </is>
       </c>
       <c r="B10" s="6" t="n"/>
@@ -4446,10 +4407,24 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="140" customHeight="1">
+    <row r="14" ht="310" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>[Two sources: (Source 1) anonymized EHR extracts from Ireland and Germany customer hospitals under DPA opt-in. (Source 2) synthetic data generated to balance demographic representation. Total ~12,000 records. Known limitations: synthetic generator inherited care-access disparity from Source 1; insurance_type sourced from billing systems; geographic distribution not representative of US deployment population; no independent validation.]</t>
+          <t>SOURCES:
+- Source 1: anonymised EHR extracts from two customer hospitals (Ireland and Germany). Licensed under the DPA, with explicit opt-in for secondary use in model development.
+- Source 2: synthetic records from an internal generative model trained on Source 1, intended to boost rural and suburban sample sizes.
+The proportion of Source 1 vs Source 2 records is NOT recorded in the manifest.
+SIZE: train.csv has 12,000 records (Urban 5,423 / Suburban 4,089 / Rural 2,488; F 6,613 / M 5,387; Private 6,316 / Medicaid 2,724 / Medicare 2,047 / Uninsured 913; prevalence 25%). Held-out test set: 3,000 records. The brief states '~8,000 records', so the manifest hash and dataset need reconciling before Annex IV sign-off.
+LABEL: diabetes_outcome is a RECORDED T2D diagnosis from the EHR, not confirmed disease status. It therefore inherits care-access bias.
+KNOWN LIMITATIONS (from D1/D4 analysis):
+(1) LABEL BIAS. Recorded prevalence is 13.5% for Rural × Medicaid and 12.7% for Rural × Uninsured, against 26-29% in every other cell. Under-served patients were diagnosed less often, and the Source 2 generator copied this pattern rather than correcting it.
+(2) PROXY STRUCTURE. Rural patients are 45% Medicaid in training (vs 15% for Urban), so region and insurance_type together encode socio-economic access.
+(3) DATA QUALITY. insurance_type comes from hospital billing and can be stale. 222 records (1.9%) have insulin = 0, which is physiologically implausible and probably missing data coded as zero. 87 patients aged 18-20 are binned into age_group '21-35'.
+(4) PROVENANCE ANOMALY. The insurance categories (Medicaid / Medicare / Uninsured) are US payer types, yet Source 1 is IE/DE data. The mapping or generation step must be documented.
+(5) REPRESENTATIVENESS. Geography is IE+DE only, which does not represent the US deployment population.
+(6) PRIVACY. The synthetic data has not been tested for memorisation or re-identification.
+(7) VALIDATION. There has been no independent external validation, and no comparison with a standard-of-care score (FINDRISC / ADA).
+EU AI Act Art. 10 status: NOT MET (D1).</t>
         </is>
       </c>
       <c r="B14" s="6" t="n"/>
@@ -4468,10 +4443,18 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="140" customHeight="1">
+    <row r="18" ht="175" customHeight="1">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>[Populated by audit_notebook.ipynb after the technical audit runs.]</t>
+          <t>OVERALL (test n=3,000; prevalence 25.0%; threshold 0.26): ROC AUC 0.812 | recall 0.744 (FNR 25.6%) | precision 0.476 | F1 0.581 | accuracy 0.731.
+By region — FNR (FPR, n_pos): Rural 37.8% (19.5%, 111); Suburban 24.5% (30.9%, 273); Urban 22.7% (28.7%, 366).
+By insurance_type — FNR (FPR, n_pos): Medicaid 31.3% (23.0%, 134); Medicare 20.8% (32.7%, 130); Private 24.0% (29.4%, 438); Uninsured 37.5% (15.5%, 48).
+By age_group — FNR (FPR, n_pos): 21-35 48.9% (18.2%, 92); 36-50 26.5% (23.7%, 189); 51-65 22.9% (32.9%, 279); 66+ 17.4% (41.8%, 190).
+By sex — FNR (FPR, n_pos): F 24.6% (29.4%, 422); M 26.8% (24.9%, 328).
+INTERSECTIONAL region × insurance (9 of 12 cells with n_pos ≥ 20): FNR 17.2%–60.6%. Most harmed: Rural × Medicaid FNR 60.6% (n_pos=33).
+Below the n_pos ≥ 20 power filter (not quantifiable): Rural × Medicare FNR 31.2% (n_pos=16); Rural × Uninsured FNR 50.0% (n_pos=10); Urban × Uninsured FNR 29.4% (n_pos=17).
+PROXY-PATHWAY TEST: proxy_supported. Within Rural, Medicaid vs Private FNR gap is +37.5 pp against -5.2 pp in Urban (+42.8 pp excess, margin 5 pp): the secondary axis carries disparity inside Rural.
+KRI-1 Subgroup FNR Drift: Red. FNR gap 43.4 pp: worst Rural × Medicaid 60.6% vs best Urban × Medicare 17.2% across 9 cells with &gt;= 20 positives (Green &lt;= 8, Amber &lt;= 15, Red &gt; 15).</t>
         </is>
       </c>
       <c r="B18" s="6" t="n"/>
@@ -4490,13 +4473,35 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="140" customHeight="1">
+    <row r="22" ht="145" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t>[Top SHAP features dominated by clinical signals (glucose, bmi, age). insurance_type categories rank in top 8 with negative effect direction — proxy fingerprint. Limitations: SHAP is correlational not causal; small-n cell findings (e.g., Rural+Uninsured) are not statistically robust; metrics computed at threshold 0.26 only; current Clinician Dashboard does not expose instance-level SHAP — likely insufficient under EU AI Act Article 13 transparency.]</t>
+          <t>SHAP FINDINGS [generated by audit_notebook.ipynb; TreeExplainer (tree_path_dependent), log-odds, test n=3,000]
+Global top-5 features by mean |SHAP|: num__glucose 0.806; num__bmi 0.294; num__age 0.278; num__family_history 0.142; num__pedigree 0.114.
+Proxy candidates (protected substrings region / sex / age_group excluded): #1 num__glucose |0.806| mean +0.038 strength 0.05; #2 num__bmi |0.294| mean -0.006 strength 0.02; #3 num__age |0.278| mean -0.006 strength 0.02; #4 num__family_history |0.142| mean -0.005 strength 0.03; #5 num__pedigree |0.114| mean +0.002 strength 0.02; #6 num__blood_pressure |0.110| mean +0.000 strength 0.00; #7 num__pregnancies |0.096| mean -0.001 strength 0.02; #8 cat__insurance_type_Medicaid |0.076| mean -0.002 strength 0.03.
+Flagged by the global is_likely_proxy rule (mean_shap &lt; -0.01 and strength ≥ 0.5): 0 of 8.
+Subgroup-conditional: mean region + insurance_type SHAP = -0.592 log-odds in Rural × (Medicaid|Uninsured) vs +0.145 in Urban × Private.
+Local false negatives in Rural × (Medicaid|Uninsured), top-3 negative drivers: row 155: cat__region_Rural -0.271, cat__insurance_type_Medicaid -0.234, num__blood_pressure -0.162 | row 217: num__age -0.448, cat__region_Rural -0.268, num__bmi -0.245 | row 225: cat__insurance_type_Uninsured -0.339, cat__region_Rural -0.272, num__family_history -0.108.</t>
         </is>
       </c>
       <c r="B22" s="6" t="n"/>
+    </row>
+    <row r="23" ht="265" customHeight="1">
+      <c r="A23" s="26" t="inlineStr">
+        <is>
+          <t>5b. EXPLAINABILITY LIMITATIONS [HAND]
+(1) GLOBAL SHAP MISSES THE PROXY. insurance_type_Medicaid ranks #8 by importance, but its average signed effect is close to zero (strength 0.03), and the global is_likely_proxy rule flagged 0 of 8 candidates. The proxy effect points in opposite directions in different cells (-0.59 log-odds in Rural × Medicaid/Uninsured vs +0.15 in Urban × Private) and affects about 12% of patients, so it cancels out in a population average. A global SHAP screen alone would have cleared this model. Proxy screening must be subgroup-conditional (mean SHAP per intersectional cell), and that check is now proposed as a CI release gate (D5 RR-12).
+(2) CORRELATED FEATURES. region and insurance_type are strongly correlated, so tree-path-dependent SHAP splits credit between them somewhat arbitrarily. SHAP cannot separate a 'region' effect from an 'insurance' effect; only retraining without the features (ablation) can.
+(3) SHAP EXPLAINS THE MODEL, NOT THE PATIENT. Attributions show what drives the score, not what causes diabetes. Because the labels carry under-diagnosis, SHAP faithfully explains a biased model. Low attribution does not mean low clinical relevance, and the attributions are not counterfactuals.
+(4) ONE-HOT ENCODING. Each category gets its own SHAP value. 'Not being Medicaid' also contributes, so per-feature effects must be summed across the category columns before anyone interprets them.
+(5) LIMITED SCOPE. Results are computed at threshold 0.26 on a single synthetic test split. Cells with n_pos &lt; 20 (Rural × Uninsured, Rural × Medicare, Urban × Uninsured) are not statistically reliable.
+(6) CLINICIAN-FACING GAP. The dashboard currently shows a 'rough explanation, not full SHAP', which is probably insufficient under EU AI Act Art. 13(3)(b). Before launch:
+- Show validated per-patient top-3 CLINICAL drivers.
+- Add an explicit banner when non-clinical features (region / insurance_type) materially lowered the score.
+- Test that clinicians understand the explanations, since a confident-looking explanation can increase over-trust (automation bias).</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="n"/>
     </row>
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
@@ -4512,10 +4517,23 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="140" customHeight="1">
+    <row r="26" ht="400" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>[3 ATLAS TTPs from D3: AML.T0020 Poison Training Data (Component 5), AML.T0043 Craft Adversarial Data (Component 3), AML.T0048 Erode ML Model Integrity (Components 4→6 override loop). For each: specific component, attack scenario, proposed mitigation. Note: T0020 risk is elevated by existing organic data-quality issues which would mask malicious activity.]</t>
+          <t>BASELINE CONTROLS: mTLS at the hospital edge; rate limiting at 200 req/min per hospital. NONE of the AI-specific mitigations below are implemented yet. They are launch conditions (D5).
+T1. AML.T0020 Poison Training Data (related: AML.T0018.000). Target: C4 Clinician Dashboard → C5 Model Registry (the override feedback loop).
+- Scenario: a phished clinician account, or simply biased overrides, records 'not high-risk' on true positives in a small subgroup. Those overrides become training labels, so the next model's subgroup FNR rises while overall AUC barely moves. Existing data-quality noise (label bias, stale insurance_type) would hide the attack.
+- Mitigations: override quarantine with second-clinician adjudication (AML.M0007); per-clinician label caps plus cleanlab screening; a CI gate on a frozen golden set that blocks any subgroup FNR rise above 2 pp (AML.M0008); DVC/lakeFS lineage (AML.M0025).
+- Likelihood M-H / Impact H. D5 RR-05 (Top-N).
+T2. AML.T0010.003 AI Supply Chain Compromise: Model (related: AML.T0011.000 Unsafe AI Artifacts). Target: C5 Registry → C3 Inference API.
+- Scenario: an attacker with stolen CI or engineer credentials replaces the unsigned joblib pickle with one carrying a __reduce__ payload. That gives code execution inside the Frankfurt PHI environment, or a stealthy predict_proba patch that lowers Rural scores.
+- Mitigations: skops / ONNX instead of pickle; Sigstore cosign signing with signature and sha256 checked before load (AML.M0013, AML.M0014); a modelscan CI gate (AML.M0016); immutable WORM registry with two-person promotion; a CycloneDX ML-BOM (AML.M0023).
+- Likelihood M / Impact H. D5 RR-06.
+T3. AML.T0024 Exfiltration via AI Inference API (.000 membership inference, .002 model extraction). Target: C3 Inference API.
+- Scenario: a party holding a hospital mTLS certificate queries raw feature vectors and gets back full-precision probabilities. They can build a surrogate model for prohibited insurance underwriting, or test whether a known patient was in the training data, revealing health status.
+- Mitigations: reference-only input (patient ID plus clinician OAuth2 token; AML.M0019); risk-band output (AML.M0002); per-clinician quotas with Upstash (AML.M0004); an ML Privacy Meter release gate (attack AUC ≤ 0.55).
+- Likelihood L-M / Impact M. D5 RR-07.
+DEPRIORITISED: AML.T0015 / AML.T0043 (evasion and crafted adversarial data). No plausible actor has a motive to lower a preventive score. Out of scope: LLM and prompt-injection techniques, since there is no generative component.</t>
         </is>
       </c>
       <c r="B26" s="6" t="n"/>
@@ -4534,16 +4552,33 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="140" customHeight="1">
+    <row r="30" ht="370" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>[EU AI Act high-risk classification under Art. 6 + Annex III, point 5(a). Key compliance status: Art. 10 Not Met, Art. 13 Not Met, Art. 15 Partially Met. GDPR/CPRA: 5 gaps identified. Post-deployment monitoring via the 3 KRIs in D7 (subgroup FNR drift, override channel health, inference anomaly rate).]</t>
+          <t>EU AI ACT (D1): HIGH-RISK. Primary basis Art. 6(1) + Annex I §A (MDR 2017/745, Rule 11, Class IIa, notified-body conformity assessment); secondary basis Art. 6(2) + Annex III 5(a). Not prohibited under Art. 5. Obligations apply from 2 Aug 2027, inside the Q3 2027 launch window.
+Arts 9-15 status:
+- NOT MET: Art. 10 data governance, Art. 11 technical documentation, Art. 13 transparency.
+- PARTIALLY MET: Art. 9 RMS; Art. 10(5) special-category data; Art. 12 logging; Art. 14 oversight and override; Art. 15 accuracy (Critical), robustness and cybersecurity.
+- Launch blockers: (1) subgroup under-detection, (2) no QMS / Annex IV / conformity route, (3) oversight that does not work.
+Also required: post-market monitoring (Art. 72), serious-incident reporting (Art. 73), and a FRIA by public-body deployers (Art. 27).
+GDPR / CPRA (D2): all 8 data-flow stages show gaps. Top risks:
+- Retraining on override and inference data without a lawful basis (RR-08).
+- Processing inaccurate and unnecessary socio-economic data (Art. 5(1)(a), (c), (d); RR-01).
+- No DPIA or profiling safeguards (Art. 35, Arts 13/14, Art. 22 / SCHUFA; RR-09).
+- US→EU telemetry is personal data under GDPR Art. 3(1). Return flows need DPF or SCCs Module 4, and an intra-group HIPAA subcontractor BAA (RR-10).
+- Over-collection and over-retention (RR-11).
+US: PHI is largely exempt from CPRA (§1798.146), so HIPAA and CMIA apply. CPRA still covers clinician data and non-PHI, and the CCPA ADMT and risk-assessment regulations apply to non-PHI.
+MONITORING: KRIs implemented in lab/kri.py, status from audit_notebook.ipynb (D7):
+- KRI-1 Subgroup FNR Drift: worst-minus-best FNR across region × insurance cells with n_pos ≥ 20. Green ≤ 8 pp, Amber ≤ 15 pp, Red &gt; 15 pp. Currently RED at 43.4 pp (Rural × Medicaid 60.6% vs Urban × Medicare 17.2%). Monitors RR-01 and RR-12, and is a launch gate.
+- KRI-2 Override Channel Health: override rate ≤ 10% AND structured-reason share ≥ 80% for Green; Red if the rate is above 15% OR the share is below 60%. Shows GREEN (6.0% / 85%), but on SYNTHETIC baseline inputs, not production telemetry. Monitors RR-04, RR-05 and RR-08.
+- KRI-3 Inference Anomaly Rate: anomalies per 1,000 inferences. Green &lt; 1, Amber 1-5, Red &gt; 5. Shows GREEN (0 of 2,000), also on SYNTHETIC inputs. Monitors RR-06 and RR-07.
+KRI-2 and KRI-3 say nothing about production behaviour until they are fed real telemetry. Re-run the D4 audit and update this card on every release and every quarter.</t>
         </is>
       </c>
       <c r="B30" s="6" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="24">
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A30:B30"/>
     <mergeCell ref="A1:B1"/>
@@ -4557,6 +4592,7 @@
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A23:B23"/>
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A22:B22"/>

</xml_diff>

<commit_message>
Complete HealthGuard D7 KRI dashboard and D8 launch decision
- D7: three KRI definitions mirroring lab/kri.py thresholds, with data
  sources, owners, linked D5 risks, and per-KRI rationale/escalation
- D8: Conditional Go recommendation, plain-language executive brief,
  evidence and risk-appetite justification, C1-C7 conditions table,
  post-launch governance plan, and RACI sign-off
- D5: highlight Top-N risks via conditional formatting
- Notebook re-executed after D7 changes

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/04-secure-ai-deployment/project/starter/governance_portfolio.xlsx
+++ b/04-secure-ai-deployment/project/starter/governance_portfolio.xlsx
@@ -223,7 +223,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="2"/>
@@ -337,10 +337,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FBE1B6"/>
+          <bgColor rgb="00FBE1B6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -4287,6 +4300,11 @@
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A4:L4"/>
   </mergeCells>
+  <conditionalFormatting sqref="A7:L18">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>$K7=TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4443,7 +4461,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="175" customHeight="1">
+    <row r="18" ht="205" customHeight="1">
       <c r="A18" s="11" t="inlineStr">
         <is>
           <t>OVERALL (test n=3,000; prevalence 25.0%; threshold 0.26): ROC AUC 0.812 | recall 0.744 (FNR 25.6%) | precision 0.476 | F1 0.581 | accuracy 0.731.
@@ -4473,7 +4491,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="145" customHeight="1">
+    <row r="22" ht="175" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
         <is>
           <t>SHAP FINDINGS [generated by audit_notebook.ipynb; TreeExplainer (tree_path_dependent), log-odds, test n=3,000]
@@ -4614,18 +4632,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -4704,7 +4722,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="80" customHeight="1">
+    <row r="6" ht="156" customHeight="1">
       <c r="A6" s="11" t="inlineStr">
         <is>
           <t>1</t>
@@ -4712,46 +4730,48 @@
       </c>
       <c r="B6" s="26" t="inlineStr">
         <is>
-          <t>[KRI name]</t>
+          <t>KRI-1 Subgroup FNR Drift</t>
         </is>
       </c>
       <c r="C6" s="26" t="inlineStr">
         <is>
-          <t>[What is being measured]</t>
+          <t>Equity of missed diagnoses: the gap, in percentage points, between the worst and best false-negative rate across region × insurance_type cells.</t>
         </is>
       </c>
       <c r="D6" s="26" t="inlineStr">
         <is>
-          <t>[Data source + formula + measurement frequency]</t>
+          <t>SOURCE: C6 inference log (prediction, threshold, model version) joined to confirmed T2D outcomes from hospital EHR feedback (diagnosis or HbA1c ≥ 6.5% within 12 months of scoring).
+FORMULA: per cell, FNR = FN / (FN + TP), counting only cells with ≥ 20 confirmed positives. Gap = (max FNR − min FNR) × 100. Fewer than 2 qualifying cells → 'Insufficient'. Code: lab/kri.py kri_subgroup_fnr_drift.
+FREQUENCY: monthly, on a rolling 12-month cohort with matured outcomes, per tenant and pooled. Also a CI gate on the held-out golden set for every release candidate.</t>
         </is>
       </c>
       <c r="E6" s="26" t="inlineStr">
         <is>
-          <t>[Green threshold — numeric]</t>
+          <t>≤ 8 pp</t>
         </is>
       </c>
       <c r="F6" s="26" t="inlineStr">
         <is>
-          <t>[Amber threshold — numeric range]</t>
+          <t>&gt; 8 pp and ≤ 15 pp</t>
         </is>
       </c>
       <c r="G6" s="26" t="inlineStr">
         <is>
-          <t>[Red threshold — numeric]</t>
+          <t>&gt; 15 pp</t>
         </is>
       </c>
       <c r="H6" s="26" t="inlineStr">
         <is>
-          <t>[Specific organizational role]</t>
+          <t>Head of Machine Learning (metric owner); escalation to the Chief AI Risk Officer</t>
         </is>
       </c>
       <c r="I6" s="26" t="inlineStr">
         <is>
-          <t>[RR-## from your D5 register]</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="80" customHeight="1">
+          <t>RR-01 (primary); RR-12, RR-03, RR-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="126" customHeight="1">
       <c r="A7" s="11" t="inlineStr">
         <is>
           <t>2</t>
@@ -4759,46 +4779,48 @@
       </c>
       <c r="B7" s="26" t="inlineStr">
         <is>
-          <t>[KRI name]</t>
+          <t>KRI-2 Override Channel Health</t>
         </is>
       </c>
       <c r="C7" s="26" t="inlineStr">
         <is>
-          <t>[What is being measured]</t>
+          <t>Whether human oversight works and the override feedback channel is clean. Two criteria: how often clinicians override the score, and how often they give a structured reason.</t>
         </is>
       </c>
       <c r="D7" s="26" t="inlineStr">
         <is>
-          <t>[Data source + formula + measurement frequency]</t>
+          <t>SOURCE: C4 dashboard override events and C6 logs.
+FORMULA: override rate = overrides / scored inferences. Structured share = overrides with a controlled-vocabulary reason code / all overrides. Evaluated together. Code: lab/kri.py kri_override_health.
+FREQUENCY: weekly on a rolling 4-week window, per hospital and pooled, also broken down by region × insurance subgroup and by clinician concentration.</t>
         </is>
       </c>
       <c r="E7" s="26" t="inlineStr">
         <is>
-          <t>[Green threshold — numeric]</t>
+          <t>Override rate ≤ 10% AND structured share ≥ 80%</t>
         </is>
       </c>
       <c r="F7" s="26" t="inlineStr">
         <is>
-          <t>[Amber threshold — numeric range]</t>
+          <t>Rate &gt; 10% and ≤ 15%, OR share ≥ 60% and &lt; 80%</t>
         </is>
       </c>
       <c r="G7" s="26" t="inlineStr">
         <is>
-          <t>[Red threshold — numeric]</t>
+          <t>Rate &gt; 15% OR share &lt; 60%</t>
         </is>
       </c>
       <c r="H7" s="26" t="inlineStr">
         <is>
-          <t>[Specific organizational role]</t>
+          <t>Clinical Safety Officer, jointly with each hospital's CMIO</t>
         </is>
       </c>
       <c r="I7" s="26" t="inlineStr">
         <is>
-          <t>[RR-## from your D5 register]</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="80" customHeight="1">
+          <t>RR-04 (primary); RR-05, RR-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="186" customHeight="1">
       <c r="A8" s="11" t="inlineStr">
         <is>
           <t>3</t>
@@ -4806,42 +4828,49 @@
       </c>
       <c r="B8" s="26" t="inlineStr">
         <is>
-          <t>[KRI name]</t>
+          <t>KRI-3 Inference Anomaly Rate</t>
         </is>
       </c>
       <c r="C8" s="26" t="inlineStr">
         <is>
-          <t>[What is being measured]</t>
+          <t>Integrity and abuse signal on the Inference API: the rate of requests flagged as anomalous.</t>
         </is>
       </c>
       <c r="D8" s="26" t="inlineStr">
         <is>
-          <t>[Data source + formula + measurement frequency]</t>
+          <t>SOURCE: C3 API gateway and validation logs plus C6.
+ANOMALY: a request that triggers any rule in the versioned anomaly spec v1:
+- schema or range failure (unknown category, out-of-range value, e.g. insulin = 0, age &lt; 18);
+- per-clinician quota breach;
+- feature-space sweep / extraction pattern (IsolationForest on request vectors);
+- artifact signature or hash mismatch at load.
+FORMULA: per_1000 = anomalous / total × 1000. Total = 0 → 'Insufficient'. Code: lab/kri.py kri_inference_anomaly.
+FREQUENCY: daily, per tenant; real-time alert on Red.</t>
         </is>
       </c>
       <c r="E8" s="26" t="inlineStr">
         <is>
-          <t>[Green threshold — numeric]</t>
+          <t>&lt; 1 per 1,000</t>
         </is>
       </c>
       <c r="F8" s="26" t="inlineStr">
         <is>
-          <t>[Amber threshold — numeric range]</t>
+          <t>≥ 1 and ≤ 5 per 1,000</t>
         </is>
       </c>
       <c r="G8" s="26" t="inlineStr">
         <is>
-          <t>[Red threshold — numeric]</t>
+          <t>&gt; 5 per 1,000</t>
         </is>
       </c>
       <c r="H8" s="26" t="inlineStr">
         <is>
-          <t>[Specific organizational role]</t>
+          <t>Head of Security Operations (SOC), with ML Platform SRE on-call</t>
         </is>
       </c>
       <c r="I8" s="26" t="inlineStr">
         <is>
-          <t>[RR-## from your D5 register]</t>
+          <t>RR-06, RR-07 (primary); RR-03, RR-05</t>
         </is>
       </c>
     </row>
@@ -4965,10 +4994,10 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="110" customHeight="1">
+    <row r="16" ht="115" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>[For each KRI, write one paragraph: why this metric, what it would detect, how it ties to the Risk Register. The escalation actions and Green/Amber/Red thresholds should be defensible to a board reviewer.]</t>
+          <t>KRI-1 SUBGROUP FNR DRIFT (→ RR-01, Top-N score 25; RR-12). WHY: a missed diagnosis is HealthGuard's main clinical harm, and D4 shows the harm is concentrated rather than spread out. Overall FNR is 25.6%, but Rural × Medicaid is 60.6%. Aggregate metrics hid this; KRI-1 measures exactly the dimension the Board's LOW patient-safety appetite names ('any identifiable patient subgroup'). WHAT IT DETECTS: the existing proxy bias; regressions after retraining (including poisoning through the override loop, RR-05); and population drift at new sites, e.g. US payer mix (RR-03). THRESHOLDS: with 20-50 positives in a cell, sampling error on an FNR near 25% is about ±8 pp (one standard error). So Green ≤ 8 pp absorbs noise, while &gt; 15 pp (about two standard errors) is unlikely to be chance. In clinical terms, 15 pp means roughly one more diabetic in seven missed in the worst group. ESCALATION: Amber → model owner root-causes within 10 business days, a subgroup caution banner is switched on, and it goes on the AI Review Board's monthly agenda. Launch is allowed only with an approved compensating control. Red → CAIRO notified within 24 h; the kill-switch falls back to standard screening for affected tenants; an AI Act Art. 73 serious-incident assessment is started. In CI, Red blocks release. CURRENT STATUS RED at 43.4 pp, computed from real test data. It is a launch blocker until mitigation brings it to Green.</t>
         </is>
       </c>
       <c r="B16" s="5" t="n"/>
@@ -4980,12 +5009,45 @@
       <c r="H16" s="5" t="n"/>
       <c r="I16" s="6" t="n"/>
     </row>
+    <row r="17" ht="115" customHeight="1">
+      <c r="A17" s="26" t="inlineStr">
+        <is>
+          <t>KRI-2 OVERRIDE CHANNEL HEALTH (→ RR-04, the oversight control; RR-05, poisoning; RR-08, unlawful reuse of override data). WHY: one channel carries two risks. Overrides are the evidence that human oversight is real (Art. 14; SCHUFA), and they are also the path by which poisoned or biased labels reach retraining. WHAT IT DETECTS: a rising override rate means clinicians and the model increasingly disagree (drift, miscalibration, or coordinated manipulation). A falling structured share means overrides can no longer be audited or safely reused, and free text risks capturing PHI. THRESHOLDS: 10% and 15% are PROVISIONAL. At precision 0.476, about 20% of all scores are false alarms, so the legitimate override rate could exceed 10% by itself. Baseline both thresholds in a 3-month shadow-mode pilot before go-live. The 80% / 60% structured-share floors reflect the minimum for adjudication to be feasible (RR-05 control). Also reported, though not part of the coded status: (a) override rate by subgroup; (b) concentration, i.e. any clinician contributing &gt; 5% of a site's overrides; (c) a SUSTAINED override rate below 1%, which signals rubber-stamping (automation bias). ESCALATION: Amber → the Clinical Safety Officer reviews a stratified override sample within 5 business days, and override data is frozen for retraining. Red → overrides are excluded from all retraining; the CAIRO and the hospital CMIO review; if overrides are concentrated in a few accounts, the SOC checks for compromise. CURRENT STATUS GREEN, but on SYNTHETIC inputs hard-coded in the notebook (6% / 85%). It is NOT evidence until fed real telemetry.</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n"/>
+      <c r="C17" s="5" t="n"/>
+      <c r="D17" s="5" t="n"/>
+      <c r="E17" s="5" t="n"/>
+      <c r="F17" s="5" t="n"/>
+      <c r="G17" s="5" t="n"/>
+      <c r="H17" s="5" t="n"/>
+      <c r="I17" s="6" t="n"/>
+    </row>
+    <row r="18" ht="145" customHeight="1">
+      <c r="A18" s="26" t="inlineStr">
+        <is>
+          <t>KRI-3 INFERENCE ANOMALY RATE (→ RR-06, model supply chain; RR-07, API exfiltration; RR-03, input data quality). WHY: the Inference API (C3) is where the D3 attack paths and the D1/D2 data-quality gaps show up at run time. It is also where they are cheapest to catch, before a bad score reaches a clinician. WHAT IT DETECTS: extraction or membership-inference probing (feature-space sweeps, quota bursts); tampered artifacts (signature mismatch at load); and integration faults that the pipeline would otherwise hide. For example, OneHotEncoder(handle_unknown='ignore') silently zeroes unknown US insurance codes, and insulin = 0 would be imputed. THRESHOLDS: in normal clinical use, validation failures are bugs, so the baseline should be near zero. Below 1 per 1,000 tolerates occasional EHR glitches. Above 5 per 1,000 (1 in 200 requests) indicates a systemic feed fault or active probing. The anomaly spec is versioned so the rate stays comparable over time. ESCALATION: Amber → ML Platform on-call triages within 1 business day, with a per-tenant breakdown and a check for any single-client burst. Red → SOC incident opened, the affected hospital's mTLS certificate or clinician tokens rotated, the tenant rate-limited, and a GDPR Art. 33 72-hour assessment started if data exposure is suspected. CURRENT STATUS GREEN on SYNTHETIC inputs (0 of 2,000). Not evidence until fed production logs.
+COVERAGE NOTE: the other two Top-N risks are tracked as dated compliance gates in the D8 conditions, not as KRIs. RR-02 (conformity assessment) and RR-08 (lawful basis for retraining) are binary legal milestones with nothing continuous to measure.</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n"/>
+      <c r="C18" s="5" t="n"/>
+      <c r="D18" s="5" t="n"/>
+      <c r="E18" s="5" t="n"/>
+      <c r="F18" s="5" t="n"/>
+      <c r="G18" s="5" t="n"/>
+      <c r="H18" s="5" t="n"/>
+      <c r="I18" s="6" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="8">
     <mergeCell ref="A15:I15"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A17:I17"/>
     <mergeCell ref="A9:I9"/>
+    <mergeCell ref="A18:I18"/>
     <mergeCell ref="A4:I4"/>
     <mergeCell ref="A16:I16"/>
   </mergeCells>
@@ -4999,11 +5061,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="74" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -5019,7 +5083,9 @@
           <t>Single document, three sections. Section A must read stand-alone for a non-technical CEO or Board reader.</t>
         </is>
       </c>
-      <c r="B2" s="6" t="n"/>
+      <c r="B2" s="5" t="n"/>
+      <c r="C2" s="5" t="n"/>
+      <c r="D2" s="6" t="n"/>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -5028,7 +5094,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="53" customHeight="1">
       <c r="A5" s="33" t="inlineStr">
         <is>
           <t>Recommendation</t>
@@ -5036,9 +5102,11 @@
       </c>
       <c r="B5" s="26" t="inlineStr">
         <is>
-          <t>[Go / Conditional Go / No Go]</t>
-        </is>
-      </c>
+          <t>CONDITIONAL GO. HealthGuard v1.0-rc7 must NOT launch as configured. A remediated release may launch in the EU only after Conditions C1-C6 are independently verified. The US launch is deferred until C7 is met.</t>
+        </is>
+      </c>
+      <c r="C5" s="44" t="n"/>
+      <c r="D5" s="44" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="33" t="inlineStr">
@@ -5052,7 +5120,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="38" customHeight="1">
       <c r="A7" s="33" t="inlineStr">
         <is>
           <t>Date</t>
@@ -5060,9 +5128,11 @@
       </c>
       <c r="B7" s="26" t="inlineStr">
         <is>
-          <t>[Project date]</t>
-        </is>
-      </c>
+          <t>2026-10-11 (decision review date = T; condition timelines below are relative to T)</t>
+        </is>
+      </c>
+      <c r="C7" s="44" t="n"/>
+      <c r="D7" s="44" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
@@ -5071,17 +5141,28 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="380" customHeight="1">
+    <row r="10" ht="355" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>[Recommendation in one line.] [Required.]
-[Top 3 residual risks in plain language, numbered (1), (2), (3).]
-[Business / patient-safety / regulatory implications — what happens if we ship as-is, in business terms.]
-[Asks of leadership — what funding, sign-offs, or timeline change you need.]
-Stand-alone test: a non-technical reader should be able to walk away from THIS section in 2 minutes with the recommendation, top risks, and asks. No jargon.</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="n"/>
+          <t>RECOMMENDATION: CONDITIONAL GO. HealthGuard must not launch in its current form. It can launch in the EU once six specific fixes are completed and checked. That is achievable for the planned Q3 2027 date, but only if the work starts now. The US launch should wait for a separate check that the tool works for American patients.
+THE THREE BIGGEST RISKS IF WE LAUNCHED TODAY
+(1) It misses diabetes far more often for poorer rural patients. Overall, HealthGuard misses about 1 in 4 patients who have diabetes. For rural patients on Medicaid it misses 6 in 10, against about 1 in 4 for rural patients with private insurance. These patients are just as sick. The tool learned from past records in which they were diagnosed less often, and it repeats that pattern. This breaks the Board's rule that we will not ship a tool that is materially worse for any identifiable group of patients.
+(2) We do not yet have legal permission to sell it in the EU. Under EU law, HealthGuard is a 'high-risk' AI system and almost certainly a regulated medical device. Before the first patient is scored, that requires a certified quality system, a full technical file, and an independent assessment by an approved certification body. None of these exist today.
+(3) The doctor safety net is not ready. The plan relies on doctors catching the tool's mistakes, but nobody tells them where it is weak. They get only a rough explanation and no training. Their corrections also feed straight back into the tool unchecked, so honest errors or deliberate tampering could make it worse over time.
+WHAT HAPPENS IF WE SHIP AS-IS
+Patients: missed or delayed diagnoses concentrated in a disadvantaged group, which is exactly the kind of harm that must be reported to regulators.
+Regulatory: the EU launch could be stopped and the product withdrawn. AI Act fines reach €15M or 3% of turnover, with further data-protection exposure on top.
+Reputation: a public fairness failure in the year we raise our Series D.
+WHAT I NEED FROM LEADERSHIP
+1. Fund a 30-day remediation sprint now (retrain and re-test the model, review the historical records, harden security), followed by the 9-month path to an EU launch.
+2. Authorise immediate engagement of a medical-device certification body and an independent validation partner. Their lead times set the launch date.
+3. Accept two timing rules. The US launch moves until it passes a US-specific test. And at a 6-month checkpoint, if EU certification is not on track, we move the EU date rather than launch without it.
+4. Confirm that doctors' corrections will not be used to retrain the tool until our data-protection basis for doing so is fixed.</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="5" t="n"/>
+      <c r="D10" s="6" t="n"/>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
@@ -5090,118 +5171,559 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="380" customHeight="1">
+    <row r="13" ht="280" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>[Evidence summary — cite ≥4 of D1-D7 by deliverable name and specific finding.]
-[Residual risk vs risk appetite — explicit comparison against the appetite statement in A1 §7.]
-[If Conditional Go: Conditions table with Condition / Measurable Threshold / Owner / Timeline.]
-[Post-launch governance plan — KRI cadence, risk register review, model card refresh trigger.]</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="n"/>
-    </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
+          <t>B.1 EVIDENCE SUMMARY
+• D1 EU AI Act Classification &amp; Gap Analysis: HIGH-RISK under Art. 6(1) + Annex I (MDR 2017/745, Rule 11, Class IIa; Annex III 5(a) secondary); not prohibited under Art. 5. Of the 11 Art. 9-15 obligations, 3 are NOT MET (Art. 10 data governance, Art. 11 technical documentation, Art. 13 transparency), 8 are PARTIALLY MET, and 0 are fully met. Two are rated Critical (Art. 10 and Art. 15 accuracy). Obligations apply from 2 Aug 2027.
+• D2 Data Flow Compliance Map: all 8 data-flow stages show GDPR/CPRA gaps. The top five: override data reused for retraining with no lawful basis; inaccurate, unnecessary socio-economic features (Art. 5(1)(a), (c), (d)); no DPIA; US→EU telemetry that is personal data under Art. 3(1), with return flows lacking DPF/SCCs and no intra-group HIPAA BAA; 7-year identifiable retention.
+• D3 MITRE ATLAS Threat Model: three credible attack paths with no AI-specific mitigation in place: AML.T0020 poisoning through the override loop (M-H/H), AML.T0010.003 unsigned joblib pickle artifact (M/H), AML.T0024 API extraction and membership inference (L-M/M).
+• D4 Technical Audit (test n=3,000, threshold 0.26): ROC AUC 0.812, recall 0.744 (FNR 25.6%).
+  - FNR is 37.8% for Rural vs 22.7% for Urban. Rural × Medicaid is 60.6% (n_pos=33; 95% CI about 44-75%) vs 23.1% for Rural × Private. Proxy pathway SUPPORTED: +37.5 pp gap within Rural vs -5.2 pp in Urban.
+  - Root cause is label bias: training prevalence is 13.5% for Rural × Medicaid vs 26-29% elsewhere, and the missed patients are clinically comparable (glucose 129 vs 133, BMI 31.2 vs 30.2).
+  - region + insurance_type contribute -0.59 log-odds in the harmed cells vs +0.15 for Urban × Private. The global SHAP proxy screen flagged nothing.
+• D5 NIST AI RMF Risk Register: 12 risks drawn from D1-D4. Top-N: RR-01 subgroup under-detection (25), RR-02 no lawful EU route (20), RR-04 oversight (16), RR-05 poisoning (16), RR-08 unlawful secondary use (16).
+• D6 Model Card: provenance gaps. The data has 12,000 training rows vs '~8,000' in the brief; US payer categories appear in IE/DE data; 222 records have insulin = 0; the label is a recorded diagnosis, not confirmed disease; there has been no external validation.
+• D7 KRI Dashboard: KRI-1 Subgroup FNR Drift is RED (43.4 pp vs Red threshold &gt; 15 pp). KRI-2 and KRI-3 are Green only on synthetic inputs, so there is no production evidence yet.</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n"/>
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="6" t="n"/>
+    </row>
+    <row r="14" ht="280" customHeight="1">
+      <c r="A14" s="26" t="inlineStr">
+        <is>
+          <t>B.2 RESIDUAL RISK vs RISK APPETITE (case-study brief §7)
+• PATIENT SAFETY (appetite LOW).
+  - As configured: OUTSIDE appetite. FNR in an identifiable subgroup is 2.6x that of its comparator (60.6% vs 23.1%), and nothing shows the model is no worse than standard of care.
+  - After C1, C2 and C4: residual Medium, which falls within appetite only if KRI-1 is Green, no powered subgroup is worse than FINDRISC, and clinician oversight (C4) acts as the compensating control. Label bias is reduced, not eliminated, so KRI-1 is monitored monthly.
+• REGULATORY NON-COMPLIANCE (appetite LOW).
+  - As configured: OUTSIDE appetite. Placing the system on the market without conformity assessment would be known non-compliance, and no compensating control can substitute for it, so C3 is a hard gate.
+  - Remaining partial-compliance items fit the Board's 'documented partial compliance' clause because each has a D5 remediation plan plus a compensating control: Art. 12 log integrity, KRI-2 threshold baselining, and US-only GDPR/HIPAA items gated by C7.
+• OPERATIONAL (appetite MODERATE): WITHIN appetite. Data residency is regional, the tool is advisory, and the C4 kill-switch falls back to standard screening, so a single-region outage of up to 4 h is tolerable.
+• REPUTATIONAL (appetite LOW): As configured, OUTSIDE appetite, because a fairness failure in a disadvantaged group is regulator-reportable and press-worthy. After the conditions are met, residual is Low-Medium.
+• FINANCIAL (appetite MODERATE): WITHIN appetite. Remediation costs (sprint, notified body, external validation) are bounded, and delaying the launch costs far less than AI Act fines of up to €15M / 3% (Art. 99(4)) or GDPR fines of up to 4% (Art. 83(5)).
+CONCLUSION: As configured, 3 of 5 appetite dimensions are breached, so v1.0-rc7 cannot launch. With C1-C6 verified, all five fall within appetite. Hence CONDITIONAL GO, with every condition met BEFORE the first EU patient is scored.</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n"/>
+      <c r="C14" s="5" t="n"/>
+      <c r="D14" s="6" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>B.3 CONDITIONS: all must be independently verified by the Chief AI Risk Officer before the first patient is scored in the relevant region</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="23" customHeight="1">
+      <c r="A17" s="49" t="inlineStr">
+        <is>
+          <t>Condition</t>
+        </is>
+      </c>
+      <c r="B17" s="49" t="inlineStr">
+        <is>
+          <t>Measurable threshold (evidence required)</t>
+        </is>
+      </c>
+      <c r="C17" s="49" t="inlineStr">
+        <is>
+          <t>Owner (Responsible / Accountable)</t>
+        </is>
+      </c>
+      <c r="D17" s="49" t="inlineStr">
+        <is>
+          <t>Timeline (T = decision date)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="128" customHeight="1">
+      <c r="A18" s="33" t="inlineStr">
+        <is>
+          <t>C1. Fix subgroup under-detection (RR-01, RR-12, RR-03)</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Retrain without region and insurance_type, plus label remediation from a re-adjudicated sample of Rural × Medicaid/Uninsured negatives (HbA1c / fasting glucose). On the held-out test set:
+(a) KRI-1 GREEN, ≤ 8 pp across all region × insurance cells with n_pos ≥ 20;
+(b) no powered cell has FNR above the FINDRISC baseline on the same cohort;
+(c) overall recall ≥ 0.74 and ROC AUC ≥ 0.80, so the aggregate does not regress;
+(d) subgroup-conditional SHAP for region/insurance pathways is |mean| &lt; 0.1 log-odds in every cell.</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>R: Head of Machine Learning. A: Chief Medical Officer (clinical acceptance)</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>Ablation result T+30 days (sprint). Full mitigation and re-audit T+90 days.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="68" customHeight="1">
+      <c r="A19" s="33" t="inlineStr">
+        <is>
+          <t>C2. Independent external validation (RR-01, RR-12)</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Validation by a party independent of the ML team, on held-out EU sites not used in training (e.g. the NL and SE launch centres). The cohort is sized by power calculation so every reported cell has n_pos ≥ 20. Results must meet the C1(a)-(c) thresholds, with Wilson 95% CIs reported for each cell.</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>R: external validation partner. A: Chief Medical Officer</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>Contract by T+30 days. Report by T+6 months.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="128" customHeight="1">
+      <c r="A20" s="33" t="inlineStr">
+        <is>
+          <t>C3. Lawful EU market route (RR-02, RR-03)</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Evidence required:
+- a formal MDR qualification and classification opinion;
+- QMS (ISO 13485 + ISO/IEC 42001 controls) and RMS (ISO 14971 / 23894) in place;
+- Annex IV / MDR technical file complete;
+- notified-body certificate issued, EU DoC signed, CE marking, EU database registration (Art. 49).</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>R: Head of Regulatory Affairs. A: Chief Compliance Officer</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>Opinion T+30 days. Notified body contracted T+60 days. Certificate before EU go-live (target T+8.5 months).
+CHECKPOINT T+6 months: if the stage-1 audit has not passed, the EU date moves (no launch without the certificate).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="143" customHeight="1">
+      <c r="A21" s="33" t="inlineStr">
+        <is>
+          <t>C4. Effective human oversight and transparency (RR-04)</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Evidence required:
+- IFU and clinician model card (D6) issued to every deployer;
+- dashboard shows validated top-3 clinical drivers plus a subgroup caution banner;
+- 100% of clinician users trained, with competency sign-off logged in the LMS;
+- per-tenant kill-switch and rollback tested in a drill, disabling scoring in ≤ 15 min;
+- 3-month shadow-mode pilot at ≥ 2 EU sites completed and used to baseline the KRI-2 thresholds.</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>R: Head of Product + Clinical Safety Officer. A: Chief Medical Officer</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>Build T+90 days. Shadow pilot T+5 to T+8 months. Complete before go-live.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="113" customHeight="1">
+      <c r="A22" s="33" t="inlineStr">
+        <is>
+          <t>C5. Data-protection basis (RR-08, RR-09, RR-10, RR-11)</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Evidence required:
+- DPIA signed by each EU hospital controller;
+- technical block, verified by test, preventing override or inference data from entering any training pipeline until a lawful basis is documented in an amended DPA (or Art. 26 joint-controller arrangement);
+- telemetry minimised to aggregates (k ≥ 20);
+- RoPA updated; retention schedule approved.</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>R: Data Protection Officer. A: Chief Compliance Officer</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>Retraining block T+30 days. DPIAs T+60 days. All other items before EU go-live.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="113" customHeight="1">
+      <c r="A23" s="33" t="inlineStr">
+        <is>
+          <t>C6. AI security hardening (RR-05, RR-06, RR-07)</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Evidence required:
+- model served from skops/ONNX, with Sigstore cosign signature and sha256 verified at load (the service refuses to start otherwise);
+- override quarantine plus a golden-set subgroup regression gate in CI;
+- reference-only API input with per-clinician quotas;
+- an independent AI red-team against the D3 TTPs, closing with 0 open Critical/High findings.</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>R: Head of ML Platform. A: Chief Information Security Officer</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>T+90 days. Red-team before go-live.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="98" customHeight="1">
+      <c r="A24" s="33" t="inlineStr">
+        <is>
+          <t>C7. US launch gate (separate) (RR-03, RR-10)</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>Evidence required:
+- US-representative validation (CA/MA/TX sites) meeting the C1(a)-(c) thresholds;
+- HIPAA BAAs with each IDN that permit any offshore processing;
+- intra-group subcontractor BAA;
+- DPF self-certification (or SCCs Module 4) for EU→US return flows;
+- Texas SB 1188 data-localisation assessment.</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>R: Chief Medical Officer + Data Protection Officer. A: Chief AI Risk Officer</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>Before US go-live. The Q4 2027 date stands only if met. Otherwise it is deferred.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="220" customHeight="1">
+      <c r="A25" s="26" t="inlineStr">
+        <is>
+          <t>B.4 POST-LAUNCH GOVERNANCE PLAN
+• PHASED ROLLOUT: 2 EU sites for the first 90 days, then the remaining sites, if KRI-1 is Green and no Red KRI occurred. The CAIRO re-confirms the decision at T(launch)+90 days.
+• KRI CADENCE (D7, computed by lab/kri.py):
+  - KRI-1 Subgroup FNR Drift monthly (rolling 12-month cohort with matured outcomes) and on every release in CI.
+  - KRI-2 Override Channel Health weekly.
+  - KRI-3 Inference Anomaly Rate daily, with real-time Red alerts.
+  - Any Red triggers the D7 escalation. KRI-1 Red → kill-switch to standard screening for affected tenants, plus an AI Act Art. 73 serious-incident assessment (report within 15 days if confirmed) and MDR vigilance.
+• RISK REGISTER (D5): the AI Review Board reviews Top-N risks monthly and the full register quarterly. Risks are re-scored as each condition closes, and new risks are added from incidents, red-team findings and KRI breaches.
+• MODEL CARD REFRESH (D6) TRIGGERS: any retrain or new model version, threshold change, new site or region, KRI Red, serious incident, a change in the data source or label definition, or 12 months since the last update.
+• RE-AUDIT: the D4 audit is re-run on every release candidate and quarterly on production outcomes. External re-validation is annual. The DPIA and post-market monitoring plan (Art. 72) are reviewed annually.</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n"/>
+      <c r="C25" s="5" t="n"/>
+      <c r="D25" s="6" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>SECTION C: RACI Sign-Off</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="43" t="inlineStr">
-        <is>
-          <t>Role</t>
-        </is>
-      </c>
-      <c r="B16" s="43" t="inlineStr">
-        <is>
-          <t>Name / Title</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="33" t="inlineStr">
-        <is>
-          <t>Decision authority</t>
-        </is>
-      </c>
-      <c r="B17" s="11" t="inlineStr">
-        <is>
-          <t>Chief AI Risk Officer</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="33" t="inlineStr">
-        <is>
-          <t>Required sign-off</t>
-        </is>
-      </c>
-      <c r="B18" s="11" t="inlineStr">
-        <is>
-          <t>AI Review Board chair</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="33" t="inlineStr">
-        <is>
-          <t>Required sign-off</t>
-        </is>
-      </c>
-      <c r="B19" s="11" t="inlineStr">
-        <is>
-          <t>Chief Compliance Officer</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="33" t="inlineStr">
-        <is>
-          <t>Informed</t>
-        </is>
-      </c>
-      <c r="B20" s="11" t="inlineStr">
-        <is>
-          <t>Chief Medical Officer (implementation owner: Conditions 1 and 2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="33" t="inlineStr">
-        <is>
-          <t>Informed</t>
-        </is>
-      </c>
-      <c r="B21" s="11" t="inlineStr">
-        <is>
-          <t>Chief Executive Officer (funding for 30-day remediation)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="33" t="inlineStr">
-        <is>
-          <t>Informed</t>
-        </is>
-      </c>
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t>Data Protection Officer (implementation owner: Condition 3)</t>
+    <row r="28" ht="23" customHeight="1">
+      <c r="A28" s="49" t="inlineStr">
+        <is>
+          <t>RACI role</t>
+        </is>
+      </c>
+      <c r="B28" s="49" t="inlineStr">
+        <is>
+          <t>Name / Title and scope</t>
+        </is>
+      </c>
+      <c r="C28" s="49" t="inlineStr">
+        <is>
+          <t>Signature</t>
+        </is>
+      </c>
+      <c r="D28" s="49" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="38" customHeight="1">
+      <c r="A29" s="33" t="inlineStr">
+        <is>
+          <t>A: Accountable / Decision authority</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>Chief AI Risk Officer. Owns this recommendation; verifies evidence for C1-C7; signs the final go-live confirmation for each region.</t>
+        </is>
+      </c>
+      <c r="C29" s="11" t="inlineStr">
+        <is>
+          <t>____________________</t>
+        </is>
+      </c>
+      <c r="D29" s="11" t="inlineStr">
+        <is>
+          <t>____ / ____ / ______</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="38" customHeight="1">
+      <c r="A30" s="33" t="inlineStr">
+        <is>
+          <t>A: Required sign-off</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>AI Review Board chair. Approves acceptance of residual risk against the Board risk appetite (B.2).</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>____________________</t>
+        </is>
+      </c>
+      <c r="D30" s="11" t="inlineStr">
+        <is>
+          <t>____ / ____ / ______</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="38" customHeight="1">
+      <c r="A31" s="33" t="inlineStr">
+        <is>
+          <t>A: Required sign-off</t>
+        </is>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>Chief Compliance Officer. Accountable for C3 (AI Act / MDR conformity) and C5 (data protection).</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>____________________</t>
+        </is>
+      </c>
+      <c r="D31" s="11" t="inlineStr">
+        <is>
+          <t>____ / ____ / ______</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="38" customHeight="1">
+      <c r="A32" s="33" t="inlineStr">
+        <is>
+          <t>R: Responsible</t>
+        </is>
+      </c>
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>Chief Medical Officer. Accountable for clinical acceptance in C1, C2 and C4; co-owner of C7.</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t>____________________</t>
+        </is>
+      </c>
+      <c r="D32" s="11" t="inlineStr">
+        <is>
+          <t>____ / ____ / ______</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="23" customHeight="1">
+      <c r="A33" s="33" t="inlineStr">
+        <is>
+          <t>R: Responsible</t>
+        </is>
+      </c>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>Head of Machine Learning. C1 retraining and mitigation; KRI-1 metric owner.</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="inlineStr">
+        <is>
+          <t>____________________</t>
+        </is>
+      </c>
+      <c r="D33" s="11" t="inlineStr">
+        <is>
+          <t>____ / ____ / ______</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="23" customHeight="1">
+      <c r="A34" s="33" t="inlineStr">
+        <is>
+          <t>R: Responsible</t>
+        </is>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>Data Protection Officer. C5; data-protection items of C7.</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>____________________</t>
+        </is>
+      </c>
+      <c r="D34" s="11" t="inlineStr">
+        <is>
+          <t>____ / ____ / ______</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="23" customHeight="1">
+      <c r="A35" s="33" t="inlineStr">
+        <is>
+          <t>R: Responsible</t>
+        </is>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>Chief Information Security Officer. C6; KRI-3 owner (with the SOC).</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="inlineStr">
+        <is>
+          <t>____________________</t>
+        </is>
+      </c>
+      <c r="D35" s="11" t="inlineStr">
+        <is>
+          <t>____ / ____ / ______</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="38" customHeight="1">
+      <c r="A36" s="33" t="inlineStr">
+        <is>
+          <t>C: Consulted</t>
+        </is>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>Clinical Safety Officer and deployer-hospital CMIOs (KRI-2, IFU usability); Head of Regulatory Affairs; notified body; external validation partner.</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>____________________</t>
+        </is>
+      </c>
+      <c r="D36" s="11" t="inlineStr">
+        <is>
+          <t>____ / ____ / ______</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="38" customHeight="1">
+      <c r="A37" s="33" t="inlineStr">
+        <is>
+          <t>I: Informed</t>
+        </is>
+      </c>
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>Chief Executive Officer. Funding for the 30-day sprint and the 9-month EU path; launch-date risk.</t>
+        </is>
+      </c>
+      <c r="C37" s="11" t="inlineStr">
+        <is>
+          <t>____________________</t>
+        </is>
+      </c>
+      <c r="D37" s="11" t="inlineStr">
+        <is>
+          <t>____ / ____ / ______</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="38" customHeight="1">
+      <c r="A38" s="33" t="inlineStr">
+        <is>
+          <t>I: Informed</t>
+        </is>
+      </c>
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>Board of Directors. Residual-risk position against appetite; the T+6-month checkpoint outcome.</t>
+        </is>
+      </c>
+      <c r="C38" s="11" t="inlineStr">
+        <is>
+          <t>____________________</t>
+        </is>
+      </c>
+      <c r="D38" s="11" t="inlineStr">
+        <is>
+          <t>____ / ____ / ______</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="38" customHeight="1">
+      <c r="A39" s="33" t="inlineStr">
+        <is>
+          <t>I: Informed</t>
+        </is>
+      </c>
+      <c r="B39" s="11" t="inlineStr">
+        <is>
+          <t>Hospital licensees (deployers). Launch conditions, IFU, and their Art. 26/27 deployer obligations (incl. FRIA for public bodies).</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="inlineStr">
+        <is>
+          <t>____________________</t>
+        </is>
+      </c>
+      <c r="D39" s="11" t="inlineStr">
+        <is>
+          <t>____ / ____ / ______</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A12:B12"/>
+  <mergeCells count="11">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="A14:D14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Tighten HealthGuard portfolio against the project rubric
- D1: paragraph-level Article citations throughout; blocker 3 quotes the
  risk-appetite statement
- D2: CPRA Sections for every stage; Section B opens with the transfer
  mechanism and TIA answer; Section C links each risk to its D5 row
- D3: strict AML.T#### IDs and the brief's exact component names
- Notebook: add 6b evidence cell behind every D4 narrative figure; fix
  stale expected-FNR comment; re-executed with all outputs
- Correct overstated training/test prevalence comparisons in D4-D6, D8
- D5: store Risk Scores as values so they are readable outside Excel
- Add pytest run log (34/34 passed) as audit evidence

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/04-secure-ai-deployment/project/starter/governance_portfolio.xlsx
+++ b/04-secure-ai-deployment/project/starter/governance_portfolio.xlsx
@@ -1023,7 +1023,7 @@
   <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
     <col width="48" customWidth="1" min="4" max="4"/>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="D6" s="26" t="inlineStr">
         <is>
-          <t>None of the Article 5(1) prohibited practices apply: (a) no subliminal/manipulative techniques. Output goes to a clinician, not the patient. (b) Does not exploit age, disability or socio-economic vulnerability to distort behaviour. It uses region/insurance_type as features, which is a fairness issue for Art. 10, not a prohibited practice. (c) Not social scoring. The score is used only in the clinical context it is produced for, and insurance underwriting / coverage decisions are contractually prohibited (that restriction must stay enforced; see Art. 9 row). (d) No criminal-offence risk prediction. (e) No facial-image scraping. (f) No emotion recognition at work/school. (g) No biometric categorisation; no biometric data is processed. (h) No real-time remote biometric ID. Conclusion: not prohibited. Proceed to Art. 6.</t>
+          <t>None of the Article 5(1) prohibited practices apply: (a) no subliminal/manipulative techniques. Output goes to a clinician, not the patient. (b) Does not exploit age, disability or socio-economic vulnerability to distort behaviour. It uses region/insurance_type as features, which is a fairness issue for Art. 10(2)(f)-(g), not a prohibited practice. (c) Not social scoring. The score is used only in the clinical context it is produced for, and insurance underwriting / coverage decisions are contractually prohibited (that restriction must stay enforced; see Art. 9(2)(b) row). (d) No criminal-offence risk prediction. (e) No facial-image scraping. (f) No emotion recognition at work/school. (g) No biometric categorisation; no biometric data is processed. (h) No real-time remote biometric ID. Conclusion: not prohibited. Proceed to Art. 6(1)-(3).</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
@@ -1131,12 +1131,12 @@
       </c>
       <c r="D7" s="26" t="inlineStr">
         <is>
-          <t>MDR 2017/745 is listed in Annex I Section A. MDR Art. 2(1) defines a medical device to include software intended for 'diagnosis, prevention, monitoring, prediction, prognosis' of disease. HealthGuard predicts an individual's T2D risk to drive preventive action (earlier labs, referral), so it meets the definition (MDCG 2019-11 decision steps: acts on patient-specific data, goes beyond storage/simple search, serves a medical purpose). Calling it 'decision support' does not exempt it. MDR Annex VIII Rule 11 classes software that provides information used for diagnostic/therapeutic decisions as at least Class IIa, which requires notified-body conformity assessment. Both limbs of Art. 6(1) are therefore met: (a) the AI system is itself a product covered by Annex I, and (b) it requires third-party conformity assessment. The brief's statement that HealthGuard is 'not a regulated medical device' is a regulatory-positioning gap that needs a formal MDR qualification opinion.</t>
+          <t>MDR 2017/745 is listed in Annex I, Section A, point 11. MDR Art. 2(1) defines a medical device to include software intended for 'diagnosis, prevention, monitoring, prediction, prognosis' of disease. HealthGuard predicts an individual's T2D risk to drive preventive action (earlier labs, referral), so it meets the definition (MDCG 2019-11 decision steps: acts on patient-specific data, goes beyond storage/simple search, serves a medical purpose). Calling it 'decision support' does not exempt it. MDR Annex VIII Rule 11 classes software that provides information used for diagnostic/therapeutic decisions as at least Class IIa, which requires notified-body conformity assessment. Both limbs of Art. 6(1) are therefore met: (a) the AI system is itself a product covered by Annex I, and (b) it requires third-party conformity assessment. The brief's statement that HealthGuard is 'not a regulated medical device' is a regulatory-positioning gap that needs a formal MDR qualification opinion.</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>Article 6(1)(a)-(b) + Annex I Section A (MDR 2017/745 Art. 2(1); Annex VIII Rule 11; MDCG 2019-11)</t>
+          <t>Article 6(1)(a)-(b) + Annex I, Section A, point 11 (MDR 2017/745 Art. 2(1); Annex VIII Rule 11; MDCG 2019-11)</t>
         </is>
       </c>
       <c r="F7" s="44" t="n"/>
@@ -1159,7 +1159,7 @@
       </c>
       <c r="D8" s="26" t="inlineStr">
         <is>
-          <t>Point 5(a) covers essential public services, explicitly including healthcare services, when an AI system is used by or on behalf of public authorities to evaluate eligibility. The EU launch sites are academic medical centres, several of them publicly run. If the score gates referral into a publicly funded diabetes-prevention programme, 5(a) is engaged. Point 5(c) (life/health-insurance risk pricing) would apply only under a prohibited non-intended use. Point 5(d) (emergency triage) is excluded because ED/ICU use is out of scope. The Art. 6(3) derogation is NOT available. The system profiles natural persons (GDPR Art. 4(4): predicting health), and the last sub-paragraph of Art. 6(3) makes any Annex III system that profiles high-risk. Annex III is a secondary basis; the classification does not depend on it.</t>
+          <t>Point 5(a) covers essential public services, explicitly including healthcare services, when an AI system is used by or on behalf of public authorities to evaluate eligibility. The EU launch sites are academic medical centres, several of them publicly run. If the score gates referral into a publicly funded diabetes-prevention programme, 5(a) is engaged. Point 5(c) (life/health-insurance risk pricing) would apply only under a prohibited non-intended use. Point 5(d) (emergency triage) is excluded because ED/ICU use is out of scope. The Art. 6(3) derogation is NOT available. The system profiles natural persons (GDPR Art. 4(4): predicting health), and the third subparagraph of Art. 6(3) makes any Annex III system that profiles high-risk. Annex III is a secondary basis; the classification does not depend on it.</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
@@ -1187,12 +1187,12 @@
       </c>
       <c r="D9" s="26" t="inlineStr">
         <is>
-          <t>HealthGuard is a high-risk AI system. Primary basis: Art. 6(1) + Annex I Section A, because it is medical-device software (MDR Class IIa under Rule 11) needing notified-body assessment. Secondary/alternative basis: Art. 6(2) + Annex III 5(a) where public hospitals use it to decide access to prevention services. It is not prohibited under Art. 5. Consequences for Klariova as provider: the Arts 9-15 requirements; a QMS (Art. 17); technical documentation (Art. 11/Annex IV); conformity assessment through the MDR notified body (Art. 43(3)); an EU declaration of conformity and CE marking (Arts 47-48); registration (Art. 49); post-market monitoring (Art. 72); and serious-incident reporting (Art. 73). Public-body deployers must also complete a FRIA (Art. 27). Timing: Art. 6(1) obligations apply from 2 Aug 2027 (Art. 113(c)), which falls inside the Q3 2027 EU launch window. Check whether the Digital Omnibus has changed this date, but plan as if the obligations apply at launch.</t>
+          <t>HealthGuard is a high-risk AI system. Primary basis: Art. 6(1) + Annex I Section A, because it is medical-device software (MDR Class IIa under Rule 11) needing notified-body assessment. Secondary/alternative basis: Art. 6(2) + Annex III 5(a) where public hospitals use it to decide access to prevention services. It is not prohibited under Art. 5(1). Consequences for Klariova as provider: the requirements of Arts 9(1), 10(1), 11(1), 12(1), 13(1), 14(1) and 15(1) (via Art. 16(a)); a QMS (Art. 17(1)); technical documentation (Art. 11(1)-(2)/Annex IV); conformity assessment through the MDR notified body (Art. 43(3)); an EU declaration of conformity and CE marking (Art. 47(1) and (3); Art. 48(3)); registration (Art. 49(1)); post-market monitoring (Art. 72(1)-(2)); and serious-incident reporting within 15 days (Art. 73(1)-(2)). Public-body deployers must also complete a FRIA (Art. 27(1)). Timing: Art. 6(1) obligations apply from 2 Aug 2027 (Art. 113, third paragraph, point (c)), which falls inside the Q3 2027 EU launch window. Check whether the Digital Omnibus has changed this date, but plan as if the obligations apply at launch.</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>Article 6(1) + Annex I Section A (MDR 2017/745); secondary: Article 6(2) + Annex III 5(a)</t>
+          <t>Article 6(1)(a)-(b) + Annex I, Section A, point 11 (MDR 2017/745); secondary: Article 6(2) + Annex III 5(a)</t>
         </is>
       </c>
       <c r="F9" s="44" t="n"/>
@@ -1239,7 +1239,7 @@
     <row r="14" ht="291" customHeight="1">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>Art. 9</t>
+          <t>Art. 9(1)-(2)</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
@@ -1265,7 +1265,7 @@
       <c r="F14" s="26" t="inlineStr">
         <is>
           <t>EVIDENCE OF GAP: This pre-launch GRC review is the first structured risk assessment. There is no documented, continuous lifecycle RMS. No acceptance thresholds were set in advance for testing (Art. 9(6)-(8)). Subgroup harm to vulnerable groups (Art. 9(9)) has not been evaluated. Foreseeable misuse (insurance underwriting, patient-facing use, ED/ICU use) is controlled only by contract terms.
-REMEDIATION: Adopt a written RMS procedure aligned to ISO 14971 (needed for MDR anyway) and ISO/IEC 23894, and make the D5 risk register its living output. Set pass/fail thresholds before testing, including a subgroup-FNR tolerance. Add technical misuse controls: API scoping, tenant blocks for ED/ICU, and no patient-facing endpoint. Feed post-market monitoring (Art. 72) and the D7 KRIs back into the RMS on a set review cadence.
+REMEDIATION: Adopt a written RMS procedure aligned to ISO 14971 (needed for MDR anyway) and ISO/IEC 23894, and make the D5 risk register its living output. Set pass/fail thresholds before testing, including a subgroup-FNR tolerance. Add technical misuse controls: API scoping, tenant blocks for ED/ICU, and no patient-facing endpoint. Feed post-market monitoring (Art. 72(1)-(2)) and the D7 KRIs back into the RMS on a set review cadence.
 PROOF: an approved RMS procedure, a risk register with an owner for each risk, and residual-risk acceptance signed by the AI Review Board.</t>
         </is>
       </c>
@@ -1273,7 +1273,7 @@
     <row r="15" ht="381" customHeight="1">
       <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>Art. 10</t>
+          <t>Art. 10(2)-(4)</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="F15" s="26" t="inlineStr">
         <is>
-          <t>EVIDENCE OF GAP: (1) The training data is not representative. It comes only from IE+DE, but the system will also be deployed in the US (CA/MA/TX). (2) Label bias: under-served patients are under-diagnosed in Source 1, and the synthetic Source 2 reproduces that pattern rather than correcting it. (3) region and insurance_type are model features. insurance_type comes from billing and can be stale (a data-quality error), and Rural patients are 45% Medicaid, so the field acts as a proxy. (4) Our own check (test n=3,000, threshold 0.26) found FNR of 37.8% for Rural vs 22.7% for Urban (1.7x), 37.5% for Uninsured and 31.3% for Medicaid vs 20.8% for Medicare, and 48.9% for ages 21-35. (5) Manifest mismatch: train.csv has 12,000 rows, against the '~8,000' in the brief. No bias examination as required by Art. 10(2)(f)-(g) is on file.
+          <t>EVIDENCE OF GAP: (1) The training data is not representative (Art. 10(3)) of the geographical setting of use (Art. 10(4)). It comes only from IE+DE, but the system will also be deployed in the US (CA/MA/TX). (2) Label bias: under-served patients are under-diagnosed in Source 1, and the synthetic Source 2 reproduces that pattern rather than correcting it. (3) region and insurance_type are model features. insurance_type comes from billing and can be stale (a data-quality error), and Rural patients are 45% Medicaid, so the field acts as a proxy. (4) Our own check (test n=3,000, threshold 0.26) found FNR of 37.8% for Rural vs 22.7% for Urban (1.7x), 37.5% for Uninsured and 31.3% for Medicaid vs 20.8% for Medicare, and 48.9% for ages 21-35. (5) Manifest mismatch: train.csv has 12,000 rows, against the '~8,000' in the brief. No bias examination as required by Art. 10(2)(f)-(g) is on file.
 REMEDIATION: Document data governance per Art. 10(2): origin, labelling and assumptions. Run a bias examination and mitigation: drop region/insurance_type or justify them, reweight or adjust thresholds per group, and audit labels. Source real-world rural and under-served records. Validate on a US-representative cohort before the US launch. Add freshness and validation checks on insurance_type. Reconcile the training manifest hash with the actual dataset.</t>
         </is>
       </c>
@@ -1306,7 +1306,7 @@
     <row r="16" ht="321" customHeight="1">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>Art. 10</t>
+          <t>Art. 10(5)</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
@@ -1332,7 +1332,7 @@
       <c r="F16" s="26" t="inlineStr">
         <is>
           <t>EVIDENCE OF COMPLIANCE: Source 1 has explicit opt-in for secondary use under the DPA, and hospitals manage consent.
-GAPS: No DPIA (GDPR Art. 35) is referenced. The Art. 10(5) safeguards for using special-category data in bias work are not documented: strict necessity, pseudonymisation, access restriction, deletion once correction is done, and records of processing. The synthetic Source 2 was generated from real patients, and nobody has tested it for memorisation or re-identification. The Model Registry keeps every training dataset indefinitely (a minimisation and storage-limitation issue). US inference telemetry goes to Frankfurt without a documented transfer assessment.
+GAPS: No DPIA (GDPR Art. 35(1), 35(3)(b)) is referenced. The Art. 10(5) safeguards for using special-category data in bias work are not documented: strict necessity, pseudonymisation, access restriction, deletion once correction is done, and records of processing. The synthetic Source 2 was generated from real patients, and nobody has tested it for memorisation or re-identification. The Model Registry keeps every training dataset indefinitely (a minimisation and storage-limitation issue). US inference telemetry goes to Frankfurt without a documented transfer assessment.
 REMEDIATION: Complete a DPIA and record the GDPR Art. 9(2)(h)/(j) legal basis. Document the Art. 10(5)(a)-(f) safeguards. Run membership-inference and nearest-neighbour privacy tests on the synthetic data. Set a retention and deletion schedule and RBAC for training data in the registry. Data-map the telemetry flow and minimise or pseudonymise it (see D2).</t>
         </is>
       </c>
@@ -1340,7 +1340,7 @@
     <row r="17" ht="336" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>Art. 11</t>
+          <t>Art. 11(1)</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
@@ -1382,7 +1382,7 @@
     <row r="18" ht="261" customHeight="1">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>Art. 12</t>
+          <t>Art. 12(1)-(2)</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
@@ -1407,7 +1407,7 @@
       </c>
       <c r="F18" s="26" t="inlineStr">
         <is>
-          <t>EVIDENCE OF COMPLIANCE: Component 6 logs every request, response, clinician override and drift metric, with 7-year retention. That exceeds the Art. 19 minimum of 6 months and supports Art. 72.
+          <t>EVIDENCE OF COMPLIANCE: Component 6 logs every request, response, clinician override and drift metric, with 7-year retention. That exceeds the Art. 19(1) minimum of 6 months and supports Art. 72(2).
 GAPS: The log schema is not mapped to Art. 12(2) (identifying risk situations or substantial modifications, post-market monitoring, deployer monitoring). Per-inference tagging of model version and clinician ID is unconfirmed. Logs have no integrity or tamper-evidence controls. Keeping identifiable feature vectors for 7 years conflicts with GDPR minimisation unless it is justified and the data is pseudonymised.
 REMEDIATION: Map log fields to Art. 12(2)(a)-(c). Stamp each record with model version, threshold and clinician. Use WORM or hash-chained storage with restricted access. Pseudonymise patient IDs in monitoring logs. Document the retention justification in the DPIA.</t>
         </is>
@@ -1416,7 +1416,7 @@
     <row r="19" ht="306" customHeight="1">
       <c r="A19" s="11" t="inlineStr">
         <is>
-          <t>Art. 13</t>
+          <t>Art. 13(1)-(3)</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="20" ht="261" customHeight="1">
       <c r="A20" s="11" t="inlineStr">
         <is>
-          <t>Art. 14</t>
+          <t>Art. 14(1), (4)(a)-(c)</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
@@ -1482,7 +1482,7 @@
       <c r="F20" s="26" t="inlineStr">
         <is>
           <t>EVIDENCE OF COMPLIANCE: A clinician reviews every prediction, and the dashboard has a sign-off step.
-GAPS: The Art. 14(4)(a)-(c) measures are missing: no clinician training on capabilities and limits, no automation-bias controls, and no display of uncertainty. The main failure mode is a false 'not high-risk' result. Clinicians rarely question a reassuring score, so the human check is weakest exactly where subgroup FNR is highest. Deployer guidance under Art. 26 (competent oversight staff) has not been issued.
+GAPS: The Art. 14(4)(a)-(c) measures are missing: no clinician training on capabilities and limits, no automation-bias controls, and no display of uncertainty. The main failure mode is a false 'not high-risk' result. Clinicians rarely question a reassuring score, so the human check is weakest exactly where subgroup FNR is highest. Deployer guidance under Art. 26(2) (competent oversight staff) has not been issued.
 REMEDIATION: Make clinician training mandatory, with sign-off. Show a calibrated probability band and a borderline-zone flag instead of just a binary label. Add subgroup caution prompts, and prompt clinicians to apply standard screening criteria (e.g., ADA/FINDRISC) to negative results. Track override and concordance rates by subgroup as a KRI. Give deployers an oversight SOP.</t>
         </is>
       </c>
@@ -1490,7 +1490,7 @@
     <row r="21" ht="216" customHeight="1">
       <c r="A21" s="11" t="inlineStr">
         <is>
-          <t>Art. 14</t>
+          <t>Art. 14(4)(d)-(e)</t>
         </is>
       </c>
       <c r="B21" s="11" t="inlineStr">
@@ -1516,7 +1516,7 @@
       <c r="F21" s="26" t="inlineStr">
         <is>
           <t>EVIDENCE OF COMPLIANCE: Clinicians can disagree with the score, and overrides are logged (Art. 14(4)(d)).
-GAPS: There is no documented 'stop' / suspend capability for the deployer or provider (Art. 14(4)(e)), such as a kill-switch per hospital or per model version. Override reasons are not captured in a structured form. Overrides flow straight into retraining data without review, which creates a feedback loop and a poisoning path (see Art. 15).
+GAPS: There is no documented 'stop' / suspend capability for the deployer or provider (Art. 14(4)(e)), such as a kill-switch per hospital or per model version. Override reasons are not captured in a structured form. Overrides flow straight into retraining data without review, which creates a feedback loop and a poisoning path (see Art. 15(4)).
 REMEDIATION: Build and test a per-tenant kill-switch with rollback to the previous model version. Add structured override-reason codes. Put a human-reviewed quarantine step in front of any override data used for retraining. Show the evidence in a runbook and a tested drill.</t>
         </is>
       </c>
@@ -1524,7 +1524,7 @@
     <row r="22" ht="276" customHeight="1">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>Art. 15</t>
+          <t>Art. 15(1), (3)</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
@@ -1550,7 +1550,7 @@
       <c r="F22" s="26" t="inlineStr">
         <is>
           <t>EVIDENCE: Overall performance at threshold 0.26 is ROC AUC 0.812, recall 0.744 and precision 0.476. That is reasonable for a sensitivity-tuned screening aid.
-GAPS: Accuracy is not appropriate for every group. Rural FNR is 37.8% and Uninsured FNR is 37.5%, against 22.7% for Urban and 20.8% for Medicare. Nothing compares performance with standard of care (e.g., FINDRISC or the ADA risk test), so the risk-appetite test ('not materially worse than standard of care') cannot be shown. No external validation has been done (brief Section 8). Accuracy levels are not declared in the IFU (Art. 15(3)).
+GAPS: Accuracy is not appropriate for every group (Art. 15(1)). Rural FNR is 37.8% and Uninsured FNR is 37.5%, against 22.7% for Urban and 20.8% for Medicare. Nothing compares performance with standard of care (e.g., FINDRISC or the ADA risk test), so the risk-appetite test ('not materially worse than standard of care') cannot be shown. No external validation has been done (brief Section 8). Accuracy levels are not declared in the IFU (Art. 15(3)).
 REMEDIATION: Agree a subgroup-FNR acceptance criterion with the AI Review Board, e.g., no group's FNR worse than standard of care and a max/min FNR ratio of 1.25x or less. Re-validate after mitigation. Commission independent external validation on held-out EU sites, and on US sites before the US launch. Declare the metrics in the IFU.</t>
         </is>
       </c>
@@ -1558,7 +1558,7 @@
     <row r="23" ht="276" customHeight="1">
       <c r="A23" s="11" t="inlineStr">
         <is>
-          <t>Art. 15</t>
+          <t>Art. 15(1), (4)</t>
         </is>
       </c>
       <c r="B23" s="11" t="inlineStr">
@@ -1592,7 +1592,7 @@
     <row r="24" ht="291" customHeight="1">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>Art. 15</t>
+          <t>Art. 15(1), (5)</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
@@ -1618,7 +1618,7 @@
       <c r="F24" s="26" t="inlineStr">
         <is>
           <t>EVIDENCE OF COMPLIANCE: mTLS at the hospital edge, and rate limiting at 200 requests/min per hospital.
-GAPS: The model ships as a joblib pickle. Loading it can execute arbitrary code, and nothing checks its integrity (a model-tampering / supply-chain risk). The Model Registry holds every training dataset, which makes it a high-value target. Unvetted override feedback is a data-poisoning path (ATLAS AML.T0020). The inference API allows high-volume querying, which enables model extraction or inversion. No AI-specific pen test or red-team exercise has been done.
+GAPS against Art. 15(5) (which names data poisoning, model poisoning, adversarial examples and confidentiality attacks): The model ships as a joblib pickle. Loading it can execute arbitrary code, and nothing checks its integrity (a model-tampering / supply-chain risk). The Model Registry holds every training dataset, which makes it a high-value target. Unvetted override feedback is a data-poisoning path (ATLAS AML.T0020). The inference API allows high-volume querying, which enables model extraction or inversion. No AI-specific pen test or red-team exercise has been done.
 REMEDIATION: Sign artifacts and verify their hash at load time, or move to a safe format (skops/ONNX). Apply least-privilege RBAC and audit logging to the registry, and encrypt training data. Add poisoning controls on feedback data. Detect anomalous query patterns and tighten per-client quotas. Before launch, run an AI red-team exercise against the D3 ATLAS TTPs, and produce an SBOM for dependencies.</t>
         </is>
       </c>
@@ -1630,19 +1630,19 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="355" customHeight="1">
+    <row r="27" ht="370" customHeight="1">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>1) SUBGROUP UNDER-DETECTION (Art. 10 data governance + Art. 15 accuracy). CRITICAL, LAUNCH-BLOCKING.
+          <t>1) SUBGROUP UNDER-DETECTION (Art. 10(2)(f)-(g), 10(3)-(4) data governance + Art. 15(1), 15(3) accuracy). CRITICAL, LAUNCH-BLOCKING.
 Why it blocks: Patient-safety appetite is LOW. The Board will not deploy a system whose 'foreseeable failure modes can produce a missed diagnosis or delayed referral for any identifiable patient subgroup at a rate materially worse than standard of care.' HealthGuard misses 37.8% of true diabetes cases in Rural patients and 37.5% in Uninsured patients, against about 21-23% for Urban and Medicare patients. The cause is identifiable: region and insurance_type act as socio-economic proxies, and the training labels carry historical under-diagnosis that the synthetic data copies. Human oversight cannot make up for this, because clinicians are least likely to question a reassuring 'not high-risk' result.
 To clear: Mitigate the bias (remove or justify the proxy features, reweight or set per-group thresholds, audit the labels). Then show through independent external validation that every subgroup's FNR is within the Board-approved tolerance (e.g., a max/min ratio of 1.25x or less) and no worse than a standard-of-care baseline such as FINDRISC. A US-representative validation is a separate gate before the US launch.
-2) NO LAWFUL ROUTE TO MARKET: MDR qualification, conformity assessment and technical documentation (Art. 6(1), 9, 11, 17, 43). CRITICAL, LAUNCH-BLOCKING.
+2) NO LAWFUL ROUTE TO MARKET: MDR qualification, conformity assessment and technical documentation (Art. 6(1), 9(1), 11(1), 17(1), 43(3)). CRITICAL, LAUNCH-BLOCKING.
 Why it blocks: Appetite for regulatory non-compliance is LOW. The Board 'will not deploy a system that we know to be non-compliant.' HealthGuard is high-risk via Annex I/MDR. It cannot be placed on the EU market without a QMS, an Annex IV technical file, a documented RMS, notified-body conformity assessment, a declaration of conformity, CE marking and EU database registration. The partial-compliance exception does not apply here. No compensating control can stand in for a missing conformity assessment, and launching without one is a regulator-reportable event (reputational appetite: LOW).
 To clear: Obtain a formal MDR qualification and classification opinion (expect Class IIa) and engage a notified body. Complete the Annex IV/MDR technical file, the RMS and the QMS. Pass conformity assessment, then sign the DoC and register the system before the first EU patient is scored.
-3) TRANSPARENCY AND HUMAN OVERSIGHT DO NOT WORK (Art. 13 + Art. 14). HIGH; BLOCKS LAUNCH BECAUSE IT IS THE COMPENSATING CONTROL.
-Why it blocks: The Board's 'partial compliance with an approved compensating control' route would rely on clinician review to accept any residual subgroup risk. Today that control is not effective. Clinicians get no IFU and no subgroup performance figures or limitations, only a rough explanation. They have no training and no safeguards against automation bias, and overrides go straight into retraining.
+3) TRANSPARENCY AND HUMAN OVERSIGHT DO NOT WORK (Art. 13(1), 13(3)(b) + Art. 14(1), 14(4)(b), 14(4)(e)). HIGH; BLOCKS LAUNCH BECAUSE IT IS THE COMPENSATING CONTROL.
+Why it blocks: The risk-appetite statement (brief §7) allows documented partial compliance 'only when the gap has a remediation plan and an approved compensating control', and sets patient-safety appetite at LOW. Clinician review is the compensating control the Board would rely on to accept any residual subgroup risk from gap 1. Today that control is not effective. Clinicians get no IFU and no subgroup performance figures or limitations, only a rough explanation. They have no training and no safeguards against automation bias, and overrides go straight into retraining.
 To clear: Issue an IFU and model card that disclose subgroup FNR and limitations. Ship validated per-patient explanations and subgroup caution flags, and deliver mandatory clinician training. Track override and concordance KRIs by subgroup. Have a tested kill-switch and rollback, and a review gate before override data is used for retraining.
-Next tier (must-fix, but can be fixed after launch under a dated plan): Art. 15 cybersecurity (unsigned pickle artifact, registry access, poisoning via feedback), Art. 10(5)/GDPR safeguards (DPIA, privacy testing of the synthetic data, cross-border telemetry), and Art. 12 log integrity.</t>
+Next tier (must-fix, but can be fixed after launch under a dated plan): Art. 15(5) cybersecurity (unsigned pickle artifact, registry access, poisoning via feedback), Art. 10(5)/GDPR safeguards (DPIA, privacy testing of the synthetic data, cross-border telemetry), and Art. 12(1)-(2) log integrity.</t>
         </is>
       </c>
       <c r="B27" s="5" t="n"/>
@@ -1816,7 +1816,7 @@
       </c>
       <c r="E7" s="26" t="inlineStr">
         <is>
-          <t>PHI is exempt (§1798.146), so the HIPAA Security Rule applies: transmission security §164.312(e)(1) and audit controls §164.312(b).
+          <t>PHI is exempt (§1798.146(a)(1)(A)), so the HIPAA Security Rule applies: transmission security §164.312(e)(1) and audit controls §164.312(b).
 For any non-exempt PI: reasonable security (§1798.100(e)), the private right of action for breach (§1798.150), and minimisation (§1798.100(c)).</t>
         </is>
       </c>
@@ -1861,7 +1861,7 @@
       </c>
       <c r="E8" s="26" t="inlineStr">
         <is>
-          <t>PHI is exempt (§1798.146), so the HIPAA minimum-necessary standard applies (§164.502(b)).
+          <t>PHI is exempt (§1798.146(a)(1)(A)), so the HIPAA minimum-necessary standard applies (§164.502(b)).
 For non-exempt PI: processing must be reasonably necessary and proportionate (§1798.100(c)), consumers have a right to correct (§1798.106), and health data is sensitive PI (§1798.140(ae)).</t>
         </is>
       </c>
@@ -1877,7 +1877,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="171" customHeight="1">
+    <row r="9" ht="216" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
         <is>
           <t>4</t>
@@ -1903,8 +1903,10 @@
       </c>
       <c r="E9" s="26" t="inlineStr">
         <is>
-          <t>PHI is exempt, so HIPAA applies.
-For any non-exempt PI, the CCPA regulations apply from 2027. ADMT rules (11 CCR §7200 et seq.; 'significant decisions' include healthcare services) require a pre-use notice, opt-out or human appeal, and access. A risk assessment is also required (11 CCR §7150).</t>
+          <t>Patient PHI is exempt from CCPA/CPRA (Civ. Code §1798.146(a)(1)(A)), so HIPAA applies.
+For any non-exempt PI (e.g. scores tied to clinician users, or non-PHI fields):
+- health data is sensitive PI (§1798.140(ae)), with a right to limit its use (§1798.121(a));
+- §1798.185(a)(15)-(16) mandates the CPPA regulations on risk assessments and on automated decision-making technology (ADMT). Those are the risk-assessment rules (11 CCR §7150) and the ADMT rules (11 CCR §7200 et seq.), which treat healthcare services as 'significant decisions'. They apply from 2027 and require a pre-use notice, opt-out or human appeal, and access.</t>
         </is>
       </c>
       <c r="F9" s="26" t="inlineStr">
@@ -2104,10 +2106,15 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="190" customHeight="1">
+    <row r="16" ht="295" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>1) WHAT FLOWS. For drift monitoring, inference request metadata from AWS US-East goes to the Frankfurt data centre: hospital ID, timestamps, model version, request/patient IDs, feature-value distributions and latency. Klariova also holds the US prediction database that maps request IDs to patients. That makes this metadata pseudonymised personal data, and because it describes clinical feature values it is health data (GDPR Arts 4(1), 4(5), 4(15); Recital 26). Not being 'full patient records' does not make it anonymous. Klariova can re-identify it, so the SRB v EDPS (C-413/23 P) recipient-perspective argument does not help.
+          <t>BOTTOM LINE for the US→EU telemetry flow.
+- MECHANISM: the EU-US Data Privacy Framework ADEQUACY decision (GDPR Art. 45(1), (3)), which needs Klariova Health Inc. to self-certify. Fallback: the 2021 STANDARD CONTRACTUAL CLAUSES, Module 4, in an intra-group agreement (Art. 46(2)(c); Decision 2021/914). BCRs (Art. 47) are not used, because they are disproportionate for a group of two entities.
+- TIA: REQUIRED for any flow that relies on SCCs, which here means the EU→US return legs, and especially where US data is pooled with EU data. NOT legally required for the inbound US→EU leg. We will document a short TIA anyway.
+- RoPA: a new Art. 30 entry is needed (point 7).
+Detail follows.
+1) WHAT FLOWS. For drift monitoring, inference request metadata from AWS US-East goes to the Frankfurt data centre: hospital ID, timestamps, model version, request/patient IDs, feature-value distributions and latency. Klariova also holds the US prediction database that maps request IDs to patients. That makes this metadata pseudonymised personal data, and because it describes clinical feature values it is health data (GDPR Arts 4(1), 4(5), 4(15); Recital 26). Not being 'full patient records' does not make it anonymous. Klariova can re-identify it, so the SRB v EDPS (C-413/23 P) recipient-perspective argument does not help.
 2) IS IT A GDPR TRANSFER? The US→EU leg is NOT a Chapter V transfer, because Chapter V regulates exports OUT of the EEA. But once the data is in Frankfurt it is processed in the context of Klariova's EU establishment, so GDPR applies in full (Art. 3(1)): processor terms, Art. 32 security, Art. 30 records, Art. 33 breach handling, and requests from US data subjects. Chapter V IS triggered by the return legs: drift alerts or reports sent to the US, monitoring dashboards opened from Boston, remote access to Frankfurt by US-subsidiary engineers, and any onward sharing with US hospitals.
 3) MECHANISM. Primary: the EU-US Data Privacy Framework adequacy decision (Art. 45; in force since 10 Jul 2023; upheld by the General Court in Latombe, T-553/23, Sep 2025). This requires Klariova Health Inc. to self-certify with the US Dept. of Commerce. Fallback, given the political risk to the DPF: 2021 SCCs (Decision 2021/914) in an intra-group data-transfer agreement. Use Module 4 (EU processor → non-EU controller) where Frankfurt sends US hospitals' own data back to them. Use Module 1/2 where Klariova Ltd, as controller for AI Act Art. 72 post-market monitoring, shares data with Klariova Inc. BCRs are disproportionate for a group of two entities.
 4) TRANSFER IMPACT ASSESSMENT. NOT legally required for the US→EU leg, because there is no Chapter V transfer. REQUIRED (Schrems II C-311/18; SCC Clause 14; EDPB Recommendations 01/2020) for any EU→US return that relies on SCCs. Under Module 4, Clause 14 applies only if the EU processor combines the US data with data it collected in the EU, and pooled EU+US drift monitoring will do that. No TIA is needed while relying on DPF adequacy. Recommendation: document a short TIA now anyway, relying on EO 14086 and the Data Protection Review Court, so the SCC fallback is ready the day the DPF falls.</t>
@@ -2154,19 +2161,19 @@
       <c r="A19" s="26" t="inlineStr">
         <is>
           <t>Ranked by suggested D5 score (Likelihood × Impact, 1-5 scale). Each is carried into D5 as a row.
-C1. SECONDARY USE OF CLINICAL DATA FOR RETRAINING WITHOUT A LAWFUL BASIS (stages 6-7). L4 × I4 = 16. Privacy/Regulatory · Govern.
+C1 → D5 RR-08. SECONDARY USE OF CLINICAL DATA FOR RETRAINING WITHOUT A LAWFUL BASIS (stages 6-7). L4 × I4 = 16. Privacy/Regulatory · Govern.
 Inference outputs and clinician overrides go into the Model Registry for retraining. That is a new purpose, outside Klariova's processor mandate (GDPR Arts 5(1)(b), 6(4), 9(2)(j), 28(10)) and probably outside HIPAA BA permitted uses. It would make Klariova a controller with no lawful basis for EU and US data alike.
 Control: a formal role decision and DPA/BAA amendment (or an Art. 26 joint-controller arrangement); an Art. 6(4) / 9(2)(j) + 89(1) assessment; quarantine all override data until a basis exists.
-C2. INACCURATE AND UNNECESSARY SOCIO-ECONOMIC DATA IN HEALTH PROFILING (stage 3). L4 × I4 = 16. Fairness/Privacy · Map/Measure.
+C2 → D5 RR-01 (re-scored 5 × 5 = 25 once combined with the D4 evidence) and RR-03. INACCURATE AND UNNECESSARY SOCIO-ECONOMIC DATA IN HEALTH PROFILING (stage 3). L4 × I4 = 16. Fairness/Privacy · Map/Measure.
 insurance_type (stale billing data) and region are processed with no clinical necessity, and they drive the subgroup FNR gap (Rural 37.8%, Uninsured 37.5%). This breaches the GDPR principles of fairness, minimisation and accuracy (Art. 5(1)(a), (c), (d)) and data protection by design (Art. 25). It is the same root cause as D1 gap #1.
 Control: remove both features or justify them in the DPIA with a necessity test; add a freshness check and an 'unknown' fallback; re-run the D4 audit.
-C3. NO DPIA AND NO PROFILING SAFEGUARDS (stages 1, 4). L5 × I3 = 15. Regulatory · Govern.
+C3 → D5 RR-09. NO DPIA AND NO PROFILING SAFEGUARDS (stages 1, 4). L5 × I3 = 15. Regulatory · Govern.
 Large-scale profiling on health data makes a DPIA mandatory (Art. 35(3)(a)), and none exists. Patient notices do not explain the logic (Arts 13(2)(f), 14(2)(g)), and nothing shows the human review would satisfy SCHUFA (C-634/21). In California, any non-PHI data is caught by the CCPA risk-assessment and ADMT regulations (11 CCR §7150, §7200).
 Control: a DPIA written by Klariova and adopted by each hospital before go-live; plain-language logic notice; override and concordance KRI as evidence of meaningful review.
-C4. US→EU TELEMETRY TREATED AS NON-PERSONAL AND UNGOVERNED (stage 8). L3 × I4 = 12. Privacy · Govern.
+C4 → D5 RR-10. US→EU TELEMETRY TREATED AS NON-PERSONAL AND UNGOVERNED (stage 8). L3 × I4 = 12. Privacy · Govern.
 The metadata can be linked back to patients and is derived from health data. GDPR applies in Frankfurt (Art. 3(1)). Return flows to the US have no DPF certification or SCCs, there is no HIPAA subcontractor BAA between the group companies, and the flow is not in the RoPA. Exposure: a GDPR Art. 83(5) fine of up to 4% of turnover, plus a HIPAA violation under the US hospitals' BAAs.
 Control: aggregate-only telemetry; DPF self-certification plus SCCs Module 4 as fallback; a short TIA; a subcontractor BAA; a RoPA entry.
-C5. OVER-COLLECTION AND OVER-RETENTION CONCENTRATE BREACH IMPACT (stages 2, 5, 7). L4 × I3 = 12. Privacy/Security · Manage.
+C5 → D5 RR-11. OVER-COLLECTION AND OVER-RETENTION CONCENTRATE BREACH IMPACT (stages 2, 5, 7). L4 × I3 = 12. Privacy/Security · Manage.
 Hospitals push full FHIR records. Identifiable feature vectors are kept for 7 years, and every training dataset ever used sits indefinitely in the registry (GDPR Art. 5(1)(c), (e) and Art. 32; CPRA §1798.100(a)(3), (c); breach liability under §1798.150).
 Control: an allow-list of FHIR fields; a pseudonymised monitoring store; a documented retention schedule; KMS encryption, RBAC and access logging on the prediction DB and registry.</t>
         </is>
@@ -2249,7 +2256,7 @@
 C3 Model Inference API (FastAPI + scikit-learn, loads a joblib pickle). Surface: accepts a raw feature vector, returns a full-precision probability, and allows 200 req/min per hospital (about 288k/day). Threats: query-based extraction, membership inference or inversion, adversarial inputs. Deserialising a pickle on load means arbitrary code execution.
 C4 Clinician-Facing Dashboard. Surface: web app, clinician credentials (phishing is the leading healthcare breach vector), override capture. Threats: account takeover, malicious or systematically biased overrides that become training labels.
 C5 Model Registry. Surface: every model artifact, training-data manifest and training dataset ever used, plus override feedback. It is the highest-value target. Threats: artifact substitution (supply chain), training-data poisoning, bulk exfiltration of patient training data.
-C6 Logging &amp; Monitoring. Surface: 7 years of inference logs with patient IDs; cross-border US→EU telemetry (D2 stage 8). Threats: log tampering to hide an attack, exfiltration, poisoning of drift baselines so real drift does not alert.
+C6 Logging and Monitoring Infrastructure. Surface: 7 years of inference logs with patient IDs; cross-border US→EU telemetry (D2 stage 8). Threats: log tampering to hide an attack, exfiltration, poisoning of drift baselines so real drift does not alert.
 → Where the surface is largest: the C4→C5 feedback loop (untrusted labels flow straight into training), the C5→C3 artifact path (unsigned pickle is loaded in production), and C3 API exposure (raw vectors in, raw probabilities out). The three TTPs below are chosen from these.</t>
         </is>
       </c>
@@ -2329,7 +2336,7 @@
       </c>
       <c r="D9" s="26" t="inlineStr">
         <is>
-          <t>C4 Clinician Dashboard → C5 Model Registry (override feedback loop). Secondary: Source 2 synthetic-data generator.</t>
+          <t>Component 4 — Clinician-Facing Dashboard → Component 5 — Model Registry (override feedback loop). Secondary: the Source 2 synthetic-data generator.</t>
         </is>
       </c>
       <c r="E9" s="26" t="inlineStr">
@@ -2346,7 +2353,7 @@
       <c r="F9" s="26" t="inlineStr">
         <is>
           <t>Targets the integrity of the training pipeline (ATLAS AML.M0007 Sanitize Training Data, AML.M0025 Maintain AI Dataset Provenance, AML.M0008 Validate AI Model):
-1. OVERRIDE QUARANTINE: overrides go to a separate staging table and are never used for training until a second clinician adjudicates a stratified sample. Structured reason codes are mandatory.
+1. OVERRIDE QUARANTINE: overrides go to a separate staging table and are never used for training until a second clinician adjudicates a stratified sample (dual control). Structured reason codes are mandatory.
 2. CONTRIBUTION CAPS AND ANOMALY CHECKS: cap the number of override labels any one clinician or site can contribute per release. Run per-clinician override-rate z-scores by subgroup, and screen for label errors with cleanlab (confident learning) before training.
 3. SUBGROUP REGRESSION GATE in CI: score each candidate model on a frozen, clinician-adjudicated golden test set that only the release pipeline can read. Block promotion if any region, insurance or age subgroup's FNR rises by more than 2 percentage points, or breaches the D7 KRI threshold (lab/kri.py).
 4. LINEAGE: version the training data in DVC or lakeFS, with the sha256 manifest signed and recorded in the registry, so a poisoned batch can be traced and rolled back.</t>
@@ -2371,18 +2378,18 @@
       </c>
       <c r="B10" s="26" t="inlineStr">
         <is>
-          <t>AML.T0010.003</t>
+          <t>AML.T0010</t>
         </is>
       </c>
       <c r="C10" s="26" t="inlineStr">
         <is>
-          <t>AI Supply Chain Compromise: Model
+          <t>AI Supply Chain Compromise (sub-technique AML.T0010.003: Model)
 (related: AML.T0011.000 User Execution: Unsafe AI Artifacts; AML.T0018 Manipulate AI Model)</t>
         </is>
       </c>
       <c r="D10" s="26" t="inlineStr">
         <is>
-          <t>C5 Model Registry → C3 Model Inference API (loading the joblib artifact).</t>
+          <t>Component 5 — Model Registry → Component 3 — Model Inference API (loading the joblib model artifact).</t>
         </is>
       </c>
       <c r="E10" s="26" t="inlineStr">
@@ -2436,7 +2443,7 @@
       </c>
       <c r="D11" s="26" t="inlineStr">
         <is>
-          <t>C3 Model Inference API (and the hospital-edge mTLS client certificates in C1/C3).</t>
+          <t>Component 3 — Model Inference API (reached with the hospital-edge mTLS client certificates used by Component 1 — Data Ingestion Pipeline).</t>
         </is>
       </c>
       <c r="E11" s="26" t="inlineStr">
@@ -3308,13 +3315,13 @@
         </is>
       </c>
     </row>
-    <row r="58" ht="310" customHeight="1">
+    <row r="58" ht="340" customHeight="1">
       <c r="A58" s="11" t="inlineStr">
         <is>
           <t>HYPOTHESIS. HealthGuard's Rural FNR disparity is not a 'Rural' effect. It runs through insurance_type and region acting as proxies for historical under-diagnosis. In the training labels, poorer rural patients (Medicaid / Uninsured) were diagnosed at about half the true rate. The model learned that being 'Rural + Medicaid/Uninsured' means low risk, and now repeats the access gap at the point of care.
 EVIDENCE (test n=3,000, threshold 0.26):
 1) Disparity is concentrated in one cell. Rural FNR is 37.8% vs 22.7% for Urban (+15.2 pp region gap). Within Rural, Medicaid FNR is 60.6% (n_pos=33, Wilson 95% CI about 44-75%) vs 23.1% for Rural × Private (n_pos=52, CI about 14-36%), a +37.5 pp gap. In the Urban reference the same comparison is -5.2 pp (Medicaid 19.2% vs Private 24.5%). Insurance matters only inside Rural, and Rural × Private performs like Urban. Verdict from assess_proxy_pathway: proxy_supported (+42.8 pp excess over the reference, margin 5 pp). This is the most-harmed cell at n_pos &gt;= 20. KRI-1 = Red (43.4 pp gap, Rural × Medicaid vs Urban × Medicare).
-2) The training labels carry the bias. Recorded diabetes prevalence in train is 13.5% for Rural × Medicaid and 12.7% for Rural × Uninsured, against 26-29% in every other cell, including Urban × Medicaid at 26.1%. In train, Rural is 45% Medicaid. This matches brief §8: under-served patients get fewer encounters, so fewer diagnoses, and the Source 2 synthetic generator copied the pattern.
+2) The training labels carry the bias. Recorded diabetes prevalence in train is 13.5% for Rural × Medicaid and 12.7% for Rural × Uninsured, against 25-29% in every Urban cell and every Medicare or Private cell (Urban × Medicaid is 26.1%). Suburban × Medicaid / Uninsured sit in between (19.8% / 21.5%). The deficit follows care access: deepest for rural Medicaid/uninsured patients, partial for suburban ones, absent for urban ones. In train, Rural is 45% Medicaid. This matches brief §8: under-served patients get fewer encounters, so fewer diagnoses, and the Source 2 synthetic generator copied the pattern.
 3) The missed patients are clinically comparable. True positives in Rural × Medicaid have mean glucose 129, BMI 31.2 and age 54, compared with 133 / 30.2 / 54 for Rural × Private, and a higher family-history rate (0.39 vs 0.29). Milder disease does not explain the misses.
 4) SHAP shows the mechanism locally. On false negatives in Rural × (Medicaid|Uninsured), region + insurance_type contribute -0.63 log-odds on average, against +0.07 on FNs in all other cells. Across all patients the same features give -0.59 to Rural × Medicaid/Uninsured and +0.15 to Urban × Private, a 0.74 log-odds swing from non-clinical features alone. The notebook's local examples show cat__region_Rural (about -0.27) and cat__insurance_type_Medicaid/Uninsured (-0.23 / -0.34) among the top-3 negative drivers. Removing only the region + insurance attributions would lift 8 of 25 (32%) of these FNs above the threshold, against 3 of 167 (2%) elsewhere.</t>
         </is>
@@ -3330,7 +3337,7 @@
         <is>
           <t>WHY THE GLOBAL SHAP TABLE SAYS 'no'. detect_proxy_features ranks insurance_type_Medicaid 8th (mean |SHAP| 0.076) but finds signed_strength of only about 0.03. So the notebook's is_likely_proxy rule (mean_shap &lt; -0.01 AND strength &gt;= 0.5) flags nothing. The proxy effect points in opposite directions in different cells (negative for Rural/Medicaid, positive for Urban/Private) and lands on about 12% of patients, so it averages out in a population-level summary. Lesson for D6/D8: a global-SHAP proxy screen is necessary but NOT sufficient. Proxy detection must be subgroup-conditional, meaning SHAP averaged within each intersectional cell.
 VERDICT: proxy-bias pathway SUPPORTED. insurance_type (with region) acts as a proxy for under-diagnosis in the labels, not for diabetes risk. The harm is about 2.6x the missed-diagnosis rate (60.6% vs 23.1%) for an identifiable, disadvantaged group. That breaches the Board's low patient-safety appetite (D1 gap #1; D5 Fairness risk; D7 KRI-1 Red).
-LIMITATIONS. (a) The test labels carry the same under-diagnosis: Rural × Medicaid prevalence is 11.6% vs about 26% elsewhere. Undiagnosed diabetics in this cell are labelled 0 and cannot count as misses, so the measured 60.6% FNR is probably an UNDER-estimate. (b) Rural × Uninsured (FNR 50%, n_pos=10) and Rural × Medicare (n_pos=16) fall below the n_pos &gt;= 20 power filter and cannot be quantified (residual risk for D5). (c) SHAP attributions are not counterfactuals. The 32% 'would-flip' figure is an attribution heuristic, not a causal estimate. (d) Synthetic, single-split data from IE/DE only. Not validated for the US population.
+LIMITATIONS. (a) The test labels carry the same under-diagnosis: Rural × Medicaid prevalence is 11.6% (Rural × Uninsured 11.1%) vs 25-28% in every other test cell. Undiagnosed diabetics in this cell are labelled 0 and cannot count as misses, so the measured 60.6% FNR is probably an UNDER-estimate. (b) Rural × Uninsured (FNR 50%, n_pos=10) and Rural × Medicare (n_pos=16) fall below the n_pos &gt;= 20 power filter and cannot be quantified (residual risk for D5). (c) SHAP attributions are not counterfactuals. The 32% 'would-flip' figure is an attribution heuristic, not a causal estimate. (d) Synthetic, single-split data from IE/DE only. Not validated for the US population.
 WHAT WOULD CONFIRM OR REFUTE IT (pre-launch actions): (1) Ablation: retrain without region and insurance_type, then re-run this audit. Expect the Rural × Medicaid FNR gap to shrink but not close, because the label bias remains. (2) Label audit: re-adjudicate a sample of Rural × Medicaid negatives against HbA1c/fasting-glucose criteria to estimate the hidden positives. (3) Mitigate through relabelling / reweighting plus group-aware threshold review, then re-test against KRI-1 (Green &lt;= 8 pp). (4) Add subgroup-conditional SHAP to the CI release gate.</t>
         </is>
       </c>
@@ -3562,9 +3569,8 @@
       <c r="G7" s="47" t="n">
         <v>5</v>
       </c>
-      <c r="H7" s="48">
-        <f>IFERROR(F7*G7,"")</f>
-        <v/>
+      <c r="H7" s="48" t="n">
+        <v>25</v>
       </c>
       <c r="I7" s="26" t="inlineStr">
         <is>
@@ -3617,9 +3623,8 @@
       <c r="G8" s="47" t="n">
         <v>4</v>
       </c>
-      <c r="H8" s="48">
-        <f>IFERROR(F8*G8,"")</f>
-        <v/>
+      <c r="H8" s="48" t="n">
+        <v>20</v>
       </c>
       <c r="I8" s="26" t="inlineStr">
         <is>
@@ -3672,9 +3677,8 @@
       <c r="G9" s="47" t="n">
         <v>4</v>
       </c>
-      <c r="H9" s="48">
-        <f>IFERROR(F9*G9,"")</f>
-        <v/>
+      <c r="H9" s="48" t="n">
+        <v>16</v>
       </c>
       <c r="I9" s="26" t="inlineStr">
         <is>
@@ -3727,9 +3731,8 @@
       <c r="G10" s="47" t="n">
         <v>4</v>
       </c>
-      <c r="H10" s="48">
-        <f>IFERROR(F10*G10,"")</f>
-        <v/>
+      <c r="H10" s="48" t="n">
+        <v>16</v>
       </c>
       <c r="I10" s="26" t="inlineStr">
         <is>
@@ -3782,9 +3785,8 @@
       <c r="G11" s="47" t="n">
         <v>4</v>
       </c>
-      <c r="H11" s="48">
-        <f>IFERROR(F11*G11,"")</f>
-        <v/>
+      <c r="H11" s="48" t="n">
+        <v>16</v>
       </c>
       <c r="I11" s="26" t="inlineStr">
         <is>
@@ -3837,9 +3839,8 @@
       <c r="G12" s="47" t="n">
         <v>5</v>
       </c>
-      <c r="H12" s="48">
-        <f>IFERROR(F12*G12,"")</f>
-        <v/>
+      <c r="H12" s="48" t="n">
+        <v>15</v>
       </c>
       <c r="I12" s="26" t="inlineStr">
         <is>
@@ -3892,9 +3893,8 @@
       <c r="G13" s="47" t="n">
         <v>3</v>
       </c>
-      <c r="H13" s="48">
-        <f>IFERROR(F13*G13,"")</f>
-        <v/>
+      <c r="H13" s="48" t="n">
+        <v>6</v>
       </c>
       <c r="I13" s="26" t="inlineStr">
         <is>
@@ -3947,9 +3947,8 @@
       <c r="G14" s="47" t="n">
         <v>4</v>
       </c>
-      <c r="H14" s="48">
-        <f>IFERROR(F14*G14,"")</f>
-        <v/>
+      <c r="H14" s="48" t="n">
+        <v>16</v>
       </c>
       <c r="I14" s="26" t="inlineStr">
         <is>
@@ -4002,9 +4001,8 @@
       <c r="G15" s="47" t="n">
         <v>3</v>
       </c>
-      <c r="H15" s="48">
-        <f>IFERROR(F15*G15,"")</f>
-        <v/>
+      <c r="H15" s="48" t="n">
+        <v>15</v>
       </c>
       <c r="I15" s="26" t="inlineStr">
         <is>
@@ -4057,9 +4055,8 @@
       <c r="G16" s="47" t="n">
         <v>4</v>
       </c>
-      <c r="H16" s="48">
-        <f>IFERROR(F16*G16,"")</f>
-        <v/>
+      <c r="H16" s="48" t="n">
+        <v>12</v>
       </c>
       <c r="I16" s="26" t="inlineStr">
         <is>
@@ -4112,9 +4109,8 @@
       <c r="G17" s="47" t="n">
         <v>3</v>
       </c>
-      <c r="H17" s="48">
-        <f>IFERROR(F17*G17,"")</f>
-        <v/>
+      <c r="H17" s="48" t="n">
+        <v>12</v>
       </c>
       <c r="I17" s="26" t="inlineStr">
         <is>
@@ -4143,7 +4139,7 @@
       </c>
       <c r="B18" s="26" t="inlineStr">
         <is>
-          <t>SUBGROUP HARM WE CANNOT FULLY MEASURE. Rural × Uninsured (FNR 50%, n_pos=10) and Rural × Medicare (n_pos=16) are below the n_pos &gt;= 20 power filter. Test labels carry the same under-diagnosis (Rural × Medicaid prevalence 11.6% vs about 26%), so the measured FNR is probably an under-estimate. The global SHAP proxy screen flagged nothing (is_likely_proxy = 'no' for every feature). There is no standard-of-care baseline.</t>
+          <t>SUBGROUP HARM WE CANNOT FULLY MEASURE. Rural × Uninsured (FNR 50%, n_pos=10) and Rural × Medicare (n_pos=16) are below the n_pos &gt;= 20 power filter. Test labels carry the same under-diagnosis (Rural × Medicaid prevalence 11.6% vs 25-28% in every other test cell), so the measured FNR is probably an under-estimate. The global SHAP proxy screen flagged nothing (is_likely_proxy = 'no' for every feature). There is no standard-of-care baseline.</t>
         </is>
       </c>
       <c r="C18" s="26" t="inlineStr">
@@ -4167,9 +4163,8 @@
       <c r="G18" s="47" t="n">
         <v>4</v>
       </c>
-      <c r="H18" s="48">
-        <f>IFERROR(F18*G18,"")</f>
-        <v/>
+      <c r="H18" s="48" t="n">
+        <v>16</v>
       </c>
       <c r="I18" s="26" t="inlineStr">
         <is>
@@ -4425,7 +4420,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="310" customHeight="1">
+    <row r="14" ht="325" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
         <is>
           <t>SOURCES:
@@ -4435,7 +4430,7 @@
 SIZE: train.csv has 12,000 records (Urban 5,423 / Suburban 4,089 / Rural 2,488; F 6,613 / M 5,387; Private 6,316 / Medicaid 2,724 / Medicare 2,047 / Uninsured 913; prevalence 25%). Held-out test set: 3,000 records. The brief states '~8,000 records', so the manifest hash and dataset need reconciling before Annex IV sign-off.
 LABEL: diabetes_outcome is a RECORDED T2D diagnosis from the EHR, not confirmed disease status. It therefore inherits care-access bias.
 KNOWN LIMITATIONS (from D1/D4 analysis):
-(1) LABEL BIAS. Recorded prevalence is 13.5% for Rural × Medicaid and 12.7% for Rural × Uninsured, against 26-29% in every other cell. Under-served patients were diagnosed less often, and the Source 2 generator copied this pattern rather than correcting it.
+(1) LABEL BIAS. Recorded prevalence is 13.5% for Rural × Medicaid and 12.7% for Rural × Uninsured, against 25-29% in every Urban cell and every Medicare or Private cell. Suburban × Medicaid / Uninsured are intermediate (19.8% / 21.5%). Under-served patients were diagnosed less often, and the Source 2 generator copied this pattern rather than correcting it.
 (2) PROXY STRUCTURE. Rural patients are 45% Medicaid in training (vs 15% for Urban), so region and insurance_type together encode socio-economic access.
 (3) DATA QUALITY. insurance_type comes from hospital billing and can be stale. 222 records (1.9%) have insulin = 0, which is physiologically implausible and probably missing data coded as zero. 87 patients aged 18-20 are binned into age_group '21-35'.
 (4) PROVENANCE ANOMALY. The insurance categories (Medicaid / Medicare / Uninsured) are US payer types, yet Source 1 is IE/DE data. The mapping or generation step must be documented.
@@ -5171,7 +5166,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="280" customHeight="1">
+    <row r="13" ht="295" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
         <is>
           <t>B.1 EVIDENCE SUMMARY
@@ -5180,7 +5175,7 @@
 • D3 MITRE ATLAS Threat Model: three credible attack paths with no AI-specific mitigation in place: AML.T0020 poisoning through the override loop (M-H/H), AML.T0010.003 unsigned joblib pickle artifact (M/H), AML.T0024 API extraction and membership inference (L-M/M).
 • D4 Technical Audit (test n=3,000, threshold 0.26): ROC AUC 0.812, recall 0.744 (FNR 25.6%).
   - FNR is 37.8% for Rural vs 22.7% for Urban. Rural × Medicaid is 60.6% (n_pos=33; 95% CI about 44-75%) vs 23.1% for Rural × Private. Proxy pathway SUPPORTED: +37.5 pp gap within Rural vs -5.2 pp in Urban.
-  - Root cause is label bias: training prevalence is 13.5% for Rural × Medicaid vs 26-29% elsewhere, and the missed patients are clinically comparable (glucose 129 vs 133, BMI 31.2 vs 30.2).
+  - Root cause is label bias: training prevalence is 13.5% for Rural × Medicaid vs 25-29% in Urban and Medicare/Private cells (Suburban Medicaid/Uninsured intermediate at 19.8% / 21.5%), and the missed patients are clinically comparable (glucose 129 vs 133, BMI 31.2 vs 30.2).
   - region + insurance_type contribute -0.59 log-odds in the harmed cells vs +0.15 for Urban × Private. The global SHAP proxy screen flagged nothing.
 • D5 NIST AI RMF Risk Register: 12 risks drawn from D1-D4. Top-N: RR-01 subgroup under-detection (25), RR-02 no lawful EU route (20), RR-04 oversight (16), RR-05 poisoning (16), RR-08 unlawful secondary use (16).
 • D6 Model Card: provenance gaps. The data has 12,000 training rows vs '~8,000' in the brief; US payer categories appear in IE/DE data; 222 records have insulin = 0; the label is a recorded diagnosis, not confirmed disease; there has been no external validation.

</xml_diff>